<commit_message>
daily auto-refresh 2026-08-17 15:40
</commit_message>
<xml_diff>
--- a/daily_slab_mix.xlsx
+++ b/daily_slab_mix.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M311"/>
+  <dimension ref="A1:O314"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,6 +482,16 @@
           <t>Total creators</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Sample orders</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Sample units</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -525,6 +535,12 @@
       <c r="M2" t="n">
         <v>4</v>
       </c>
+      <c r="N2" t="n">
+        <v>4</v>
+      </c>
+      <c r="O2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -568,6 +584,12 @@
       <c r="M3" t="n">
         <v>3</v>
       </c>
+      <c r="N3" t="n">
+        <v>3</v>
+      </c>
+      <c r="O3" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -611,6 +633,12 @@
       <c r="M4" t="n">
         <v>1</v>
       </c>
+      <c r="N4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -654,6 +682,12 @@
       <c r="M5" t="n">
         <v>2</v>
       </c>
+      <c r="N5" t="n">
+        <v>2</v>
+      </c>
+      <c r="O5" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -697,6 +731,12 @@
       <c r="M6" t="n">
         <v>16</v>
       </c>
+      <c r="N6" t="n">
+        <v>17</v>
+      </c>
+      <c r="O6" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -740,6 +780,12 @@
       <c r="M7" t="n">
         <v>3</v>
       </c>
+      <c r="N7" t="n">
+        <v>3</v>
+      </c>
+      <c r="O7" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -783,6 +829,12 @@
       <c r="M8" t="n">
         <v>1</v>
       </c>
+      <c r="N8" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -826,6 +878,12 @@
       <c r="M9" t="n">
         <v>6</v>
       </c>
+      <c r="N9" t="n">
+        <v>6</v>
+      </c>
+      <c r="O9" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -869,6 +927,12 @@
       <c r="M10" t="n">
         <v>4</v>
       </c>
+      <c r="N10" t="n">
+        <v>4</v>
+      </c>
+      <c r="O10" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -912,6 +976,12 @@
       <c r="M11" t="n">
         <v>1</v>
       </c>
+      <c r="N11" t="n">
+        <v>1</v>
+      </c>
+      <c r="O11" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -955,6 +1025,12 @@
       <c r="M12" t="n">
         <v>5</v>
       </c>
+      <c r="N12" t="n">
+        <v>5</v>
+      </c>
+      <c r="O12" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -998,6 +1074,12 @@
       <c r="M13" t="n">
         <v>6</v>
       </c>
+      <c r="N13" t="n">
+        <v>6</v>
+      </c>
+      <c r="O13" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1041,6 +1123,12 @@
       <c r="M14" t="n">
         <v>9</v>
       </c>
+      <c r="N14" t="n">
+        <v>9</v>
+      </c>
+      <c r="O14" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1084,6 +1172,12 @@
       <c r="M15" t="n">
         <v>7</v>
       </c>
+      <c r="N15" t="n">
+        <v>7</v>
+      </c>
+      <c r="O15" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1127,6 +1221,12 @@
       <c r="M16" t="n">
         <v>20</v>
       </c>
+      <c r="N16" t="n">
+        <v>21</v>
+      </c>
+      <c r="O16" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1170,6 +1270,12 @@
       <c r="M17" t="n">
         <v>15</v>
       </c>
+      <c r="N17" t="n">
+        <v>15</v>
+      </c>
+      <c r="O17" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1213,6 +1319,12 @@
       <c r="M18" t="n">
         <v>32</v>
       </c>
+      <c r="N18" t="n">
+        <v>34</v>
+      </c>
+      <c r="O18" t="n">
+        <v>34</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1256,6 +1368,12 @@
       <c r="M19" t="n">
         <v>28</v>
       </c>
+      <c r="N19" t="n">
+        <v>28</v>
+      </c>
+      <c r="O19" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1299,6 +1417,12 @@
       <c r="M20" t="n">
         <v>26</v>
       </c>
+      <c r="N20" t="n">
+        <v>26</v>
+      </c>
+      <c r="O20" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1342,6 +1466,12 @@
       <c r="M21" t="n">
         <v>1</v>
       </c>
+      <c r="N21" t="n">
+        <v>1</v>
+      </c>
+      <c r="O21" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1385,6 +1515,12 @@
       <c r="M22" t="n">
         <v>29</v>
       </c>
+      <c r="N22" t="n">
+        <v>29</v>
+      </c>
+      <c r="O22" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1428,6 +1564,12 @@
       <c r="M23" t="n">
         <v>29</v>
       </c>
+      <c r="N23" t="n">
+        <v>29</v>
+      </c>
+      <c r="O23" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1471,6 +1613,12 @@
       <c r="M24" t="n">
         <v>20</v>
       </c>
+      <c r="N24" t="n">
+        <v>21</v>
+      </c>
+      <c r="O24" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1514,6 +1662,12 @@
       <c r="M25" t="n">
         <v>21</v>
       </c>
+      <c r="N25" t="n">
+        <v>21</v>
+      </c>
+      <c r="O25" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1557,6 +1711,12 @@
       <c r="M26" t="n">
         <v>14</v>
       </c>
+      <c r="N26" t="n">
+        <v>14</v>
+      </c>
+      <c r="O26" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1600,6 +1760,12 @@
       <c r="M27" t="n">
         <v>17</v>
       </c>
+      <c r="N27" t="n">
+        <v>18</v>
+      </c>
+      <c r="O27" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1643,6 +1809,12 @@
       <c r="M28" t="n">
         <v>10</v>
       </c>
+      <c r="N28" t="n">
+        <v>10</v>
+      </c>
+      <c r="O28" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1686,6 +1858,12 @@
       <c r="M29" t="n">
         <v>14</v>
       </c>
+      <c r="N29" t="n">
+        <v>14</v>
+      </c>
+      <c r="O29" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1729,6 +1907,12 @@
       <c r="M30" t="n">
         <v>26</v>
       </c>
+      <c r="N30" t="n">
+        <v>27</v>
+      </c>
+      <c r="O30" t="n">
+        <v>27</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1772,6 +1956,12 @@
       <c r="M31" t="n">
         <v>22</v>
       </c>
+      <c r="N31" t="n">
+        <v>22</v>
+      </c>
+      <c r="O31" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1815,6 +2005,12 @@
       <c r="M32" t="n">
         <v>15</v>
       </c>
+      <c r="N32" t="n">
+        <v>15</v>
+      </c>
+      <c r="O32" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1858,6 +2054,12 @@
       <c r="M33" t="n">
         <v>34</v>
       </c>
+      <c r="N33" t="n">
+        <v>34</v>
+      </c>
+      <c r="O33" t="n">
+        <v>34</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1901,6 +2103,12 @@
       <c r="M34" t="n">
         <v>9</v>
       </c>
+      <c r="N34" t="n">
+        <v>9</v>
+      </c>
+      <c r="O34" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1944,6 +2152,12 @@
       <c r="M35" t="n">
         <v>4</v>
       </c>
+      <c r="N35" t="n">
+        <v>4</v>
+      </c>
+      <c r="O35" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1987,6 +2201,12 @@
       <c r="M36" t="n">
         <v>23</v>
       </c>
+      <c r="N36" t="n">
+        <v>23</v>
+      </c>
+      <c r="O36" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2030,6 +2250,12 @@
       <c r="M37" t="n">
         <v>4</v>
       </c>
+      <c r="N37" t="n">
+        <v>4</v>
+      </c>
+      <c r="O37" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2073,6 +2299,12 @@
       <c r="M38" t="n">
         <v>1</v>
       </c>
+      <c r="N38" t="n">
+        <v>1</v>
+      </c>
+      <c r="O38" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2116,6 +2348,12 @@
       <c r="M39" t="n">
         <v>11</v>
       </c>
+      <c r="N39" t="n">
+        <v>11</v>
+      </c>
+      <c r="O39" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2159,6 +2397,12 @@
       <c r="M40" t="n">
         <v>1</v>
       </c>
+      <c r="N40" t="n">
+        <v>1</v>
+      </c>
+      <c r="O40" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2202,6 +2446,12 @@
       <c r="M41" t="n">
         <v>16</v>
       </c>
+      <c r="N41" t="n">
+        <v>16</v>
+      </c>
+      <c r="O41" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2245,6 +2495,12 @@
       <c r="M42" t="n">
         <v>20</v>
       </c>
+      <c r="N42" t="n">
+        <v>20</v>
+      </c>
+      <c r="O42" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2288,6 +2544,12 @@
       <c r="M43" t="n">
         <v>24</v>
       </c>
+      <c r="N43" t="n">
+        <v>24</v>
+      </c>
+      <c r="O43" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2331,6 +2593,12 @@
       <c r="M44" t="n">
         <v>24</v>
       </c>
+      <c r="N44" t="n">
+        <v>24</v>
+      </c>
+      <c r="O44" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2374,6 +2642,12 @@
       <c r="M45" t="n">
         <v>20</v>
       </c>
+      <c r="N45" t="n">
+        <v>22</v>
+      </c>
+      <c r="O45" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2417,6 +2691,12 @@
       <c r="M46" t="n">
         <v>2</v>
       </c>
+      <c r="N46" t="n">
+        <v>2</v>
+      </c>
+      <c r="O46" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2460,6 +2740,12 @@
       <c r="M47" t="n">
         <v>13</v>
       </c>
+      <c r="N47" t="n">
+        <v>16</v>
+      </c>
+      <c r="O47" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2503,6 +2789,12 @@
       <c r="M48" t="n">
         <v>41</v>
       </c>
+      <c r="N48" t="n">
+        <v>52</v>
+      </c>
+      <c r="O48" t="n">
+        <v>52</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2546,6 +2838,12 @@
       <c r="M49" t="n">
         <v>40</v>
       </c>
+      <c r="N49" t="n">
+        <v>44</v>
+      </c>
+      <c r="O49" t="n">
+        <v>44</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2589,6 +2887,12 @@
       <c r="M50" t="n">
         <v>52</v>
       </c>
+      <c r="N50" t="n">
+        <v>58</v>
+      </c>
+      <c r="O50" t="n">
+        <v>58</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2632,6 +2936,12 @@
       <c r="M51" t="n">
         <v>25</v>
       </c>
+      <c r="N51" t="n">
+        <v>26</v>
+      </c>
+      <c r="O51" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2675,6 +2985,12 @@
       <c r="M52" t="n">
         <v>38</v>
       </c>
+      <c r="N52" t="n">
+        <v>40</v>
+      </c>
+      <c r="O52" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2718,6 +3034,12 @@
       <c r="M53" t="n">
         <v>2</v>
       </c>
+      <c r="N53" t="n">
+        <v>3</v>
+      </c>
+      <c r="O53" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2761,6 +3083,12 @@
       <c r="M54" t="n">
         <v>3</v>
       </c>
+      <c r="N54" t="n">
+        <v>3</v>
+      </c>
+      <c r="O54" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2804,6 +3132,12 @@
       <c r="M55" t="n">
         <v>31</v>
       </c>
+      <c r="N55" t="n">
+        <v>32</v>
+      </c>
+      <c r="O55" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2847,6 +3181,12 @@
       <c r="M56" t="n">
         <v>1</v>
       </c>
+      <c r="N56" t="n">
+        <v>1</v>
+      </c>
+      <c r="O56" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2890,6 +3230,12 @@
       <c r="M57" t="n">
         <v>3</v>
       </c>
+      <c r="N57" t="n">
+        <v>3</v>
+      </c>
+      <c r="O57" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2933,6 +3279,12 @@
       <c r="M58" t="n">
         <v>70</v>
       </c>
+      <c r="N58" t="n">
+        <v>72</v>
+      </c>
+      <c r="O58" t="n">
+        <v>72</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2976,6 +3328,12 @@
       <c r="M59" t="n">
         <v>26</v>
       </c>
+      <c r="N59" t="n">
+        <v>26</v>
+      </c>
+      <c r="O59" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3019,6 +3377,12 @@
       <c r="M60" t="n">
         <v>45</v>
       </c>
+      <c r="N60" t="n">
+        <v>47</v>
+      </c>
+      <c r="O60" t="n">
+        <v>47</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3062,6 +3426,12 @@
       <c r="M61" t="n">
         <v>28</v>
       </c>
+      <c r="N61" t="n">
+        <v>29</v>
+      </c>
+      <c r="O61" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3105,6 +3475,12 @@
       <c r="M62" t="n">
         <v>37</v>
       </c>
+      <c r="N62" t="n">
+        <v>40</v>
+      </c>
+      <c r="O62" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3148,6 +3524,12 @@
       <c r="M63" t="n">
         <v>27</v>
       </c>
+      <c r="N63" t="n">
+        <v>27</v>
+      </c>
+      <c r="O63" t="n">
+        <v>27</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3191,6 +3573,12 @@
       <c r="M64" t="n">
         <v>17</v>
       </c>
+      <c r="N64" t="n">
+        <v>18</v>
+      </c>
+      <c r="O64" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3234,6 +3622,12 @@
       <c r="M65" t="n">
         <v>1</v>
       </c>
+      <c r="N65" t="n">
+        <v>1</v>
+      </c>
+      <c r="O65" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3277,6 +3671,12 @@
       <c r="M66" t="n">
         <v>32</v>
       </c>
+      <c r="N66" t="n">
+        <v>32</v>
+      </c>
+      <c r="O66" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3320,6 +3720,12 @@
       <c r="M67" t="n">
         <v>39</v>
       </c>
+      <c r="N67" t="n">
+        <v>41</v>
+      </c>
+      <c r="O67" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3363,6 +3769,12 @@
       <c r="M68" t="n">
         <v>4</v>
       </c>
+      <c r="N68" t="n">
+        <v>4</v>
+      </c>
+      <c r="O68" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3406,6 +3818,12 @@
       <c r="M69" t="n">
         <v>38</v>
       </c>
+      <c r="N69" t="n">
+        <v>39</v>
+      </c>
+      <c r="O69" t="n">
+        <v>39</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3449,6 +3867,12 @@
       <c r="M70" t="n">
         <v>29</v>
       </c>
+      <c r="N70" t="n">
+        <v>29</v>
+      </c>
+      <c r="O70" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3492,6 +3916,12 @@
       <c r="M71" t="n">
         <v>4</v>
       </c>
+      <c r="N71" t="n">
+        <v>4</v>
+      </c>
+      <c r="O71" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3535,6 +3965,12 @@
       <c r="M72" t="n">
         <v>29</v>
       </c>
+      <c r="N72" t="n">
+        <v>29</v>
+      </c>
+      <c r="O72" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3578,6 +4014,12 @@
       <c r="M73" t="n">
         <v>34</v>
       </c>
+      <c r="N73" t="n">
+        <v>35</v>
+      </c>
+      <c r="O73" t="n">
+        <v>35</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3621,6 +4063,12 @@
       <c r="M74" t="n">
         <v>35</v>
       </c>
+      <c r="N74" t="n">
+        <v>35</v>
+      </c>
+      <c r="O74" t="n">
+        <v>35</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3664,6 +4112,12 @@
       <c r="M75" t="n">
         <v>12</v>
       </c>
+      <c r="N75" t="n">
+        <v>13</v>
+      </c>
+      <c r="O75" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3707,6 +4161,12 @@
       <c r="M76" t="n">
         <v>45</v>
       </c>
+      <c r="N76" t="n">
+        <v>46</v>
+      </c>
+      <c r="O76" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3750,6 +4210,12 @@
       <c r="M77" t="n">
         <v>26</v>
       </c>
+      <c r="N77" t="n">
+        <v>26</v>
+      </c>
+      <c r="O77" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3793,6 +4259,12 @@
       <c r="M78" t="n">
         <v>2</v>
       </c>
+      <c r="N78" t="n">
+        <v>3</v>
+      </c>
+      <c r="O78" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3836,6 +4308,12 @@
       <c r="M79" t="n">
         <v>10</v>
       </c>
+      <c r="N79" t="n">
+        <v>11</v>
+      </c>
+      <c r="O79" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3879,6 +4357,12 @@
       <c r="M80" t="n">
         <v>62</v>
       </c>
+      <c r="N80" t="n">
+        <v>63</v>
+      </c>
+      <c r="O80" t="n">
+        <v>63</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3922,6 +4406,12 @@
       <c r="M81" t="n">
         <v>43</v>
       </c>
+      <c r="N81" t="n">
+        <v>44</v>
+      </c>
+      <c r="O81" t="n">
+        <v>44</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3965,6 +4455,12 @@
       <c r="M82" t="n">
         <v>31</v>
       </c>
+      <c r="N82" t="n">
+        <v>32</v>
+      </c>
+      <c r="O82" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4008,6 +4504,12 @@
       <c r="M83" t="n">
         <v>20</v>
       </c>
+      <c r="N83" t="n">
+        <v>20</v>
+      </c>
+      <c r="O83" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4051,6 +4553,12 @@
       <c r="M84" t="n">
         <v>36</v>
       </c>
+      <c r="N84" t="n">
+        <v>39</v>
+      </c>
+      <c r="O84" t="n">
+        <v>39</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4094,6 +4602,12 @@
       <c r="M85" t="n">
         <v>1</v>
       </c>
+      <c r="N85" t="n">
+        <v>1</v>
+      </c>
+      <c r="O85" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4137,6 +4651,12 @@
       <c r="M86" t="n">
         <v>21</v>
       </c>
+      <c r="N86" t="n">
+        <v>21</v>
+      </c>
+      <c r="O86" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4180,6 +4700,12 @@
       <c r="M87" t="n">
         <v>34</v>
       </c>
+      <c r="N87" t="n">
+        <v>35</v>
+      </c>
+      <c r="O87" t="n">
+        <v>35</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4223,6 +4749,12 @@
       <c r="M88" t="n">
         <v>50</v>
       </c>
+      <c r="N88" t="n">
+        <v>51</v>
+      </c>
+      <c r="O88" t="n">
+        <v>51</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4266,6 +4798,12 @@
       <c r="M89" t="n">
         <v>34</v>
       </c>
+      <c r="N89" t="n">
+        <v>36</v>
+      </c>
+      <c r="O89" t="n">
+        <v>36</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4309,6 +4847,12 @@
       <c r="M90" t="n">
         <v>35</v>
       </c>
+      <c r="N90" t="n">
+        <v>38</v>
+      </c>
+      <c r="O90" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4352,6 +4896,12 @@
       <c r="M91" t="n">
         <v>19</v>
       </c>
+      <c r="N91" t="n">
+        <v>20</v>
+      </c>
+      <c r="O91" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4395,6 +4945,12 @@
       <c r="M92" t="n">
         <v>16</v>
       </c>
+      <c r="N92" t="n">
+        <v>17</v>
+      </c>
+      <c r="O92" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4438,6 +4994,12 @@
       <c r="M93" t="n">
         <v>39</v>
       </c>
+      <c r="N93" t="n">
+        <v>39</v>
+      </c>
+      <c r="O93" t="n">
+        <v>39</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -4481,6 +5043,12 @@
       <c r="M94" t="n">
         <v>27</v>
       </c>
+      <c r="N94" t="n">
+        <v>28</v>
+      </c>
+      <c r="O94" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -4524,6 +5092,12 @@
       <c r="M95" t="n">
         <v>21</v>
       </c>
+      <c r="N95" t="n">
+        <v>21</v>
+      </c>
+      <c r="O95" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4567,6 +5141,12 @@
       <c r="M96" t="n">
         <v>56</v>
       </c>
+      <c r="N96" t="n">
+        <v>61</v>
+      </c>
+      <c r="O96" t="n">
+        <v>61</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -4610,6 +5190,12 @@
       <c r="M97" t="n">
         <v>23</v>
       </c>
+      <c r="N97" t="n">
+        <v>24</v>
+      </c>
+      <c r="O97" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -4653,6 +5239,12 @@
       <c r="M98" t="n">
         <v>8</v>
       </c>
+      <c r="N98" t="n">
+        <v>8</v>
+      </c>
+      <c r="O98" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -4696,6 +5288,12 @@
       <c r="M99" t="n">
         <v>2</v>
       </c>
+      <c r="N99" t="n">
+        <v>2</v>
+      </c>
+      <c r="O99" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -4739,6 +5337,12 @@
       <c r="M100" t="n">
         <v>26</v>
       </c>
+      <c r="N100" t="n">
+        <v>27</v>
+      </c>
+      <c r="O100" t="n">
+        <v>27</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -4782,6 +5386,12 @@
       <c r="M101" t="n">
         <v>23</v>
       </c>
+      <c r="N101" t="n">
+        <v>23</v>
+      </c>
+      <c r="O101" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -4825,6 +5435,12 @@
       <c r="M102" t="n">
         <v>2</v>
       </c>
+      <c r="N102" t="n">
+        <v>2</v>
+      </c>
+      <c r="O102" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -4868,6 +5484,12 @@
       <c r="M103" t="n">
         <v>49</v>
       </c>
+      <c r="N103" t="n">
+        <v>49</v>
+      </c>
+      <c r="O103" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -4911,6 +5533,12 @@
       <c r="M104" t="n">
         <v>36</v>
       </c>
+      <c r="N104" t="n">
+        <v>37</v>
+      </c>
+      <c r="O104" t="n">
+        <v>37</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -4954,6 +5582,12 @@
       <c r="M105" t="n">
         <v>6</v>
       </c>
+      <c r="N105" t="n">
+        <v>6</v>
+      </c>
+      <c r="O105" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -4997,6 +5631,12 @@
       <c r="M106" t="n">
         <v>60</v>
       </c>
+      <c r="N106" t="n">
+        <v>60</v>
+      </c>
+      <c r="O106" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -5040,6 +5680,12 @@
       <c r="M107" t="n">
         <v>32</v>
       </c>
+      <c r="N107" t="n">
+        <v>33</v>
+      </c>
+      <c r="O107" t="n">
+        <v>33</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -5083,6 +5729,12 @@
       <c r="M108" t="n">
         <v>26</v>
       </c>
+      <c r="N108" t="n">
+        <v>26</v>
+      </c>
+      <c r="O108" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -5126,6 +5778,12 @@
       <c r="M109" t="n">
         <v>11</v>
       </c>
+      <c r="N109" t="n">
+        <v>12</v>
+      </c>
+      <c r="O109" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -5169,6 +5827,12 @@
       <c r="M110" t="n">
         <v>2</v>
       </c>
+      <c r="N110" t="n">
+        <v>2</v>
+      </c>
+      <c r="O110" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -5212,6 +5876,12 @@
       <c r="M111" t="n">
         <v>14</v>
       </c>
+      <c r="N111" t="n">
+        <v>14</v>
+      </c>
+      <c r="O111" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -5255,6 +5925,12 @@
       <c r="M112" t="n">
         <v>1</v>
       </c>
+      <c r="N112" t="n">
+        <v>1</v>
+      </c>
+      <c r="O112" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -5298,6 +5974,12 @@
       <c r="M113" t="n">
         <v>38</v>
       </c>
+      <c r="N113" t="n">
+        <v>38</v>
+      </c>
+      <c r="O113" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -5341,6 +6023,12 @@
       <c r="M114" t="n">
         <v>21</v>
       </c>
+      <c r="N114" t="n">
+        <v>21</v>
+      </c>
+      <c r="O114" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -5384,6 +6072,12 @@
       <c r="M115" t="n">
         <v>32</v>
       </c>
+      <c r="N115" t="n">
+        <v>32</v>
+      </c>
+      <c r="O115" t="n">
+        <v>36</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -5427,6 +6121,12 @@
       <c r="M116" t="n">
         <v>2</v>
       </c>
+      <c r="N116" t="n">
+        <v>2</v>
+      </c>
+      <c r="O116" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -5470,6 +6170,12 @@
       <c r="M117" t="n">
         <v>55</v>
       </c>
+      <c r="N117" t="n">
+        <v>55</v>
+      </c>
+      <c r="O117" t="n">
+        <v>56</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -5513,6 +6219,12 @@
       <c r="M118" t="n">
         <v>52</v>
       </c>
+      <c r="N118" t="n">
+        <v>55</v>
+      </c>
+      <c r="O118" t="n">
+        <v>56</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -5556,6 +6268,12 @@
       <c r="M119" t="n">
         <v>34</v>
       </c>
+      <c r="N119" t="n">
+        <v>36</v>
+      </c>
+      <c r="O119" t="n">
+        <v>36</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -5599,6 +6317,12 @@
       <c r="M120" t="n">
         <v>29</v>
       </c>
+      <c r="N120" t="n">
+        <v>31</v>
+      </c>
+      <c r="O120" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -5642,6 +6366,12 @@
       <c r="M121" t="n">
         <v>36</v>
       </c>
+      <c r="N121" t="n">
+        <v>36</v>
+      </c>
+      <c r="O121" t="n">
+        <v>37</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -5685,6 +6415,12 @@
       <c r="M122" t="n">
         <v>122</v>
       </c>
+      <c r="N122" t="n">
+        <v>123</v>
+      </c>
+      <c r="O122" t="n">
+        <v>156</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -5728,6 +6464,12 @@
       <c r="M123" t="n">
         <v>29</v>
       </c>
+      <c r="N123" t="n">
+        <v>29</v>
+      </c>
+      <c r="O123" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -5771,6 +6513,12 @@
       <c r="M124" t="n">
         <v>30</v>
       </c>
+      <c r="N124" t="n">
+        <v>30</v>
+      </c>
+      <c r="O124" t="n">
+        <v>34</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -5814,6 +6562,12 @@
       <c r="M125" t="n">
         <v>30</v>
       </c>
+      <c r="N125" t="n">
+        <v>30</v>
+      </c>
+      <c r="O125" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -5857,6 +6611,12 @@
       <c r="M126" t="n">
         <v>9</v>
       </c>
+      <c r="N126" t="n">
+        <v>9</v>
+      </c>
+      <c r="O126" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -5900,6 +6660,12 @@
       <c r="M127" t="n">
         <v>101</v>
       </c>
+      <c r="N127" t="n">
+        <v>101</v>
+      </c>
+      <c r="O127" t="n">
+        <v>103</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -5943,6 +6709,12 @@
       <c r="M128" t="n">
         <v>12</v>
       </c>
+      <c r="N128" t="n">
+        <v>12</v>
+      </c>
+      <c r="O128" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -5986,6 +6758,12 @@
       <c r="M129" t="n">
         <v>33</v>
       </c>
+      <c r="N129" t="n">
+        <v>34</v>
+      </c>
+      <c r="O129" t="n">
+        <v>35</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -6029,6 +6807,12 @@
       <c r="M130" t="n">
         <v>26</v>
       </c>
+      <c r="N130" t="n">
+        <v>26</v>
+      </c>
+      <c r="O130" t="n">
+        <v>27</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -6072,6 +6856,12 @@
       <c r="M131" t="n">
         <v>28</v>
       </c>
+      <c r="N131" t="n">
+        <v>28</v>
+      </c>
+      <c r="O131" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -6115,6 +6905,12 @@
       <c r="M132" t="n">
         <v>36</v>
       </c>
+      <c r="N132" t="n">
+        <v>40</v>
+      </c>
+      <c r="O132" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -6158,6 +6954,12 @@
       <c r="M133" t="n">
         <v>5</v>
       </c>
+      <c r="N133" t="n">
+        <v>6</v>
+      </c>
+      <c r="O133" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -6201,6 +7003,12 @@
       <c r="M134" t="n">
         <v>3</v>
       </c>
+      <c r="N134" t="n">
+        <v>3</v>
+      </c>
+      <c r="O134" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -6244,6 +7052,12 @@
       <c r="M135" t="n">
         <v>94</v>
       </c>
+      <c r="N135" t="n">
+        <v>95</v>
+      </c>
+      <c r="O135" t="n">
+        <v>106</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -6287,6 +7101,12 @@
       <c r="M136" t="n">
         <v>32</v>
       </c>
+      <c r="N136" t="n">
+        <v>34</v>
+      </c>
+      <c r="O136" t="n">
+        <v>42</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -6330,6 +7150,12 @@
       <c r="M137" t="n">
         <v>37</v>
       </c>
+      <c r="N137" t="n">
+        <v>37</v>
+      </c>
+      <c r="O137" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -6373,6 +7199,12 @@
       <c r="M138" t="n">
         <v>58</v>
       </c>
+      <c r="N138" t="n">
+        <v>60</v>
+      </c>
+      <c r="O138" t="n">
+        <v>88</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -6416,6 +7248,12 @@
       <c r="M139" t="n">
         <v>35</v>
       </c>
+      <c r="N139" t="n">
+        <v>35</v>
+      </c>
+      <c r="O139" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -6459,6 +7297,12 @@
       <c r="M140" t="n">
         <v>2</v>
       </c>
+      <c r="N140" t="n">
+        <v>2</v>
+      </c>
+      <c r="O140" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -6502,6 +7346,12 @@
       <c r="M141" t="n">
         <v>39</v>
       </c>
+      <c r="N141" t="n">
+        <v>42</v>
+      </c>
+      <c r="O141" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -6545,6 +7395,12 @@
       <c r="M142" t="n">
         <v>55</v>
       </c>
+      <c r="N142" t="n">
+        <v>55</v>
+      </c>
+      <c r="O142" t="n">
+        <v>76</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -6588,6 +7444,12 @@
       <c r="M143" t="n">
         <v>56</v>
       </c>
+      <c r="N143" t="n">
+        <v>56</v>
+      </c>
+      <c r="O143" t="n">
+        <v>75</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -6631,6 +7493,12 @@
       <c r="M144" t="n">
         <v>49</v>
       </c>
+      <c r="N144" t="n">
+        <v>49</v>
+      </c>
+      <c r="O144" t="n">
+        <v>63</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -6674,6 +7542,12 @@
       <c r="M145" t="n">
         <v>36</v>
       </c>
+      <c r="N145" t="n">
+        <v>36</v>
+      </c>
+      <c r="O145" t="n">
+        <v>45</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -6717,6 +7591,12 @@
       <c r="M146" t="n">
         <v>50</v>
       </c>
+      <c r="N146" t="n">
+        <v>51</v>
+      </c>
+      <c r="O146" t="n">
+        <v>78</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -6760,6 +7640,12 @@
       <c r="M147" t="n">
         <v>44</v>
       </c>
+      <c r="N147" t="n">
+        <v>44</v>
+      </c>
+      <c r="O147" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -6803,6 +7689,12 @@
       <c r="M148" t="n">
         <v>76</v>
       </c>
+      <c r="N148" t="n">
+        <v>76</v>
+      </c>
+      <c r="O148" t="n">
+        <v>113</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -6846,6 +7738,12 @@
       <c r="M149" t="n">
         <v>33</v>
       </c>
+      <c r="N149" t="n">
+        <v>34</v>
+      </c>
+      <c r="O149" t="n">
+        <v>44</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -6889,6 +7787,12 @@
       <c r="M150" t="n">
         <v>91</v>
       </c>
+      <c r="N150" t="n">
+        <v>92</v>
+      </c>
+      <c r="O150" t="n">
+        <v>122</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -6932,6 +7836,12 @@
       <c r="M151" t="n">
         <v>1</v>
       </c>
+      <c r="N151" t="n">
+        <v>1</v>
+      </c>
+      <c r="O151" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -6975,6 +7885,12 @@
       <c r="M152" t="n">
         <v>46</v>
       </c>
+      <c r="N152" t="n">
+        <v>46</v>
+      </c>
+      <c r="O152" t="n">
+        <v>61</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -7018,6 +7934,12 @@
       <c r="M153" t="n">
         <v>43</v>
       </c>
+      <c r="N153" t="n">
+        <v>43</v>
+      </c>
+      <c r="O153" t="n">
+        <v>54</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -7061,6 +7983,12 @@
       <c r="M154" t="n">
         <v>33</v>
       </c>
+      <c r="N154" t="n">
+        <v>34</v>
+      </c>
+      <c r="O154" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -7104,6 +8032,12 @@
       <c r="M155" t="n">
         <v>45</v>
       </c>
+      <c r="N155" t="n">
+        <v>45</v>
+      </c>
+      <c r="O155" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -7147,6 +8081,12 @@
       <c r="M156" t="n">
         <v>108</v>
       </c>
+      <c r="N156" t="n">
+        <v>109</v>
+      </c>
+      <c r="O156" t="n">
+        <v>167</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -7190,6 +8130,12 @@
       <c r="M157" t="n">
         <v>41</v>
       </c>
+      <c r="N157" t="n">
+        <v>41</v>
+      </c>
+      <c r="O157" t="n">
+        <v>52</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -7233,6 +8179,12 @@
       <c r="M158" t="n">
         <v>44</v>
       </c>
+      <c r="N158" t="n">
+        <v>45</v>
+      </c>
+      <c r="O158" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -7276,6 +8228,12 @@
       <c r="M159" t="n">
         <v>56</v>
       </c>
+      <c r="N159" t="n">
+        <v>57</v>
+      </c>
+      <c r="O159" t="n">
+        <v>72</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -7319,6 +8277,12 @@
       <c r="M160" t="n">
         <v>39</v>
       </c>
+      <c r="N160" t="n">
+        <v>39</v>
+      </c>
+      <c r="O160" t="n">
+        <v>58</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -7362,6 +8326,12 @@
       <c r="M161" t="n">
         <v>40</v>
       </c>
+      <c r="N161" t="n">
+        <v>44</v>
+      </c>
+      <c r="O161" t="n">
+        <v>55</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -7405,6 +8375,12 @@
       <c r="M162" t="n">
         <v>36</v>
       </c>
+      <c r="N162" t="n">
+        <v>36</v>
+      </c>
+      <c r="O162" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -7448,6 +8424,12 @@
       <c r="M163" t="n">
         <v>36</v>
       </c>
+      <c r="N163" t="n">
+        <v>36</v>
+      </c>
+      <c r="O163" t="n">
+        <v>62</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -7491,6 +8473,12 @@
       <c r="M164" t="n">
         <v>37</v>
       </c>
+      <c r="N164" t="n">
+        <v>37</v>
+      </c>
+      <c r="O164" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -7534,6 +8522,12 @@
       <c r="M165" t="n">
         <v>31</v>
       </c>
+      <c r="N165" t="n">
+        <v>31</v>
+      </c>
+      <c r="O165" t="n">
+        <v>44</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -7577,6 +8571,12 @@
       <c r="M166" t="n">
         <v>121</v>
       </c>
+      <c r="N166" t="n">
+        <v>122</v>
+      </c>
+      <c r="O166" t="n">
+        <v>197</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -7620,6 +8620,12 @@
       <c r="M167" t="n">
         <v>48</v>
       </c>
+      <c r="N167" t="n">
+        <v>50</v>
+      </c>
+      <c r="O167" t="n">
+        <v>61</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -7663,6 +8669,12 @@
       <c r="M168" t="n">
         <v>122</v>
       </c>
+      <c r="N168" t="n">
+        <v>124</v>
+      </c>
+      <c r="O168" t="n">
+        <v>171</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -7706,6 +8718,12 @@
       <c r="M169" t="n">
         <v>40</v>
       </c>
+      <c r="N169" t="n">
+        <v>41</v>
+      </c>
+      <c r="O169" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -7749,6 +8767,12 @@
       <c r="M170" t="n">
         <v>69</v>
       </c>
+      <c r="N170" t="n">
+        <v>70</v>
+      </c>
+      <c r="O170" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -7792,6 +8816,12 @@
       <c r="M171" t="n">
         <v>71</v>
       </c>
+      <c r="N171" t="n">
+        <v>73</v>
+      </c>
+      <c r="O171" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -7835,6 +8865,12 @@
       <c r="M172" t="n">
         <v>50</v>
       </c>
+      <c r="N172" t="n">
+        <v>50</v>
+      </c>
+      <c r="O172" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -7878,6 +8914,12 @@
       <c r="M173" t="n">
         <v>70</v>
       </c>
+      <c r="N173" t="n">
+        <v>74</v>
+      </c>
+      <c r="O173" t="n">
+        <v>75</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -7921,6 +8963,12 @@
       <c r="M174" t="n">
         <v>126</v>
       </c>
+      <c r="N174" t="n">
+        <v>126</v>
+      </c>
+      <c r="O174" t="n">
+        <v>126</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -7964,6 +9012,12 @@
       <c r="M175" t="n">
         <v>115</v>
       </c>
+      <c r="N175" t="n">
+        <v>115</v>
+      </c>
+      <c r="O175" t="n">
+        <v>115</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -8007,6 +9061,12 @@
       <c r="M176" t="n">
         <v>38</v>
       </c>
+      <c r="N176" t="n">
+        <v>38</v>
+      </c>
+      <c r="O176" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -8050,6 +9110,12 @@
       <c r="M177" t="n">
         <v>1</v>
       </c>
+      <c r="N177" t="n">
+        <v>1</v>
+      </c>
+      <c r="O177" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -8093,6 +9159,12 @@
       <c r="M178" t="n">
         <v>135</v>
       </c>
+      <c r="N178" t="n">
+        <v>136</v>
+      </c>
+      <c r="O178" t="n">
+        <v>138</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -8136,6 +9208,12 @@
       <c r="M179" t="n">
         <v>128</v>
       </c>
+      <c r="N179" t="n">
+        <v>129</v>
+      </c>
+      <c r="O179" t="n">
+        <v>129</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -8179,6 +9257,12 @@
       <c r="M180" t="n">
         <v>46</v>
       </c>
+      <c r="N180" t="n">
+        <v>50</v>
+      </c>
+      <c r="O180" t="n">
+        <v>53</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -8222,6 +9306,12 @@
       <c r="M181" t="n">
         <v>66</v>
       </c>
+      <c r="N181" t="n">
+        <v>66</v>
+      </c>
+      <c r="O181" t="n">
+        <v>68</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -8265,6 +9355,12 @@
       <c r="M182" t="n">
         <v>32</v>
       </c>
+      <c r="N182" t="n">
+        <v>32</v>
+      </c>
+      <c r="O182" t="n">
+        <v>33</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -8308,6 +9404,12 @@
       <c r="M183" t="n">
         <v>2</v>
       </c>
+      <c r="N183" t="n">
+        <v>2</v>
+      </c>
+      <c r="O183" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -8351,6 +9453,12 @@
       <c r="M184" t="n">
         <v>131</v>
       </c>
+      <c r="N184" t="n">
+        <v>133</v>
+      </c>
+      <c r="O184" t="n">
+        <v>133</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -8394,6 +9502,12 @@
       <c r="M185" t="n">
         <v>118</v>
       </c>
+      <c r="N185" t="n">
+        <v>118</v>
+      </c>
+      <c r="O185" t="n">
+        <v>128</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -8437,6 +9551,12 @@
       <c r="M186" t="n">
         <v>3</v>
       </c>
+      <c r="N186" t="n">
+        <v>3</v>
+      </c>
+      <c r="O186" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -8480,6 +9600,12 @@
       <c r="M187" t="n">
         <v>83</v>
       </c>
+      <c r="N187" t="n">
+        <v>83</v>
+      </c>
+      <c r="O187" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -8523,6 +9649,12 @@
       <c r="M188" t="n">
         <v>60</v>
       </c>
+      <c r="N188" t="n">
+        <v>60</v>
+      </c>
+      <c r="O188" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -8566,6 +9698,12 @@
       <c r="M189" t="n">
         <v>1</v>
       </c>
+      <c r="N189" t="n">
+        <v>1</v>
+      </c>
+      <c r="O189" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -8609,6 +9747,12 @@
       <c r="M190" t="n">
         <v>103</v>
       </c>
+      <c r="N190" t="n">
+        <v>104</v>
+      </c>
+      <c r="O190" t="n">
+        <v>104</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -8652,6 +9796,12 @@
       <c r="M191" t="n">
         <v>63</v>
       </c>
+      <c r="N191" t="n">
+        <v>63</v>
+      </c>
+      <c r="O191" t="n">
+        <v>63</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -8695,6 +9845,12 @@
       <c r="M192" t="n">
         <v>62</v>
       </c>
+      <c r="N192" t="n">
+        <v>62</v>
+      </c>
+      <c r="O192" t="n">
+        <v>62</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -8738,6 +9894,12 @@
       <c r="M193" t="n">
         <v>58</v>
       </c>
+      <c r="N193" t="n">
+        <v>58</v>
+      </c>
+      <c r="O193" t="n">
+        <v>58</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -8781,6 +9943,12 @@
       <c r="M194" t="n">
         <v>44</v>
       </c>
+      <c r="N194" t="n">
+        <v>45</v>
+      </c>
+      <c r="O194" t="n">
+        <v>45</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -8824,6 +9992,12 @@
       <c r="M195" t="n">
         <v>2</v>
       </c>
+      <c r="N195" t="n">
+        <v>2</v>
+      </c>
+      <c r="O195" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -8867,6 +10041,12 @@
       <c r="M196" t="n">
         <v>181</v>
       </c>
+      <c r="N196" t="n">
+        <v>182</v>
+      </c>
+      <c r="O196" t="n">
+        <v>182</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -8910,6 +10090,12 @@
       <c r="M197" t="n">
         <v>1</v>
       </c>
+      <c r="N197" t="n">
+        <v>1</v>
+      </c>
+      <c r="O197" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -8953,6 +10139,12 @@
       <c r="M198" t="n">
         <v>104</v>
       </c>
+      <c r="N198" t="n">
+        <v>105</v>
+      </c>
+      <c r="O198" t="n">
+        <v>105</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -8996,6 +10188,12 @@
       <c r="M199" t="n">
         <v>100</v>
       </c>
+      <c r="N199" t="n">
+        <v>100</v>
+      </c>
+      <c r="O199" t="n">
+        <v>103</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -9039,6 +10237,12 @@
       <c r="M200" t="n">
         <v>25</v>
       </c>
+      <c r="N200" t="n">
+        <v>25</v>
+      </c>
+      <c r="O200" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -9082,6 +10286,12 @@
       <c r="M201" t="n">
         <v>9</v>
       </c>
+      <c r="N201" t="n">
+        <v>9</v>
+      </c>
+      <c r="O201" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -9125,6 +10335,12 @@
       <c r="M202" t="n">
         <v>10</v>
       </c>
+      <c r="N202" t="n">
+        <v>10</v>
+      </c>
+      <c r="O202" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -9168,6 +10384,12 @@
       <c r="M203" t="n">
         <v>15</v>
       </c>
+      <c r="N203" t="n">
+        <v>15</v>
+      </c>
+      <c r="O203" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -9211,6 +10433,12 @@
       <c r="M204" t="n">
         <v>10</v>
       </c>
+      <c r="N204" t="n">
+        <v>10</v>
+      </c>
+      <c r="O204" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -9254,6 +10482,12 @@
       <c r="M205" t="n">
         <v>24</v>
       </c>
+      <c r="N205" t="n">
+        <v>24</v>
+      </c>
+      <c r="O205" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -9297,6 +10531,12 @@
       <c r="M206" t="n">
         <v>22</v>
       </c>
+      <c r="N206" t="n">
+        <v>23</v>
+      </c>
+      <c r="O206" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -9340,6 +10580,12 @@
       <c r="M207" t="n">
         <v>18</v>
       </c>
+      <c r="N207" t="n">
+        <v>18</v>
+      </c>
+      <c r="O207" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -9383,6 +10629,12 @@
       <c r="M208" t="n">
         <v>1</v>
       </c>
+      <c r="N208" t="n">
+        <v>1</v>
+      </c>
+      <c r="O208" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -9426,6 +10678,12 @@
       <c r="M209" t="n">
         <v>22</v>
       </c>
+      <c r="N209" t="n">
+        <v>22</v>
+      </c>
+      <c r="O209" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -9469,6 +10727,12 @@
       <c r="M210" t="n">
         <v>27</v>
       </c>
+      <c r="N210" t="n">
+        <v>27</v>
+      </c>
+      <c r="O210" t="n">
+        <v>27</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -9512,6 +10776,12 @@
       <c r="M211" t="n">
         <v>1</v>
       </c>
+      <c r="N211" t="n">
+        <v>1</v>
+      </c>
+      <c r="O211" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -9555,6 +10825,12 @@
       <c r="M212" t="n">
         <v>53</v>
       </c>
+      <c r="N212" t="n">
+        <v>53</v>
+      </c>
+      <c r="O212" t="n">
+        <v>53</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -9598,6 +10874,12 @@
       <c r="M213" t="n">
         <v>33</v>
       </c>
+      <c r="N213" t="n">
+        <v>33</v>
+      </c>
+      <c r="O213" t="n">
+        <v>33</v>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -9641,6 +10923,12 @@
       <c r="M214" t="n">
         <v>1</v>
       </c>
+      <c r="N214" t="n">
+        <v>1</v>
+      </c>
+      <c r="O214" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -9684,6 +10972,12 @@
       <c r="M215" t="n">
         <v>1</v>
       </c>
+      <c r="N215" t="n">
+        <v>1</v>
+      </c>
+      <c r="O215" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -9727,6 +11021,12 @@
       <c r="M216" t="n">
         <v>58</v>
       </c>
+      <c r="N216" t="n">
+        <v>59</v>
+      </c>
+      <c r="O216" t="n">
+        <v>59</v>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -9770,6 +11070,12 @@
       <c r="M217" t="n">
         <v>29</v>
       </c>
+      <c r="N217" t="n">
+        <v>29</v>
+      </c>
+      <c r="O217" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -9813,6 +11119,12 @@
       <c r="M218" t="n">
         <v>25</v>
       </c>
+      <c r="N218" t="n">
+        <v>25</v>
+      </c>
+      <c r="O218" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -9856,6 +11168,12 @@
       <c r="M219" t="n">
         <v>25</v>
       </c>
+      <c r="N219" t="n">
+        <v>26</v>
+      </c>
+      <c r="O219" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -9899,6 +11217,12 @@
       <c r="M220" t="n">
         <v>24</v>
       </c>
+      <c r="N220" t="n">
+        <v>24</v>
+      </c>
+      <c r="O220" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -9942,6 +11266,12 @@
       <c r="M221" t="n">
         <v>2</v>
       </c>
+      <c r="N221" t="n">
+        <v>2</v>
+      </c>
+      <c r="O221" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -9985,6 +11315,12 @@
       <c r="M222" t="n">
         <v>1</v>
       </c>
+      <c r="N222" t="n">
+        <v>1</v>
+      </c>
+      <c r="O222" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -10028,6 +11364,12 @@
       <c r="M223" t="n">
         <v>49</v>
       </c>
+      <c r="N223" t="n">
+        <v>49</v>
+      </c>
+      <c r="O223" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -10071,6 +11413,12 @@
       <c r="M224" t="n">
         <v>34</v>
       </c>
+      <c r="N224" t="n">
+        <v>35</v>
+      </c>
+      <c r="O224" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -10114,6 +11462,12 @@
       <c r="M225" t="n">
         <v>43</v>
       </c>
+      <c r="N225" t="n">
+        <v>46</v>
+      </c>
+      <c r="O225" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -10157,6 +11511,12 @@
       <c r="M226" t="n">
         <v>78</v>
       </c>
+      <c r="N226" t="n">
+        <v>79</v>
+      </c>
+      <c r="O226" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -10200,6 +11560,12 @@
       <c r="M227" t="n">
         <v>3</v>
       </c>
+      <c r="N227" t="n">
+        <v>3</v>
+      </c>
+      <c r="O227" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -10243,6 +11609,12 @@
       <c r="M228" t="n">
         <v>1</v>
       </c>
+      <c r="N228" t="n">
+        <v>1</v>
+      </c>
+      <c r="O228" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -10286,6 +11658,12 @@
       <c r="M229" t="n">
         <v>86</v>
       </c>
+      <c r="N229" t="n">
+        <v>89</v>
+      </c>
+      <c r="O229" t="n">
+        <v>89</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -10329,6 +11707,12 @@
       <c r="M230" t="n">
         <v>53</v>
       </c>
+      <c r="N230" t="n">
+        <v>61</v>
+      </c>
+      <c r="O230" t="n">
+        <v>61</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -10372,6 +11756,12 @@
       <c r="M231" t="n">
         <v>91</v>
       </c>
+      <c r="N231" t="n">
+        <v>96</v>
+      </c>
+      <c r="O231" t="n">
+        <v>96</v>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -10415,6 +11805,12 @@
       <c r="M232" t="n">
         <v>231</v>
       </c>
+      <c r="N232" t="n">
+        <v>241</v>
+      </c>
+      <c r="O232" t="n">
+        <v>243</v>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -10458,6 +11854,12 @@
       <c r="M233" t="n">
         <v>129</v>
       </c>
+      <c r="N233" t="n">
+        <v>135</v>
+      </c>
+      <c r="O233" t="n">
+        <v>135</v>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -10501,6 +11903,12 @@
       <c r="M234" t="n">
         <v>168</v>
       </c>
+      <c r="N234" t="n">
+        <v>180</v>
+      </c>
+      <c r="O234" t="n">
+        <v>185</v>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -10544,6 +11952,12 @@
       <c r="M235" t="n">
         <v>50</v>
       </c>
+      <c r="N235" t="n">
+        <v>50</v>
+      </c>
+      <c r="O235" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -10587,6 +12001,12 @@
       <c r="M236" t="n">
         <v>31</v>
       </c>
+      <c r="N236" t="n">
+        <v>31</v>
+      </c>
+      <c r="O236" t="n">
+        <v>31</v>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -10630,6 +12050,12 @@
       <c r="M237" t="n">
         <v>196</v>
       </c>
+      <c r="N237" t="n">
+        <v>207</v>
+      </c>
+      <c r="O237" t="n">
+        <v>215</v>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -10673,6 +12099,12 @@
       <c r="M238" t="n">
         <v>104</v>
       </c>
+      <c r="N238" t="n">
+        <v>109</v>
+      </c>
+      <c r="O238" t="n">
+        <v>109</v>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -10716,6 +12148,12 @@
       <c r="M239" t="n">
         <v>93</v>
       </c>
+      <c r="N239" t="n">
+        <v>98</v>
+      </c>
+      <c r="O239" t="n">
+        <v>98</v>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -10759,6 +12197,12 @@
       <c r="M240" t="n">
         <v>38</v>
       </c>
+      <c r="N240" t="n">
+        <v>44</v>
+      </c>
+      <c r="O240" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -10802,6 +12246,12 @@
       <c r="M241" t="n">
         <v>58</v>
       </c>
+      <c r="N241" t="n">
+        <v>59</v>
+      </c>
+      <c r="O241" t="n">
+        <v>61</v>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -10845,6 +12295,12 @@
       <c r="M242" t="n">
         <v>34</v>
       </c>
+      <c r="N242" t="n">
+        <v>34</v>
+      </c>
+      <c r="O242" t="n">
+        <v>34</v>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -10888,6 +12344,12 @@
       <c r="M243" t="n">
         <v>47</v>
       </c>
+      <c r="N243" t="n">
+        <v>47</v>
+      </c>
+      <c r="O243" t="n">
+        <v>47</v>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -10931,6 +12393,12 @@
       <c r="M244" t="n">
         <v>206</v>
       </c>
+      <c r="N244" t="n">
+        <v>224</v>
+      </c>
+      <c r="O244" t="n">
+        <v>234</v>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -10974,6 +12442,12 @@
       <c r="M245" t="n">
         <v>84</v>
       </c>
+      <c r="N245" t="n">
+        <v>88</v>
+      </c>
+      <c r="O245" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -11017,6 +12491,12 @@
       <c r="M246" t="n">
         <v>61</v>
       </c>
+      <c r="N246" t="n">
+        <v>61</v>
+      </c>
+      <c r="O246" t="n">
+        <v>61</v>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -11060,6 +12540,12 @@
       <c r="M247" t="n">
         <v>88</v>
       </c>
+      <c r="N247" t="n">
+        <v>88</v>
+      </c>
+      <c r="O247" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -11103,6 +12589,12 @@
       <c r="M248" t="n">
         <v>39</v>
       </c>
+      <c r="N248" t="n">
+        <v>41</v>
+      </c>
+      <c r="O248" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -11146,6 +12638,12 @@
       <c r="M249" t="n">
         <v>2</v>
       </c>
+      <c r="N249" t="n">
+        <v>2</v>
+      </c>
+      <c r="O249" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -11189,6 +12687,12 @@
       <c r="M250" t="n">
         <v>1</v>
       </c>
+      <c r="N250" t="n">
+        <v>1</v>
+      </c>
+      <c r="O250" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -11232,6 +12736,12 @@
       <c r="M251" t="n">
         <v>2</v>
       </c>
+      <c r="N251" t="n">
+        <v>2</v>
+      </c>
+      <c r="O251" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -11275,6 +12785,12 @@
       <c r="M252" t="n">
         <v>50</v>
       </c>
+      <c r="N252" t="n">
+        <v>52</v>
+      </c>
+      <c r="O252" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -11318,6 +12834,12 @@
       <c r="M253" t="n">
         <v>163</v>
       </c>
+      <c r="N253" t="n">
+        <v>167</v>
+      </c>
+      <c r="O253" t="n">
+        <v>171</v>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -11361,6 +12883,12 @@
       <c r="M254" t="n">
         <v>256</v>
       </c>
+      <c r="N254" t="n">
+        <v>264</v>
+      </c>
+      <c r="O254" t="n">
+        <v>268</v>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -11404,6 +12932,12 @@
       <c r="M255" t="n">
         <v>103</v>
       </c>
+      <c r="N255" t="n">
+        <v>108</v>
+      </c>
+      <c r="O255" t="n">
+        <v>108</v>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -11447,6 +12981,12 @@
       <c r="M256" t="n">
         <v>36</v>
       </c>
+      <c r="N256" t="n">
+        <v>36</v>
+      </c>
+      <c r="O256" t="n">
+        <v>36</v>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -11490,6 +13030,12 @@
       <c r="M257" t="n">
         <v>23</v>
       </c>
+      <c r="N257" t="n">
+        <v>24</v>
+      </c>
+      <c r="O257" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -11533,6 +13079,12 @@
       <c r="M258" t="n">
         <v>315</v>
       </c>
+      <c r="N258" t="n">
+        <v>319</v>
+      </c>
+      <c r="O258" t="n">
+        <v>319</v>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -11576,6 +13128,12 @@
       <c r="M259" t="n">
         <v>1194</v>
       </c>
+      <c r="N259" t="n">
+        <v>1197</v>
+      </c>
+      <c r="O259" t="n">
+        <v>1197</v>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -11619,6 +13177,12 @@
       <c r="M260" t="n">
         <v>196</v>
       </c>
+      <c r="N260" t="n">
+        <v>199</v>
+      </c>
+      <c r="O260" t="n">
+        <v>199</v>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -11662,6 +13226,12 @@
       <c r="M261" t="n">
         <v>205</v>
       </c>
+      <c r="N261" t="n">
+        <v>206</v>
+      </c>
+      <c r="O261" t="n">
+        <v>206</v>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -11705,6 +13275,12 @@
       <c r="M262" t="n">
         <v>239</v>
       </c>
+      <c r="N262" t="n">
+        <v>240</v>
+      </c>
+      <c r="O262" t="n">
+        <v>241</v>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -11748,6 +13324,12 @@
       <c r="M263" t="n">
         <v>268</v>
       </c>
+      <c r="N263" t="n">
+        <v>269</v>
+      </c>
+      <c r="O263" t="n">
+        <v>269</v>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -11791,6 +13373,12 @@
       <c r="M264" t="n">
         <v>61</v>
       </c>
+      <c r="N264" t="n">
+        <v>61</v>
+      </c>
+      <c r="O264" t="n">
+        <v>61</v>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -11834,6 +13422,12 @@
       <c r="M265" t="n">
         <v>142</v>
       </c>
+      <c r="N265" t="n">
+        <v>145</v>
+      </c>
+      <c r="O265" t="n">
+        <v>145</v>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -11877,6 +13471,12 @@
       <c r="M266" t="n">
         <v>66</v>
       </c>
+      <c r="N266" t="n">
+        <v>67</v>
+      </c>
+      <c r="O266" t="n">
+        <v>67</v>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -11920,6 +13520,12 @@
       <c r="M267" t="n">
         <v>12</v>
       </c>
+      <c r="N267" t="n">
+        <v>12</v>
+      </c>
+      <c r="O267" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -11963,6 +13569,12 @@
       <c r="M268" t="n">
         <v>100</v>
       </c>
+      <c r="N268" t="n">
+        <v>101</v>
+      </c>
+      <c r="O268" t="n">
+        <v>101</v>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -12006,6 +13618,12 @@
       <c r="M269" t="n">
         <v>92</v>
       </c>
+      <c r="N269" t="n">
+        <v>92</v>
+      </c>
+      <c r="O269" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -12049,6 +13667,12 @@
       <c r="M270" t="n">
         <v>26</v>
       </c>
+      <c r="N270" t="n">
+        <v>26</v>
+      </c>
+      <c r="O270" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -12092,6 +13716,12 @@
       <c r="M271" t="n">
         <v>29</v>
       </c>
+      <c r="N271" t="n">
+        <v>30</v>
+      </c>
+      <c r="O271" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -12135,6 +13765,12 @@
       <c r="M272" t="n">
         <v>228</v>
       </c>
+      <c r="N272" t="n">
+        <v>233</v>
+      </c>
+      <c r="O272" t="n">
+        <v>233</v>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -12178,6 +13814,12 @@
       <c r="M273" t="n">
         <v>270</v>
       </c>
+      <c r="N273" t="n">
+        <v>271</v>
+      </c>
+      <c r="O273" t="n">
+        <v>274</v>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -12221,6 +13863,12 @@
       <c r="M274" t="n">
         <v>85</v>
       </c>
+      <c r="N274" t="n">
+        <v>85</v>
+      </c>
+      <c r="O274" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -12264,6 +13912,12 @@
       <c r="M275" t="n">
         <v>100</v>
       </c>
+      <c r="N275" t="n">
+        <v>102</v>
+      </c>
+      <c r="O275" t="n">
+        <v>103</v>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -12307,6 +13961,12 @@
       <c r="M276" t="n">
         <v>93</v>
       </c>
+      <c r="N276" t="n">
+        <v>93</v>
+      </c>
+      <c r="O276" t="n">
+        <v>93</v>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -12350,6 +14010,12 @@
       <c r="M277" t="n">
         <v>3</v>
       </c>
+      <c r="N277" t="n">
+        <v>3</v>
+      </c>
+      <c r="O277" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -12393,6 +14059,12 @@
       <c r="M278" t="n">
         <v>141</v>
       </c>
+      <c r="N278" t="n">
+        <v>143</v>
+      </c>
+      <c r="O278" t="n">
+        <v>146</v>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -12436,6 +14108,12 @@
       <c r="M279" t="n">
         <v>155</v>
       </c>
+      <c r="N279" t="n">
+        <v>155</v>
+      </c>
+      <c r="O279" t="n">
+        <v>155</v>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -12479,6 +14157,12 @@
       <c r="M280" t="n">
         <v>97</v>
       </c>
+      <c r="N280" t="n">
+        <v>101</v>
+      </c>
+      <c r="O280" t="n">
+        <v>104</v>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -12522,6 +14206,12 @@
       <c r="M281" t="n">
         <v>102</v>
       </c>
+      <c r="N281" t="n">
+        <v>103</v>
+      </c>
+      <c r="O281" t="n">
+        <v>104</v>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -12565,6 +14255,12 @@
       <c r="M282" t="n">
         <v>94</v>
       </c>
+      <c r="N282" t="n">
+        <v>101</v>
+      </c>
+      <c r="O282" t="n">
+        <v>101</v>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -12608,6 +14304,12 @@
       <c r="M283" t="n">
         <v>117</v>
       </c>
+      <c r="N283" t="n">
+        <v>120</v>
+      </c>
+      <c r="O283" t="n">
+        <v>122</v>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -12651,6 +14353,12 @@
       <c r="M284" t="n">
         <v>292</v>
       </c>
+      <c r="N284" t="n">
+        <v>294</v>
+      </c>
+      <c r="O284" t="n">
+        <v>298</v>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -12694,6 +14402,12 @@
       <c r="M285" t="n">
         <v>25</v>
       </c>
+      <c r="N285" t="n">
+        <v>26</v>
+      </c>
+      <c r="O285" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -12737,6 +14451,12 @@
       <c r="M286" t="n">
         <v>35</v>
       </c>
+      <c r="N286" t="n">
+        <v>37</v>
+      </c>
+      <c r="O286" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -12780,6 +14500,12 @@
       <c r="M287" t="n">
         <v>100</v>
       </c>
+      <c r="N287" t="n">
+        <v>107</v>
+      </c>
+      <c r="O287" t="n">
+        <v>110</v>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -12823,6 +14549,12 @@
       <c r="M288" t="n">
         <v>304</v>
       </c>
+      <c r="N288" t="n">
+        <v>312</v>
+      </c>
+      <c r="O288" t="n">
+        <v>313</v>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -12866,6 +14598,12 @@
       <c r="M289" t="n">
         <v>122</v>
       </c>
+      <c r="N289" t="n">
+        <v>125</v>
+      </c>
+      <c r="O289" t="n">
+        <v>129</v>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -12909,6 +14647,12 @@
       <c r="M290" t="n">
         <v>22</v>
       </c>
+      <c r="N290" t="n">
+        <v>24</v>
+      </c>
+      <c r="O290" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -12952,6 +14696,12 @@
       <c r="M291" t="n">
         <v>24</v>
       </c>
+      <c r="N291" t="n">
+        <v>24</v>
+      </c>
+      <c r="O291" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -12995,6 +14745,12 @@
       <c r="M292" t="n">
         <v>14</v>
       </c>
+      <c r="N292" t="n">
+        <v>14</v>
+      </c>
+      <c r="O292" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -13038,6 +14794,12 @@
       <c r="M293" t="n">
         <v>136</v>
       </c>
+      <c r="N293" t="n">
+        <v>139</v>
+      </c>
+      <c r="O293" t="n">
+        <v>147</v>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -13081,6 +14843,12 @@
       <c r="M294" t="n">
         <v>122</v>
       </c>
+      <c r="N294" t="n">
+        <v>129</v>
+      </c>
+      <c r="O294" t="n">
+        <v>130</v>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -13124,6 +14892,12 @@
       <c r="M295" t="n">
         <v>46</v>
       </c>
+      <c r="N295" t="n">
+        <v>48</v>
+      </c>
+      <c r="O295" t="n">
+        <v>52</v>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -13167,6 +14941,12 @@
       <c r="M296" t="n">
         <v>20</v>
       </c>
+      <c r="N296" t="n">
+        <v>21</v>
+      </c>
+      <c r="O296" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -13210,6 +14990,12 @@
       <c r="M297" t="n">
         <v>42</v>
       </c>
+      <c r="N297" t="n">
+        <v>43</v>
+      </c>
+      <c r="O297" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -13253,6 +15039,12 @@
       <c r="M298" t="n">
         <v>19</v>
       </c>
+      <c r="N298" t="n">
+        <v>19</v>
+      </c>
+      <c r="O298" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -13296,6 +15088,12 @@
       <c r="M299" t="n">
         <v>26</v>
       </c>
+      <c r="N299" t="n">
+        <v>26</v>
+      </c>
+      <c r="O299" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -13339,6 +15137,12 @@
       <c r="M300" t="n">
         <v>25</v>
       </c>
+      <c r="N300" t="n">
+        <v>28</v>
+      </c>
+      <c r="O300" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -13382,6 +15186,12 @@
       <c r="M301" t="n">
         <v>158</v>
       </c>
+      <c r="N301" t="n">
+        <v>192</v>
+      </c>
+      <c r="O301" t="n">
+        <v>227</v>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -13425,6 +15235,12 @@
       <c r="M302" t="n">
         <v>46</v>
       </c>
+      <c r="N302" t="n">
+        <v>49</v>
+      </c>
+      <c r="O302" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -13468,6 +15284,12 @@
       <c r="M303" t="n">
         <v>72</v>
       </c>
+      <c r="N303" t="n">
+        <v>72</v>
+      </c>
+      <c r="O303" t="n">
+        <v>74</v>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -13511,6 +15333,12 @@
       <c r="M304" t="n">
         <v>82</v>
       </c>
+      <c r="N304" t="n">
+        <v>91</v>
+      </c>
+      <c r="O304" t="n">
+        <v>108</v>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -13554,6 +15382,12 @@
       <c r="M305" t="n">
         <v>21</v>
       </c>
+      <c r="N305" t="n">
+        <v>23</v>
+      </c>
+      <c r="O305" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -13597,6 +15431,12 @@
       <c r="M306" t="n">
         <v>27</v>
       </c>
+      <c r="N306" t="n">
+        <v>28</v>
+      </c>
+      <c r="O306" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -13620,7 +15460,7 @@
         <v>10</v>
       </c>
       <c r="G307" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H307" t="n">
         <v>13</v>
@@ -13635,11 +15475,17 @@
         <v>1</v>
       </c>
       <c r="L307" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M307" t="n">
         <v>83</v>
       </c>
+      <c r="N307" t="n">
+        <v>92</v>
+      </c>
+      <c r="O307" t="n">
+        <v>105</v>
+      </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -13666,7 +15512,7 @@
         <v>62</v>
       </c>
       <c r="H308" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I308" t="n">
         <v>0</v>
@@ -13678,11 +15524,17 @@
         <v>0</v>
       </c>
       <c r="L308" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="M308" t="n">
         <v>119</v>
       </c>
+      <c r="N308" t="n">
+        <v>127</v>
+      </c>
+      <c r="O308" t="n">
+        <v>136</v>
+      </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -13691,7 +15543,7 @@
         </is>
       </c>
       <c r="B309" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C309" t="n">
         <v>1</v>
@@ -13706,7 +15558,7 @@
         <v>1</v>
       </c>
       <c r="G309" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="H309" t="n">
         <v>3</v>
@@ -13715,16 +15567,22 @@
         <v>1</v>
       </c>
       <c r="J309" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K309" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L309" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="M309" t="n">
-        <v>14</v>
+        <v>44</v>
+      </c>
+      <c r="N309" t="n">
+        <v>44</v>
+      </c>
+      <c r="O309" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="310">
@@ -13734,28 +15592,28 @@
         </is>
       </c>
       <c r="B310" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C310" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D310" t="n">
+        <v>12</v>
+      </c>
+      <c r="E310" t="n">
+        <v>22</v>
+      </c>
+      <c r="F310" t="n">
+        <v>28</v>
+      </c>
+      <c r="G310" t="n">
+        <v>57</v>
+      </c>
+      <c r="H310" t="n">
         <v>11</v>
       </c>
-      <c r="E310" t="n">
-        <v>18</v>
-      </c>
-      <c r="F310" t="n">
-        <v>18</v>
-      </c>
-      <c r="G310" t="n">
-        <v>41</v>
-      </c>
-      <c r="H310" t="n">
-        <v>7</v>
-      </c>
       <c r="I310" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J310" t="n">
         <v>1</v>
@@ -13764,10 +15622,16 @@
         <v>1</v>
       </c>
       <c r="L310" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="M310" t="n">
-        <v>108</v>
+        <v>155</v>
+      </c>
+      <c r="N310" t="n">
+        <v>233</v>
+      </c>
+      <c r="O310" t="n">
+        <v>290</v>
       </c>
     </row>
     <row r="311">
@@ -13777,40 +15641,193 @@
         </is>
       </c>
       <c r="B311" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C311" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D311" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="E311" t="n">
-        <v>3</v>
+        <v>34</v>
       </c>
       <c r="F311" t="n">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="G311" t="n">
+        <v>89</v>
+      </c>
+      <c r="H311" t="n">
+        <v>14</v>
+      </c>
+      <c r="I311" t="n">
+        <v>12</v>
+      </c>
+      <c r="J311" t="n">
+        <v>1</v>
+      </c>
+      <c r="K311" t="n">
+        <v>1</v>
+      </c>
+      <c r="L311" t="n">
+        <v>31</v>
+      </c>
+      <c r="M311" t="n">
+        <v>237</v>
+      </c>
+      <c r="N311" t="n">
+        <v>334</v>
+      </c>
+      <c r="O311" t="n">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+      <c r="B312" t="n">
+        <v>9</v>
+      </c>
+      <c r="C312" t="n">
+        <v>8</v>
+      </c>
+      <c r="D312" t="n">
         <v>15</v>
       </c>
-      <c r="H311" t="n">
-        <v>2</v>
-      </c>
-      <c r="I311" t="n">
-        <v>3</v>
-      </c>
-      <c r="J311" t="n">
-        <v>1</v>
-      </c>
-      <c r="K311" t="n">
-        <v>0</v>
-      </c>
-      <c r="L311" t="n">
-        <v>10</v>
-      </c>
-      <c r="M311" t="n">
-        <v>37</v>
+      <c r="E312" t="n">
+        <v>25</v>
+      </c>
+      <c r="F312" t="n">
+        <v>45</v>
+      </c>
+      <c r="G312" t="n">
+        <v>76</v>
+      </c>
+      <c r="H312" t="n">
+        <v>8</v>
+      </c>
+      <c r="I312" t="n">
+        <v>6</v>
+      </c>
+      <c r="J312" t="n">
+        <v>2</v>
+      </c>
+      <c r="K312" t="n">
+        <v>0</v>
+      </c>
+      <c r="L312" t="n">
+        <v>27</v>
+      </c>
+      <c r="M312" t="n">
+        <v>221</v>
+      </c>
+      <c r="N312" t="n">
+        <v>318</v>
+      </c>
+      <c r="O312" t="n">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B313" t="n">
+        <v>8</v>
+      </c>
+      <c r="C313" t="n">
+        <v>3</v>
+      </c>
+      <c r="D313" t="n">
+        <v>9</v>
+      </c>
+      <c r="E313" t="n">
+        <v>18</v>
+      </c>
+      <c r="F313" t="n">
+        <v>19</v>
+      </c>
+      <c r="G313" t="n">
+        <v>47</v>
+      </c>
+      <c r="H313" t="n">
+        <v>3</v>
+      </c>
+      <c r="I313" t="n">
+        <v>5</v>
+      </c>
+      <c r="J313" t="n">
+        <v>1</v>
+      </c>
+      <c r="K313" t="n">
+        <v>0</v>
+      </c>
+      <c r="L313" t="n">
+        <v>26</v>
+      </c>
+      <c r="M313" t="n">
+        <v>139</v>
+      </c>
+      <c r="N313" t="n">
+        <v>184</v>
+      </c>
+      <c r="O313" t="n">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B314" t="n">
+        <v>0</v>
+      </c>
+      <c r="C314" t="n">
+        <v>0</v>
+      </c>
+      <c r="D314" t="n">
+        <v>0</v>
+      </c>
+      <c r="E314" t="n">
+        <v>2</v>
+      </c>
+      <c r="F314" t="n">
+        <v>2</v>
+      </c>
+      <c r="G314" t="n">
+        <v>1</v>
+      </c>
+      <c r="H314" t="n">
+        <v>1</v>
+      </c>
+      <c r="I314" t="n">
+        <v>0</v>
+      </c>
+      <c r="J314" t="n">
+        <v>0</v>
+      </c>
+      <c r="K314" t="n">
+        <v>0</v>
+      </c>
+      <c r="L314" t="n">
+        <v>6</v>
+      </c>
+      <c r="M314" t="n">
+        <v>12</v>
+      </c>
+      <c r="N314" t="n">
+        <v>18</v>
+      </c>
+      <c r="O314" t="n">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily auto-refresh 2026-08-18 12:55
</commit_message>
<xml_diff>
--- a/daily_slab_mix.xlsx
+++ b/daily_slab_mix.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O307"/>
+  <dimension ref="A1:Q307"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -492,6 +492,16 @@
           <t>Sample units</t>
         </is>
       </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Gift units (Turmeric Ginger)</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Units incl. gifts</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -541,6 +551,12 @@
       <c r="O2" t="n">
         <v>4</v>
       </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -590,6 +606,12 @@
       <c r="O3" t="n">
         <v>3</v>
       </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -639,6 +661,12 @@
       <c r="O4" t="n">
         <v>1</v>
       </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -688,6 +716,12 @@
       <c r="O5" t="n">
         <v>2</v>
       </c>
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -737,6 +771,12 @@
       <c r="O6" t="n">
         <v>17</v>
       </c>
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -786,6 +826,12 @@
       <c r="O7" t="n">
         <v>3</v>
       </c>
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -835,6 +881,12 @@
       <c r="O8" t="n">
         <v>1</v>
       </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -884,6 +936,12 @@
       <c r="O9" t="n">
         <v>6</v>
       </c>
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -933,6 +991,12 @@
       <c r="O10" t="n">
         <v>4</v>
       </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -982,6 +1046,12 @@
       <c r="O11" t="n">
         <v>1</v>
       </c>
+      <c r="P11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1031,6 +1101,12 @@
       <c r="O12" t="n">
         <v>5</v>
       </c>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1080,6 +1156,12 @@
       <c r="O13" t="n">
         <v>6</v>
       </c>
+      <c r="P13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1129,6 +1211,12 @@
       <c r="O14" t="n">
         <v>9</v>
       </c>
+      <c r="P14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1178,6 +1266,12 @@
       <c r="O15" t="n">
         <v>7</v>
       </c>
+      <c r="P15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1227,6 +1321,12 @@
       <c r="O16" t="n">
         <v>21</v>
       </c>
+      <c r="P16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1276,6 +1376,12 @@
       <c r="O17" t="n">
         <v>15</v>
       </c>
+      <c r="P17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1325,6 +1431,12 @@
       <c r="O18" t="n">
         <v>34</v>
       </c>
+      <c r="P18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>34</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1374,6 +1486,12 @@
       <c r="O19" t="n">
         <v>28</v>
       </c>
+      <c r="P19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1423,6 +1541,12 @@
       <c r="O20" t="n">
         <v>26</v>
       </c>
+      <c r="P20" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1472,6 +1596,12 @@
       <c r="O21" t="n">
         <v>1</v>
       </c>
+      <c r="P21" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1521,6 +1651,12 @@
       <c r="O22" t="n">
         <v>29</v>
       </c>
+      <c r="P22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1570,6 +1706,12 @@
       <c r="O23" t="n">
         <v>29</v>
       </c>
+      <c r="P23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1619,6 +1761,12 @@
       <c r="O24" t="n">
         <v>22</v>
       </c>
+      <c r="P24" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1668,6 +1816,12 @@
       <c r="O25" t="n">
         <v>21</v>
       </c>
+      <c r="P25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1717,6 +1871,12 @@
       <c r="O26" t="n">
         <v>14</v>
       </c>
+      <c r="P26" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1766,6 +1926,12 @@
       <c r="O27" t="n">
         <v>18</v>
       </c>
+      <c r="P27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1815,6 +1981,12 @@
       <c r="O28" t="n">
         <v>10</v>
       </c>
+      <c r="P28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1864,6 +2036,12 @@
       <c r="O29" t="n">
         <v>14</v>
       </c>
+      <c r="P29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1913,6 +2091,12 @@
       <c r="O30" t="n">
         <v>27</v>
       </c>
+      <c r="P30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>27</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1962,6 +2146,12 @@
       <c r="O31" t="n">
         <v>22</v>
       </c>
+      <c r="P31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2011,6 +2201,12 @@
       <c r="O32" t="n">
         <v>15</v>
       </c>
+      <c r="P32" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2060,6 +2256,12 @@
       <c r="O33" t="n">
         <v>34</v>
       </c>
+      <c r="P33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>34</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2109,6 +2311,12 @@
       <c r="O34" t="n">
         <v>9</v>
       </c>
+      <c r="P34" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2158,6 +2366,12 @@
       <c r="O35" t="n">
         <v>3</v>
       </c>
+      <c r="P35" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2207,6 +2421,12 @@
       <c r="O36" t="n">
         <v>23</v>
       </c>
+      <c r="P36" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2256,6 +2476,12 @@
       <c r="O37" t="n">
         <v>1</v>
       </c>
+      <c r="P37" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2305,6 +2531,12 @@
       <c r="O38" t="n">
         <v>5</v>
       </c>
+      <c r="P38" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2354,6 +2586,12 @@
       <c r="O39" t="n">
         <v>12</v>
       </c>
+      <c r="P39" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2403,6 +2641,12 @@
       <c r="O40" t="n">
         <v>19</v>
       </c>
+      <c r="P40" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2452,6 +2696,12 @@
       <c r="O41" t="n">
         <v>24</v>
       </c>
+      <c r="P41" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2501,6 +2751,12 @@
       <c r="O42" t="n">
         <v>24</v>
       </c>
+      <c r="P42" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2550,6 +2806,12 @@
       <c r="O43" t="n">
         <v>13</v>
       </c>
+      <c r="P43" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2599,6 +2861,12 @@
       <c r="O44" t="n">
         <v>1</v>
       </c>
+      <c r="P44" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2648,6 +2916,12 @@
       <c r="O45" t="n">
         <v>10</v>
       </c>
+      <c r="P45" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2697,6 +2971,12 @@
       <c r="O46" t="n">
         <v>31</v>
       </c>
+      <c r="P46" t="n">
+        <v>21</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>52</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2746,6 +3026,12 @@
       <c r="O47" t="n">
         <v>36</v>
       </c>
+      <c r="P47" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>44</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2795,6 +3081,12 @@
       <c r="O48" t="n">
         <v>49</v>
       </c>
+      <c r="P48" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>58</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2844,6 +3136,12 @@
       <c r="O49" t="n">
         <v>24</v>
       </c>
+      <c r="P49" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2893,6 +3191,12 @@
       <c r="O50" t="n">
         <v>38</v>
       </c>
+      <c r="P50" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2942,6 +3246,12 @@
       <c r="O51" t="n">
         <v>3</v>
       </c>
+      <c r="P51" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2991,6 +3301,12 @@
       <c r="O52" t="n">
         <v>3</v>
       </c>
+      <c r="P52" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3040,6 +3356,12 @@
       <c r="O53" t="n">
         <v>31</v>
       </c>
+      <c r="P53" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3089,6 +3411,12 @@
       <c r="O54" t="n">
         <v>1</v>
       </c>
+      <c r="P54" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3138,6 +3466,12 @@
       <c r="O55" t="n">
         <v>3</v>
       </c>
+      <c r="P55" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q55" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3187,6 +3521,12 @@
       <c r="O56" t="n">
         <v>70</v>
       </c>
+      <c r="P56" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>72</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3236,6 +3576,12 @@
       <c r="O57" t="n">
         <v>26</v>
       </c>
+      <c r="P57" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3285,6 +3631,12 @@
       <c r="O58" t="n">
         <v>44</v>
       </c>
+      <c r="P58" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>47</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3334,6 +3686,12 @@
       <c r="O59" t="n">
         <v>29</v>
       </c>
+      <c r="P59" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q59" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3383,6 +3741,12 @@
       <c r="O60" t="n">
         <v>39</v>
       </c>
+      <c r="P60" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3432,6 +3796,12 @@
       <c r="O61" t="n">
         <v>27</v>
       </c>
+      <c r="P61" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q61" t="n">
+        <v>27</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3481,6 +3851,12 @@
       <c r="O62" t="n">
         <v>18</v>
       </c>
+      <c r="P62" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q62" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3530,6 +3906,12 @@
       <c r="O63" t="n">
         <v>1</v>
       </c>
+      <c r="P63" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q63" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3579,6 +3961,12 @@
       <c r="O64" t="n">
         <v>32</v>
       </c>
+      <c r="P64" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q64" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3628,6 +4016,12 @@
       <c r="O65" t="n">
         <v>41</v>
       </c>
+      <c r="P65" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3677,6 +4071,12 @@
       <c r="O66" t="n">
         <v>3</v>
       </c>
+      <c r="P66" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3726,6 +4126,12 @@
       <c r="O67" t="n">
         <v>38</v>
       </c>
+      <c r="P67" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>39</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3775,6 +4181,12 @@
       <c r="O68" t="n">
         <v>29</v>
       </c>
+      <c r="P68" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q68" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3824,6 +4236,12 @@
       <c r="O69" t="n">
         <v>4</v>
       </c>
+      <c r="P69" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q69" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3873,6 +4291,12 @@
       <c r="O70" t="n">
         <v>29</v>
       </c>
+      <c r="P70" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q70" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3922,6 +4346,12 @@
       <c r="O71" t="n">
         <v>35</v>
       </c>
+      <c r="P71" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q71" t="n">
+        <v>35</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3971,6 +4401,12 @@
       <c r="O72" t="n">
         <v>35</v>
       </c>
+      <c r="P72" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q72" t="n">
+        <v>35</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4020,6 +4456,12 @@
       <c r="O73" t="n">
         <v>12</v>
       </c>
+      <c r="P73" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q73" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -4069,6 +4511,12 @@
       <c r="O74" t="n">
         <v>46</v>
       </c>
+      <c r="P74" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q74" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4118,6 +4566,12 @@
       <c r="O75" t="n">
         <v>25</v>
       </c>
+      <c r="P75" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q75" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4167,6 +4621,12 @@
       <c r="O76" t="n">
         <v>2</v>
       </c>
+      <c r="P76" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q76" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4216,6 +4676,12 @@
       <c r="O77" t="n">
         <v>10</v>
       </c>
+      <c r="P77" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q77" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4265,6 +4731,12 @@
       <c r="O78" t="n">
         <v>57</v>
       </c>
+      <c r="P78" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q78" t="n">
+        <v>63</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4314,6 +4786,12 @@
       <c r="O79" t="n">
         <v>40</v>
       </c>
+      <c r="P79" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q79" t="n">
+        <v>44</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4363,6 +4841,12 @@
       <c r="O80" t="n">
         <v>24</v>
       </c>
+      <c r="P80" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q80" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4412,6 +4896,12 @@
       <c r="O81" t="n">
         <v>11</v>
       </c>
+      <c r="P81" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q81" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4461,6 +4951,12 @@
       <c r="O82" t="n">
         <v>22</v>
       </c>
+      <c r="P82" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q82" t="n">
+        <v>39</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4510,6 +5006,12 @@
       <c r="O83" t="n">
         <v>1</v>
       </c>
+      <c r="P83" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q83" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4559,6 +5061,12 @@
       <c r="O84" t="n">
         <v>16</v>
       </c>
+      <c r="P84" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q84" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4608,6 +5116,12 @@
       <c r="O85" t="n">
         <v>20</v>
       </c>
+      <c r="P85" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q85" t="n">
+        <v>35</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4657,6 +5171,12 @@
       <c r="O86" t="n">
         <v>36</v>
       </c>
+      <c r="P86" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q86" t="n">
+        <v>51</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4706,6 +5226,12 @@
       <c r="O87" t="n">
         <v>21</v>
       </c>
+      <c r="P87" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q87" t="n">
+        <v>36</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4755,6 +5281,12 @@
       <c r="O88" t="n">
         <v>23</v>
       </c>
+      <c r="P88" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q88" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4804,6 +5336,12 @@
       <c r="O89" t="n">
         <v>14</v>
       </c>
+      <c r="P89" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q89" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4853,6 +5391,12 @@
       <c r="O90" t="n">
         <v>13</v>
       </c>
+      <c r="P90" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q90" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4902,6 +5446,12 @@
       <c r="O91" t="n">
         <v>39</v>
       </c>
+      <c r="P91" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q91" t="n">
+        <v>39</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4951,6 +5501,12 @@
       <c r="O92" t="n">
         <v>28</v>
       </c>
+      <c r="P92" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q92" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -5000,6 +5556,12 @@
       <c r="O93" t="n">
         <v>21</v>
       </c>
+      <c r="P93" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q93" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -5049,6 +5611,12 @@
       <c r="O94" t="n">
         <v>46</v>
       </c>
+      <c r="P94" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q94" t="n">
+        <v>61</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -5098,6 +5666,12 @@
       <c r="O95" t="n">
         <v>19</v>
       </c>
+      <c r="P95" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q95" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -5147,6 +5721,12 @@
       <c r="O96" t="n">
         <v>8</v>
       </c>
+      <c r="P96" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q96" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -5196,6 +5776,12 @@
       <c r="O97" t="n">
         <v>2</v>
       </c>
+      <c r="P97" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q97" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -5245,6 +5831,12 @@
       <c r="O98" t="n">
         <v>21</v>
       </c>
+      <c r="P98" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q98" t="n">
+        <v>27</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -5294,6 +5886,12 @@
       <c r="O99" t="n">
         <v>23</v>
       </c>
+      <c r="P99" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q99" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -5343,6 +5941,12 @@
       <c r="O100" t="n">
         <v>1</v>
       </c>
+      <c r="P100" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q100" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -5392,6 +5996,12 @@
       <c r="O101" t="n">
         <v>42</v>
       </c>
+      <c r="P101" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q101" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -5441,6 +6051,12 @@
       <c r="O102" t="n">
         <v>27</v>
       </c>
+      <c r="P102" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q102" t="n">
+        <v>37</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -5490,6 +6106,12 @@
       <c r="O103" t="n">
         <v>6</v>
       </c>
+      <c r="P103" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q103" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -5539,6 +6161,12 @@
       <c r="O104" t="n">
         <v>53</v>
       </c>
+      <c r="P104" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q104" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -5588,6 +6216,12 @@
       <c r="O105" t="n">
         <v>29</v>
       </c>
+      <c r="P105" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q105" t="n">
+        <v>33</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -5637,6 +6271,12 @@
       <c r="O106" t="n">
         <v>19</v>
       </c>
+      <c r="P106" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q106" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -5686,6 +6326,12 @@
       <c r="O107" t="n">
         <v>1</v>
       </c>
+      <c r="P107" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q107" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -5735,6 +6381,12 @@
       <c r="O108" t="n">
         <v>2</v>
       </c>
+      <c r="P108" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q108" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -5784,6 +6436,12 @@
       <c r="O109" t="n">
         <v>3</v>
       </c>
+      <c r="P109" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q109" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -5833,6 +6491,12 @@
       <c r="O110" t="n">
         <v>27</v>
       </c>
+      <c r="P110" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q110" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -5882,6 +6546,12 @@
       <c r="O111" t="n">
         <v>19</v>
       </c>
+      <c r="P111" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q111" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -5931,6 +6601,12 @@
       <c r="O112" t="n">
         <v>34</v>
       </c>
+      <c r="P112" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q112" t="n">
+        <v>36</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -5980,6 +6656,12 @@
       <c r="O113" t="n">
         <v>5</v>
       </c>
+      <c r="P113" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q113" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -6029,6 +6711,12 @@
       <c r="O114" t="n">
         <v>40</v>
       </c>
+      <c r="P114" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q114" t="n">
+        <v>56</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -6078,6 +6766,12 @@
       <c r="O115" t="n">
         <v>46</v>
       </c>
+      <c r="P115" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q115" t="n">
+        <v>56</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -6127,6 +6821,12 @@
       <c r="O116" t="n">
         <v>33</v>
       </c>
+      <c r="P116" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q116" t="n">
+        <v>36</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -6176,6 +6876,12 @@
       <c r="O117" t="n">
         <v>26</v>
       </c>
+      <c r="P117" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q117" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -6225,6 +6931,12 @@
       <c r="O118" t="n">
         <v>31</v>
       </c>
+      <c r="P118" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q118" t="n">
+        <v>37</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -6274,6 +6986,12 @@
       <c r="O119" t="n">
         <v>142</v>
       </c>
+      <c r="P119" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q119" t="n">
+        <v>156</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -6323,6 +7041,12 @@
       <c r="O120" t="n">
         <v>41</v>
       </c>
+      <c r="P120" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q120" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -6372,6 +7096,12 @@
       <c r="O121" t="n">
         <v>34</v>
       </c>
+      <c r="P121" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q121" t="n">
+        <v>34</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -6421,6 +7151,12 @@
       <c r="O122" t="n">
         <v>24</v>
       </c>
+      <c r="P122" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q122" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -6470,6 +7206,12 @@
       <c r="O123" t="n">
         <v>13</v>
       </c>
+      <c r="P123" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q123" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -6519,6 +7261,12 @@
       <c r="O124" t="n">
         <v>98</v>
       </c>
+      <c r="P124" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q124" t="n">
+        <v>103</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -6568,6 +7316,12 @@
       <c r="O125" t="n">
         <v>12</v>
       </c>
+      <c r="P125" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q125" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -6617,6 +7371,12 @@
       <c r="O126" t="n">
         <v>29</v>
       </c>
+      <c r="P126" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q126" t="n">
+        <v>35</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -6666,6 +7426,12 @@
       <c r="O127" t="n">
         <v>24</v>
       </c>
+      <c r="P127" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q127" t="n">
+        <v>27</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -6715,6 +7481,12 @@
       <c r="O128" t="n">
         <v>21</v>
       </c>
+      <c r="P128" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q128" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -6764,6 +7536,12 @@
       <c r="O129" t="n">
         <v>33</v>
       </c>
+      <c r="P129" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q129" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -6813,6 +7591,12 @@
       <c r="O130" t="n">
         <v>5</v>
       </c>
+      <c r="P130" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q130" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -6862,6 +7646,12 @@
       <c r="O131" t="n">
         <v>2</v>
       </c>
+      <c r="P131" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q131" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -6911,6 +7701,12 @@
       <c r="O132" t="n">
         <v>81</v>
       </c>
+      <c r="P132" t="n">
+        <v>25</v>
+      </c>
+      <c r="Q132" t="n">
+        <v>106</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -6960,6 +7756,12 @@
       <c r="O133" t="n">
         <v>25</v>
       </c>
+      <c r="P133" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q133" t="n">
+        <v>42</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -7009,6 +7811,12 @@
       <c r="O134" t="n">
         <v>32</v>
       </c>
+      <c r="P134" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q134" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -7058,6 +7866,12 @@
       <c r="O135" t="n">
         <v>60</v>
       </c>
+      <c r="P135" t="n">
+        <v>28</v>
+      </c>
+      <c r="Q135" t="n">
+        <v>88</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -7107,6 +7921,12 @@
       <c r="O136" t="n">
         <v>28</v>
       </c>
+      <c r="P136" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q136" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -7156,6 +7976,12 @@
       <c r="O137" t="n">
         <v>2</v>
       </c>
+      <c r="P137" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q137" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -7205,6 +8031,12 @@
       <c r="O138" t="n">
         <v>34</v>
       </c>
+      <c r="P138" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q138" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -7254,6 +8086,12 @@
       <c r="O139" t="n">
         <v>45</v>
       </c>
+      <c r="P139" t="n">
+        <v>31</v>
+      </c>
+      <c r="Q139" t="n">
+        <v>76</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -7303,6 +8141,12 @@
       <c r="O140" t="n">
         <v>45</v>
       </c>
+      <c r="P140" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q140" t="n">
+        <v>75</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -7352,6 +8196,12 @@
       <c r="O141" t="n">
         <v>35</v>
       </c>
+      <c r="P141" t="n">
+        <v>28</v>
+      </c>
+      <c r="Q141" t="n">
+        <v>63</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -7401,6 +8251,12 @@
       <c r="O142" t="n">
         <v>29</v>
       </c>
+      <c r="P142" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q142" t="n">
+        <v>45</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -7450,6 +8306,12 @@
       <c r="O143" t="n">
         <v>50</v>
       </c>
+      <c r="P143" t="n">
+        <v>28</v>
+      </c>
+      <c r="Q143" t="n">
+        <v>78</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -7499,6 +8361,12 @@
       <c r="O144" t="n">
         <v>47</v>
       </c>
+      <c r="P144" t="n">
+        <v>23</v>
+      </c>
+      <c r="Q144" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -7548,6 +8416,12 @@
       <c r="O145" t="n">
         <v>77</v>
       </c>
+      <c r="P145" t="n">
+        <v>36</v>
+      </c>
+      <c r="Q145" t="n">
+        <v>113</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -7597,6 +8471,12 @@
       <c r="O146" t="n">
         <v>34</v>
       </c>
+      <c r="P146" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q146" t="n">
+        <v>44</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -7646,6 +8526,12 @@
       <c r="O147" t="n">
         <v>81</v>
       </c>
+      <c r="P147" t="n">
+        <v>41</v>
+      </c>
+      <c r="Q147" t="n">
+        <v>122</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -7695,6 +8581,12 @@
       <c r="O148" t="n">
         <v>1</v>
       </c>
+      <c r="P148" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q148" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -7744,6 +8636,12 @@
       <c r="O149" t="n">
         <v>47</v>
       </c>
+      <c r="P149" t="n">
+        <v>14</v>
+      </c>
+      <c r="Q149" t="n">
+        <v>61</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -7793,6 +8691,12 @@
       <c r="O150" t="n">
         <v>42</v>
       </c>
+      <c r="P150" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q150" t="n">
+        <v>54</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -7842,6 +8746,12 @@
       <c r="O151" t="n">
         <v>30</v>
       </c>
+      <c r="P151" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q151" t="n">
+        <v>49</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -7891,6 +8801,12 @@
       <c r="O152" t="n">
         <v>59</v>
       </c>
+      <c r="P152" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q152" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -7940,6 +8856,12 @@
       <c r="O153" t="n">
         <v>113</v>
       </c>
+      <c r="P153" t="n">
+        <v>54</v>
+      </c>
+      <c r="Q153" t="n">
+        <v>167</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -7989,6 +8911,12 @@
       <c r="O154" t="n">
         <v>44</v>
       </c>
+      <c r="P154" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q154" t="n">
+        <v>52</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -8038,6 +8966,12 @@
       <c r="O155" t="n">
         <v>52</v>
       </c>
+      <c r="P155" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q155" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -8087,6 +9021,12 @@
       <c r="O156" t="n">
         <v>55</v>
       </c>
+      <c r="P156" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q156" t="n">
+        <v>72</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -8136,6 +9076,12 @@
       <c r="O157" t="n">
         <v>42</v>
       </c>
+      <c r="P157" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q157" t="n">
+        <v>58</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -8185,6 +9131,12 @@
       <c r="O158" t="n">
         <v>37</v>
       </c>
+      <c r="P158" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q158" t="n">
+        <v>55</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -8234,6 +9186,12 @@
       <c r="O159" t="n">
         <v>27</v>
       </c>
+      <c r="P159" t="n">
+        <v>16</v>
+      </c>
+      <c r="Q159" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -8283,6 +9241,12 @@
       <c r="O160" t="n">
         <v>39</v>
       </c>
+      <c r="P160" t="n">
+        <v>23</v>
+      </c>
+      <c r="Q160" t="n">
+        <v>62</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -8332,6 +9296,12 @@
       <c r="O161" t="n">
         <v>34</v>
       </c>
+      <c r="P161" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q161" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -8381,6 +9351,12 @@
       <c r="O162" t="n">
         <v>32</v>
       </c>
+      <c r="P162" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q162" t="n">
+        <v>44</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -8430,6 +9406,12 @@
       <c r="O163" t="n">
         <v>137</v>
       </c>
+      <c r="P163" t="n">
+        <v>60</v>
+      </c>
+      <c r="Q163" t="n">
+        <v>197</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -8479,6 +9461,12 @@
       <c r="O164" t="n">
         <v>40</v>
       </c>
+      <c r="P164" t="n">
+        <v>21</v>
+      </c>
+      <c r="Q164" t="n">
+        <v>61</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -8528,6 +9516,12 @@
       <c r="O165" t="n">
         <v>119</v>
       </c>
+      <c r="P165" t="n">
+        <v>52</v>
+      </c>
+      <c r="Q165" t="n">
+        <v>171</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -8577,6 +9571,12 @@
       <c r="O166" t="n">
         <v>40</v>
       </c>
+      <c r="P166" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q166" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -8626,6 +9626,12 @@
       <c r="O167" t="n">
         <v>70</v>
       </c>
+      <c r="P167" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q167" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -8675,6 +9681,12 @@
       <c r="O168" t="n">
         <v>73</v>
       </c>
+      <c r="P168" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q168" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -8724,6 +9736,12 @@
       <c r="O169" t="n">
         <v>50</v>
       </c>
+      <c r="P169" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q169" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -8773,6 +9791,12 @@
       <c r="O170" t="n">
         <v>71</v>
       </c>
+      <c r="P170" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q170" t="n">
+        <v>75</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -8822,6 +9846,12 @@
       <c r="O171" t="n">
         <v>126</v>
       </c>
+      <c r="P171" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q171" t="n">
+        <v>126</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -8871,6 +9901,12 @@
       <c r="O172" t="n">
         <v>115</v>
       </c>
+      <c r="P172" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q172" t="n">
+        <v>115</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -8920,6 +9956,12 @@
       <c r="O173" t="n">
         <v>38</v>
       </c>
+      <c r="P173" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q173" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -8969,6 +10011,12 @@
       <c r="O174" t="n">
         <v>1</v>
       </c>
+      <c r="P174" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q174" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -9018,6 +10066,12 @@
       <c r="O175" t="n">
         <v>138</v>
       </c>
+      <c r="P175" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q175" t="n">
+        <v>138</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -9067,6 +10121,12 @@
       <c r="O176" t="n">
         <v>129</v>
       </c>
+      <c r="P176" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q176" t="n">
+        <v>129</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -9116,6 +10176,12 @@
       <c r="O177" t="n">
         <v>50</v>
       </c>
+      <c r="P177" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q177" t="n">
+        <v>53</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -9165,6 +10231,12 @@
       <c r="O178" t="n">
         <v>68</v>
       </c>
+      <c r="P178" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q178" t="n">
+        <v>68</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -9214,6 +10286,12 @@
       <c r="O179" t="n">
         <v>33</v>
       </c>
+      <c r="P179" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q179" t="n">
+        <v>33</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -9263,6 +10341,12 @@
       <c r="O180" t="n">
         <v>2</v>
       </c>
+      <c r="P180" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q180" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -9312,6 +10396,12 @@
       <c r="O181" t="n">
         <v>133</v>
       </c>
+      <c r="P181" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q181" t="n">
+        <v>133</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -9361,6 +10451,12 @@
       <c r="O182" t="n">
         <v>125</v>
       </c>
+      <c r="P182" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q182" t="n">
+        <v>128</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -9410,6 +10506,12 @@
       <c r="O183" t="n">
         <v>2</v>
       </c>
+      <c r="P183" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q183" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -9459,6 +10561,12 @@
       <c r="O184" t="n">
         <v>84</v>
       </c>
+      <c r="P184" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q184" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -9508,6 +10616,12 @@
       <c r="O185" t="n">
         <v>58</v>
       </c>
+      <c r="P185" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q185" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -9557,6 +10671,12 @@
       <c r="O186" t="n">
         <v>1</v>
       </c>
+      <c r="P186" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q186" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -9606,6 +10726,12 @@
       <c r="O187" t="n">
         <v>104</v>
       </c>
+      <c r="P187" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q187" t="n">
+        <v>104</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -9655,6 +10781,12 @@
       <c r="O188" t="n">
         <v>63</v>
       </c>
+      <c r="P188" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q188" t="n">
+        <v>63</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -9704,6 +10836,12 @@
       <c r="O189" t="n">
         <v>62</v>
       </c>
+      <c r="P189" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q189" t="n">
+        <v>62</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -9753,6 +10891,12 @@
       <c r="O190" t="n">
         <v>58</v>
       </c>
+      <c r="P190" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q190" t="n">
+        <v>58</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -9802,6 +10946,12 @@
       <c r="O191" t="n">
         <v>45</v>
       </c>
+      <c r="P191" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q191" t="n">
+        <v>45</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -9851,6 +11001,12 @@
       <c r="O192" t="n">
         <v>1</v>
       </c>
+      <c r="P192" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q192" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -9900,6 +11056,12 @@
       <c r="O193" t="n">
         <v>182</v>
       </c>
+      <c r="P193" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q193" t="n">
+        <v>182</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -9949,6 +11111,12 @@
       <c r="O194" t="n">
         <v>4</v>
       </c>
+      <c r="P194" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q194" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -9998,6 +11166,12 @@
       <c r="O195" t="n">
         <v>105</v>
       </c>
+      <c r="P195" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q195" t="n">
+        <v>105</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -10047,6 +11221,12 @@
       <c r="O196" t="n">
         <v>102</v>
       </c>
+      <c r="P196" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q196" t="n">
+        <v>103</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -10096,6 +11276,12 @@
       <c r="O197" t="n">
         <v>28</v>
       </c>
+      <c r="P197" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q197" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -10145,6 +11331,12 @@
       <c r="O198" t="n">
         <v>9</v>
       </c>
+      <c r="P198" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q198" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -10194,6 +11386,12 @@
       <c r="O199" t="n">
         <v>10</v>
       </c>
+      <c r="P199" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q199" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -10243,6 +11441,12 @@
       <c r="O200" t="n">
         <v>15</v>
       </c>
+      <c r="P200" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q200" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -10292,6 +11496,12 @@
       <c r="O201" t="n">
         <v>10</v>
       </c>
+      <c r="P201" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q201" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -10341,6 +11551,12 @@
       <c r="O202" t="n">
         <v>24</v>
       </c>
+      <c r="P202" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q202" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -10390,6 +11606,12 @@
       <c r="O203" t="n">
         <v>21</v>
       </c>
+      <c r="P203" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q203" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -10439,6 +11661,12 @@
       <c r="O204" t="n">
         <v>17</v>
       </c>
+      <c r="P204" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q204" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -10488,6 +11716,12 @@
       <c r="O205" t="n">
         <v>1</v>
       </c>
+      <c r="P205" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q205" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -10537,6 +11771,12 @@
       <c r="O206" t="n">
         <v>22</v>
       </c>
+      <c r="P206" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q206" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -10586,6 +11826,12 @@
       <c r="O207" t="n">
         <v>27</v>
       </c>
+      <c r="P207" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q207" t="n">
+        <v>27</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -10635,6 +11881,12 @@
       <c r="O208" t="n">
         <v>2</v>
       </c>
+      <c r="P208" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q208" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -10684,6 +11936,12 @@
       <c r="O209" t="n">
         <v>53</v>
       </c>
+      <c r="P209" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q209" t="n">
+        <v>53</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -10733,6 +11991,12 @@
       <c r="O210" t="n">
         <v>33</v>
       </c>
+      <c r="P210" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q210" t="n">
+        <v>33</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -10782,6 +12046,12 @@
       <c r="O211" t="n">
         <v>1</v>
       </c>
+      <c r="P211" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q211" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -10831,6 +12101,12 @@
       <c r="O212" t="n">
         <v>1</v>
       </c>
+      <c r="P212" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q212" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -10880,6 +12156,12 @@
       <c r="O213" t="n">
         <v>59</v>
       </c>
+      <c r="P213" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q213" t="n">
+        <v>59</v>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -10929,6 +12211,12 @@
       <c r="O214" t="n">
         <v>29</v>
       </c>
+      <c r="P214" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q214" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -10978,6 +12266,12 @@
       <c r="O215" t="n">
         <v>25</v>
       </c>
+      <c r="P215" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q215" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -11027,6 +12321,12 @@
       <c r="O216" t="n">
         <v>26</v>
       </c>
+      <c r="P216" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q216" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -11076,6 +12376,12 @@
       <c r="O217" t="n">
         <v>23</v>
       </c>
+      <c r="P217" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q217" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -11125,6 +12431,12 @@
       <c r="O218" t="n">
         <v>2</v>
       </c>
+      <c r="P218" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q218" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -11174,6 +12486,12 @@
       <c r="O219" t="n">
         <v>48</v>
       </c>
+      <c r="P219" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q219" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -11223,6 +12541,12 @@
       <c r="O220" t="n">
         <v>39</v>
       </c>
+      <c r="P220" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q220" t="n">
+        <v>41</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -11272,6 +12596,12 @@
       <c r="O221" t="n">
         <v>41</v>
       </c>
+      <c r="P221" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q221" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -11321,6 +12651,12 @@
       <c r="O222" t="n">
         <v>65</v>
       </c>
+      <c r="P222" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q222" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -11370,6 +12706,12 @@
       <c r="O223" t="n">
         <v>2</v>
       </c>
+      <c r="P223" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q223" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -11419,6 +12761,12 @@
       <c r="O224" t="n">
         <v>89</v>
       </c>
+      <c r="P224" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q224" t="n">
+        <v>89</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -11468,6 +12816,12 @@
       <c r="O225" t="n">
         <v>58</v>
       </c>
+      <c r="P225" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q225" t="n">
+        <v>61</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -11517,6 +12871,12 @@
       <c r="O226" t="n">
         <v>73</v>
       </c>
+      <c r="P226" t="n">
+        <v>23</v>
+      </c>
+      <c r="Q226" t="n">
+        <v>96</v>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -11566,6 +12926,12 @@
       <c r="O227" t="n">
         <v>199</v>
       </c>
+      <c r="P227" t="n">
+        <v>44</v>
+      </c>
+      <c r="Q227" t="n">
+        <v>243</v>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -11615,6 +12981,12 @@
       <c r="O228" t="n">
         <v>94</v>
       </c>
+      <c r="P228" t="n">
+        <v>41</v>
+      </c>
+      <c r="Q228" t="n">
+        <v>135</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -11664,6 +13036,12 @@
       <c r="O229" t="n">
         <v>139</v>
       </c>
+      <c r="P229" t="n">
+        <v>46</v>
+      </c>
+      <c r="Q229" t="n">
+        <v>185</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -11713,6 +13091,12 @@
       <c r="O230" t="n">
         <v>2</v>
       </c>
+      <c r="P230" t="n">
+        <v>48</v>
+      </c>
+      <c r="Q230" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -11762,6 +13146,12 @@
       <c r="O231" t="n">
         <v>168</v>
       </c>
+      <c r="P231" t="n">
+        <v>47</v>
+      </c>
+      <c r="Q231" t="n">
+        <v>215</v>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -11811,6 +13201,12 @@
       <c r="O232" t="n">
         <v>71</v>
       </c>
+      <c r="P232" t="n">
+        <v>38</v>
+      </c>
+      <c r="Q232" t="n">
+        <v>109</v>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -11860,6 +13256,12 @@
       <c r="O233" t="n">
         <v>77</v>
       </c>
+      <c r="P233" t="n">
+        <v>21</v>
+      </c>
+      <c r="Q233" t="n">
+        <v>98</v>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -11909,6 +13311,12 @@
       <c r="O234" t="n">
         <v>46</v>
       </c>
+      <c r="P234" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q234" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -11958,6 +13366,12 @@
       <c r="O235" t="n">
         <v>42</v>
       </c>
+      <c r="P235" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q235" t="n">
+        <v>61</v>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -12007,6 +13421,12 @@
       <c r="O236" t="n">
         <v>5</v>
       </c>
+      <c r="P236" t="n">
+        <v>42</v>
+      </c>
+      <c r="Q236" t="n">
+        <v>47</v>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -12056,6 +13476,12 @@
       <c r="O237" t="n">
         <v>204</v>
       </c>
+      <c r="P237" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q237" t="n">
+        <v>234</v>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -12105,6 +13531,12 @@
       <c r="O238" t="n">
         <v>50</v>
       </c>
+      <c r="P238" t="n">
+        <v>40</v>
+      </c>
+      <c r="Q238" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -12154,6 +13586,12 @@
       <c r="O239" t="n">
         <v>32</v>
       </c>
+      <c r="P239" t="n">
+        <v>29</v>
+      </c>
+      <c r="Q239" t="n">
+        <v>61</v>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -12203,6 +13641,12 @@
       <c r="O240" t="n">
         <v>61</v>
       </c>
+      <c r="P240" t="n">
+        <v>29</v>
+      </c>
+      <c r="Q240" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -12252,6 +13696,12 @@
       <c r="O241" t="n">
         <v>43</v>
       </c>
+      <c r="P241" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q241" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -12301,6 +13751,12 @@
       <c r="O242" t="n">
         <v>2</v>
       </c>
+      <c r="P242" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q242" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -12350,6 +13806,12 @@
       <c r="O243" t="n">
         <v>1</v>
       </c>
+      <c r="P243" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q243" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -12399,6 +13861,12 @@
       <c r="O244" t="n">
         <v>2</v>
       </c>
+      <c r="P244" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q244" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -12448,6 +13916,12 @@
       <c r="O245" t="n">
         <v>60</v>
       </c>
+      <c r="P245" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q245" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -12497,6 +13971,12 @@
       <c r="O246" t="n">
         <v>152</v>
       </c>
+      <c r="P246" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q246" t="n">
+        <v>171</v>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -12546,6 +14026,12 @@
       <c r="O247" t="n">
         <v>236</v>
       </c>
+      <c r="P247" t="n">
+        <v>32</v>
+      </c>
+      <c r="Q247" t="n">
+        <v>268</v>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -12595,6 +14081,12 @@
       <c r="O248" t="n">
         <v>72</v>
       </c>
+      <c r="P248" t="n">
+        <v>36</v>
+      </c>
+      <c r="Q248" t="n">
+        <v>108</v>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -12644,6 +14136,12 @@
       <c r="O249" t="n">
         <v>6</v>
       </c>
+      <c r="P249" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q249" t="n">
+        <v>36</v>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -12693,6 +14191,12 @@
       <c r="O250" t="n">
         <v>6</v>
       </c>
+      <c r="P250" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q250" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -12742,6 +14246,12 @@
       <c r="O251" t="n">
         <v>296</v>
       </c>
+      <c r="P251" t="n">
+        <v>23</v>
+      </c>
+      <c r="Q251" t="n">
+        <v>319</v>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -12791,6 +14301,12 @@
       <c r="O252" t="n">
         <v>1172</v>
       </c>
+      <c r="P252" t="n">
+        <v>25</v>
+      </c>
+      <c r="Q252" t="n">
+        <v>1197</v>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -12840,6 +14356,12 @@
       <c r="O253" t="n">
         <v>161</v>
       </c>
+      <c r="P253" t="n">
+        <v>38</v>
+      </c>
+      <c r="Q253" t="n">
+        <v>199</v>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -12889,6 +14411,12 @@
       <c r="O254" t="n">
         <v>173</v>
       </c>
+      <c r="P254" t="n">
+        <v>33</v>
+      </c>
+      <c r="Q254" t="n">
+        <v>206</v>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -12938,6 +14466,12 @@
       <c r="O255" t="n">
         <v>192</v>
       </c>
+      <c r="P255" t="n">
+        <v>49</v>
+      </c>
+      <c r="Q255" t="n">
+        <v>241</v>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -12987,6 +14521,12 @@
       <c r="O256" t="n">
         <v>269</v>
       </c>
+      <c r="P256" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q256" t="n">
+        <v>269</v>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -13036,6 +14576,12 @@
       <c r="O257" t="n">
         <v>61</v>
       </c>
+      <c r="P257" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q257" t="n">
+        <v>61</v>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -13085,6 +14631,12 @@
       <c r="O258" t="n">
         <v>135</v>
       </c>
+      <c r="P258" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q258" t="n">
+        <v>145</v>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -13134,6 +14686,12 @@
       <c r="O259" t="n">
         <v>67</v>
       </c>
+      <c r="P259" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q259" t="n">
+        <v>67</v>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -13183,6 +14741,12 @@
       <c r="O260" t="n">
         <v>12</v>
       </c>
+      <c r="P260" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q260" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -13232,6 +14796,12 @@
       <c r="O261" t="n">
         <v>64</v>
       </c>
+      <c r="P261" t="n">
+        <v>37</v>
+      </c>
+      <c r="Q261" t="n">
+        <v>101</v>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -13281,6 +14851,12 @@
       <c r="O262" t="n">
         <v>49</v>
       </c>
+      <c r="P262" t="n">
+        <v>43</v>
+      </c>
+      <c r="Q262" t="n">
+        <v>92</v>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -13330,6 +14906,12 @@
       <c r="O263" t="n">
         <v>26</v>
       </c>
+      <c r="P263" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q263" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -13379,6 +14961,12 @@
       <c r="O264" t="n">
         <v>30</v>
       </c>
+      <c r="P264" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q264" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -13428,6 +15016,12 @@
       <c r="O265" t="n">
         <v>233</v>
       </c>
+      <c r="P265" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q265" t="n">
+        <v>233</v>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -13477,6 +15071,12 @@
       <c r="O266" t="n">
         <v>274</v>
       </c>
+      <c r="P266" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q266" t="n">
+        <v>274</v>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -13526,6 +15126,12 @@
       <c r="O267" t="n">
         <v>85</v>
       </c>
+      <c r="P267" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q267" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -13575,6 +15181,12 @@
       <c r="O268" t="n">
         <v>103</v>
       </c>
+      <c r="P268" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q268" t="n">
+        <v>103</v>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -13624,6 +15236,12 @@
       <c r="O269" t="n">
         <v>93</v>
       </c>
+      <c r="P269" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q269" t="n">
+        <v>93</v>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -13673,6 +15291,12 @@
       <c r="O270" t="n">
         <v>5</v>
       </c>
+      <c r="P270" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q270" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -13722,6 +15346,12 @@
       <c r="O271" t="n">
         <v>146</v>
       </c>
+      <c r="P271" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q271" t="n">
+        <v>146</v>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -13771,6 +15401,12 @@
       <c r="O272" t="n">
         <v>155</v>
       </c>
+      <c r="P272" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q272" t="n">
+        <v>155</v>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -13820,6 +15456,12 @@
       <c r="O273" t="n">
         <v>104</v>
       </c>
+      <c r="P273" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q273" t="n">
+        <v>104</v>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -13869,6 +15511,12 @@
       <c r="O274" t="n">
         <v>104</v>
       </c>
+      <c r="P274" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q274" t="n">
+        <v>104</v>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -13918,6 +15566,12 @@
       <c r="O275" t="n">
         <v>101</v>
       </c>
+      <c r="P275" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q275" t="n">
+        <v>101</v>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -13967,6 +15621,12 @@
       <c r="O276" t="n">
         <v>122</v>
       </c>
+      <c r="P276" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q276" t="n">
+        <v>122</v>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -14016,6 +15676,12 @@
       <c r="O277" t="n">
         <v>298</v>
       </c>
+      <c r="P277" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q277" t="n">
+        <v>298</v>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -14065,6 +15731,12 @@
       <c r="O278" t="n">
         <v>30</v>
       </c>
+      <c r="P278" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q278" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -14114,6 +15786,12 @@
       <c r="O279" t="n">
         <v>38</v>
       </c>
+      <c r="P279" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q279" t="n">
+        <v>38</v>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -14163,6 +15841,12 @@
       <c r="O280" t="n">
         <v>110</v>
       </c>
+      <c r="P280" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q280" t="n">
+        <v>110</v>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -14212,6 +15896,12 @@
       <c r="O281" t="n">
         <v>313</v>
       </c>
+      <c r="P281" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q281" t="n">
+        <v>313</v>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -14261,6 +15951,12 @@
       <c r="O282" t="n">
         <v>129</v>
       </c>
+      <c r="P282" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q282" t="n">
+        <v>129</v>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -14310,6 +16006,12 @@
       <c r="O283" t="n">
         <v>26</v>
       </c>
+      <c r="P283" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q283" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -14359,6 +16061,12 @@
       <c r="O284" t="n">
         <v>25</v>
       </c>
+      <c r="P284" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q284" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -14408,6 +16116,12 @@
       <c r="O285" t="n">
         <v>14</v>
       </c>
+      <c r="P285" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q285" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -14457,6 +16171,12 @@
       <c r="O286" t="n">
         <v>147</v>
       </c>
+      <c r="P286" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q286" t="n">
+        <v>147</v>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -14506,6 +16226,12 @@
       <c r="O287" t="n">
         <v>130</v>
       </c>
+      <c r="P287" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q287" t="n">
+        <v>130</v>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -14555,6 +16281,12 @@
       <c r="O288" t="n">
         <v>52</v>
       </c>
+      <c r="P288" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q288" t="n">
+        <v>52</v>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -14604,6 +16336,12 @@
       <c r="O289" t="n">
         <v>21</v>
       </c>
+      <c r="P289" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q289" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -14653,6 +16391,12 @@
       <c r="O290" t="n">
         <v>46</v>
       </c>
+      <c r="P290" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q290" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -14702,6 +16446,12 @@
       <c r="O291" t="n">
         <v>19</v>
       </c>
+      <c r="P291" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q291" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -14751,6 +16501,12 @@
       <c r="O292" t="n">
         <v>26</v>
       </c>
+      <c r="P292" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q292" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -14800,6 +16556,12 @@
       <c r="O293" t="n">
         <v>28</v>
       </c>
+      <c r="P293" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q293" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -14849,6 +16611,12 @@
       <c r="O294" t="n">
         <v>227</v>
       </c>
+      <c r="P294" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q294" t="n">
+        <v>227</v>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -14893,10 +16661,16 @@
         <v>46</v>
       </c>
       <c r="N295" t="n">
+        <v>48</v>
+      </c>
+      <c r="O295" t="n">
         <v>49</v>
       </c>
-      <c r="O295" t="n">
-        <v>50</v>
+      <c r="P295" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q295" t="n">
+        <v>49</v>
       </c>
     </row>
     <row r="296">
@@ -14947,6 +16721,12 @@
       <c r="O296" t="n">
         <v>74</v>
       </c>
+      <c r="P296" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q296" t="n">
+        <v>74</v>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -14996,6 +16776,12 @@
       <c r="O297" t="n">
         <v>105</v>
       </c>
+      <c r="P297" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q297" t="n">
+        <v>108</v>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -15034,16 +16820,22 @@
         <v>0</v>
       </c>
       <c r="L298" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="M298" t="n">
+        <v>13</v>
+      </c>
+      <c r="N298" t="n">
         <v>14</v>
       </c>
-      <c r="N298" t="n">
-        <v>15</v>
-      </c>
       <c r="O298" t="n">
-        <v>15</v>
+        <v>14</v>
+      </c>
+      <c r="P298" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q298" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="299">
@@ -15094,6 +16886,12 @@
       <c r="O299" t="n">
         <v>15</v>
       </c>
+      <c r="P299" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q299" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -15143,6 +16941,12 @@
       <c r="O300" t="n">
         <v>100</v>
       </c>
+      <c r="P300" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q300" t="n">
+        <v>105</v>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -15192,6 +16996,12 @@
       <c r="O301" t="n">
         <v>126</v>
       </c>
+      <c r="P301" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q301" t="n">
+        <v>136</v>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -15241,6 +17051,12 @@
       <c r="O302" t="n">
         <v>37</v>
       </c>
+      <c r="P302" t="n">
+        <v>8</v>
+      </c>
+      <c r="Q302" t="n">
+        <v>45</v>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -15290,6 +17106,12 @@
       <c r="O303" t="n">
         <v>283</v>
       </c>
+      <c r="P303" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q303" t="n">
+        <v>290</v>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -15339,6 +17161,12 @@
       <c r="O304" t="n">
         <v>394</v>
       </c>
+      <c r="P304" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q304" t="n">
+        <v>399</v>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -15388,6 +17216,12 @@
       <c r="O305" t="n">
         <v>373</v>
       </c>
+      <c r="P305" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q305" t="n">
+        <v>384</v>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -15437,6 +17271,12 @@
       <c r="O306" t="n">
         <v>204</v>
       </c>
+      <c r="P306" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q306" t="n">
+        <v>217</v>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -15448,43 +17288,49 @@
         <v>0</v>
       </c>
       <c r="C307" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D307" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E307" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F307" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G307" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="H307" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I307" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J307" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K307" t="n">
         <v>0</v>
       </c>
       <c r="L307" t="n">
+        <v>24</v>
+      </c>
+      <c r="M307" t="n">
+        <v>59</v>
+      </c>
+      <c r="N307" t="n">
+        <v>78</v>
+      </c>
+      <c r="O307" t="n">
+        <v>95</v>
+      </c>
+      <c r="P307" t="n">
         <v>5</v>
       </c>
-      <c r="M307" t="n">
-        <v>11</v>
-      </c>
-      <c r="N307" t="n">
-        <v>17</v>
-      </c>
-      <c r="O307" t="n">
-        <v>20</v>
+      <c r="Q307" t="n">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily auto-refresh 2026-08-18 13:09
</commit_message>
<xml_diff>
--- a/daily_slab_mix.xlsx
+++ b/daily_slab_mix.xlsx
@@ -17080,7 +17080,7 @@
         <v>28</v>
       </c>
       <c r="G303" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H303" t="n">
         <v>11</v>
@@ -17095,7 +17095,7 @@
         <v>1</v>
       </c>
       <c r="L303" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M303" t="n">
         <v>149</v>

</xml_diff>

<commit_message>
daily auto-refresh 2026-08-18 14:15
</commit_message>
<xml_diff>
--- a/daily_slab_mix.xlsx
+++ b/daily_slab_mix.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q307"/>
+  <dimension ref="A1:Q308"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17333,6 +17333,61 @@
         <v>100</v>
       </c>
     </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="B308" t="n">
+        <v>1</v>
+      </c>
+      <c r="C308" t="n">
+        <v>0</v>
+      </c>
+      <c r="D308" t="n">
+        <v>1</v>
+      </c>
+      <c r="E308" t="n">
+        <v>0</v>
+      </c>
+      <c r="F308" t="n">
+        <v>2</v>
+      </c>
+      <c r="G308" t="n">
+        <v>2</v>
+      </c>
+      <c r="H308" t="n">
+        <v>2</v>
+      </c>
+      <c r="I308" t="n">
+        <v>1</v>
+      </c>
+      <c r="J308" t="n">
+        <v>0</v>
+      </c>
+      <c r="K308" t="n">
+        <v>0</v>
+      </c>
+      <c r="L308" t="n">
+        <v>6</v>
+      </c>
+      <c r="M308" t="n">
+        <v>15</v>
+      </c>
+      <c r="N308" t="n">
+        <v>16</v>
+      </c>
+      <c r="O308" t="n">
+        <v>18</v>
+      </c>
+      <c r="P308" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q308" t="n">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
daily auto-refresh 2026-08-25 14:13
</commit_message>
<xml_diff>
--- a/daily_slab_mix.xlsx
+++ b/daily_slab_mix.xlsx
@@ -1610,7 +1610,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C22" t="n">
         <v>4</v>
@@ -1640,7 +1640,7 @@
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M22" t="n">
         <v>29</v>
@@ -1720,7 +1720,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C24" t="n">
         <v>0</v>
@@ -1750,7 +1750,7 @@
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M24" t="n">
         <v>20</v>
@@ -5570,7 +5570,7 @@
         </is>
       </c>
       <c r="B94" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C94" t="n">
         <v>2</v>
@@ -5600,7 +5600,7 @@
         <v>0</v>
       </c>
       <c r="L94" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M94" t="n">
         <v>44</v>
@@ -10630,7 +10630,7 @@
         </is>
       </c>
       <c r="B186" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C186" t="n">
         <v>0</v>
@@ -10660,7 +10660,7 @@
         <v>0</v>
       </c>
       <c r="L186" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M186" t="n">
         <v>1</v>
@@ -12335,7 +12335,7 @@
         </is>
       </c>
       <c r="B217" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C217" t="n">
         <v>3</v>
@@ -12365,7 +12365,7 @@
         <v>0</v>
       </c>
       <c r="L217" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M217" t="n">
         <v>23</v>
@@ -12460,7 +12460,7 @@
         <v>3</v>
       </c>
       <c r="G219" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H219" t="n">
         <v>5</v>
@@ -12475,7 +12475,7 @@
         <v>1</v>
       </c>
       <c r="L219" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M219" t="n">
         <v>47</v>
@@ -12885,22 +12885,22 @@
         </is>
       </c>
       <c r="B227" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C227" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D227" t="n">
         <v>9</v>
       </c>
       <c r="E227" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F227" t="n">
         <v>29</v>
       </c>
       <c r="G227" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H227" t="n">
         <v>14</v>
@@ -12915,7 +12915,7 @@
         <v>0</v>
       </c>
       <c r="L227" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M227" t="n">
         <v>187</v>
@@ -12952,7 +12952,7 @@
         <v>16</v>
       </c>
       <c r="F228" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G228" t="n">
         <v>32</v>
@@ -12970,7 +12970,7 @@
         <v>0</v>
       </c>
       <c r="L228" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M228" t="n">
         <v>88</v>
@@ -12995,7 +12995,7 @@
         </is>
       </c>
       <c r="B229" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C229" t="n">
         <v>10</v>
@@ -13025,7 +13025,7 @@
         <v>0</v>
       </c>
       <c r="L229" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M229" t="n">
         <v>122</v>
@@ -13340,7 +13340,7 @@
         <v>5</v>
       </c>
       <c r="G235" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H235" t="n">
         <v>2</v>
@@ -13355,7 +13355,7 @@
         <v>1</v>
       </c>
       <c r="L235" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M235" t="n">
         <v>39</v>
@@ -13441,10 +13441,10 @@
         <v>4</v>
       </c>
       <c r="D237" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E237" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F237" t="n">
         <v>22</v>
@@ -13465,7 +13465,7 @@
         <v>2</v>
       </c>
       <c r="L237" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="M237" t="n">
         <v>176</v>
@@ -13496,7 +13496,7 @@
         <v>1</v>
       </c>
       <c r="D238" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E238" t="n">
         <v>5</v>
@@ -13520,7 +13520,7 @@
         <v>0</v>
       </c>
       <c r="L238" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M238" t="n">
         <v>44</v>
@@ -13655,7 +13655,7 @@
         </is>
       </c>
       <c r="B241" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C241" t="n">
         <v>0</v>
@@ -13670,7 +13670,7 @@
         <v>3</v>
       </c>
       <c r="G241" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H241" t="n">
         <v>7</v>
@@ -13685,7 +13685,7 @@
         <v>1</v>
       </c>
       <c r="L241" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M241" t="n">
         <v>39</v>
@@ -13710,7 +13710,7 @@
         </is>
       </c>
       <c r="B242" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C242" t="n">
         <v>0</v>
@@ -13740,7 +13740,7 @@
         <v>0</v>
       </c>
       <c r="L242" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M242" t="n">
         <v>2</v>
@@ -14040,7 +14040,7 @@
         </is>
       </c>
       <c r="B248" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C248" t="n">
         <v>0</v>
@@ -14070,7 +14070,7 @@
         <v>0</v>
       </c>
       <c r="L248" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M248" t="n">
         <v>67</v>
@@ -14214,7 +14214,7 @@
         <v>28</v>
       </c>
       <c r="E251" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F251" t="n">
         <v>29</v>
@@ -14235,7 +14235,7 @@
         <v>3</v>
       </c>
       <c r="L251" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="M251" t="n">
         <v>292</v>
@@ -14425,7 +14425,7 @@
         </is>
       </c>
       <c r="B255" t="n">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C255" t="n">
         <v>13</v>
@@ -14455,7 +14455,7 @@
         <v>1</v>
       </c>
       <c r="L255" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M255" t="n">
         <v>190</v>
@@ -14590,7 +14590,7 @@
         </is>
       </c>
       <c r="B258" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C258" t="n">
         <v>6</v>
@@ -14620,7 +14620,7 @@
         <v>1</v>
       </c>
       <c r="L258" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M258" t="n">
         <v>132</v>
@@ -14755,7 +14755,7 @@
         </is>
       </c>
       <c r="B261" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C261" t="n">
         <v>0</v>
@@ -14764,7 +14764,7 @@
         <v>2</v>
       </c>
       <c r="E261" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F261" t="n">
         <v>24</v>
@@ -14785,7 +14785,7 @@
         <v>0</v>
       </c>
       <c r="L261" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M261" t="n">
         <v>64</v>
@@ -14816,16 +14816,16 @@
         <v>1</v>
       </c>
       <c r="D262" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E262" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F262" t="n">
         <v>14</v>
       </c>
       <c r="G262" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H262" t="n">
         <v>1</v>
@@ -14840,7 +14840,7 @@
         <v>0</v>
       </c>
       <c r="L262" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M262" t="n">
         <v>49</v>
@@ -14865,7 +14865,7 @@
         </is>
       </c>
       <c r="B263" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C263" t="n">
         <v>0</v>
@@ -14895,7 +14895,7 @@
         <v>0</v>
       </c>
       <c r="L263" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="M263" t="n">
         <v>26</v>
@@ -14920,7 +14920,7 @@
         </is>
       </c>
       <c r="B264" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C264" t="n">
         <v>0</v>
@@ -14950,7 +14950,7 @@
         <v>0</v>
       </c>
       <c r="L264" t="n">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="M264" t="n">
         <v>29</v>
@@ -14975,13 +14975,13 @@
         </is>
       </c>
       <c r="B265" t="n">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="C265" t="n">
         <v>7</v>
       </c>
       <c r="D265" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E265" t="n">
         <v>14</v>
@@ -15005,7 +15005,7 @@
         <v>0</v>
       </c>
       <c r="L265" t="n">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="M265" t="n">
         <v>228</v>
@@ -15030,10 +15030,10 @@
         </is>
       </c>
       <c r="B266" t="n">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C266" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D266" t="n">
         <v>13</v>
@@ -15042,13 +15042,13 @@
         <v>29</v>
       </c>
       <c r="F266" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G266" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H266" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I266" t="n">
         <v>2</v>
@@ -15060,7 +15060,7 @@
         <v>1</v>
       </c>
       <c r="L266" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="M266" t="n">
         <v>270</v>
@@ -15085,7 +15085,7 @@
         </is>
       </c>
       <c r="B267" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C267" t="n">
         <v>5</v>
@@ -15094,10 +15094,10 @@
         <v>10</v>
       </c>
       <c r="E267" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F267" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G267" t="n">
         <v>7</v>
@@ -15115,7 +15115,7 @@
         <v>0</v>
       </c>
       <c r="L267" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="M267" t="n">
         <v>85</v>
@@ -15140,7 +15140,7 @@
         </is>
       </c>
       <c r="B268" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C268" t="n">
         <v>9</v>
@@ -15170,7 +15170,7 @@
         <v>0</v>
       </c>
       <c r="L268" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="M268" t="n">
         <v>100</v>
@@ -15195,19 +15195,19 @@
         </is>
       </c>
       <c r="B269" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C269" t="n">
         <v>2</v>
       </c>
       <c r="D269" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E269" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F269" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G269" t="n">
         <v>14</v>
@@ -15225,7 +15225,7 @@
         <v>0</v>
       </c>
       <c r="L269" t="n">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="M269" t="n">
         <v>93</v>
@@ -15305,7 +15305,7 @@
         </is>
       </c>
       <c r="B271" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C271" t="n">
         <v>2</v>
@@ -15335,7 +15335,7 @@
         <v>0</v>
       </c>
       <c r="L271" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="M271" t="n">
         <v>141</v>
@@ -15360,22 +15360,22 @@
         </is>
       </c>
       <c r="B272" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C272" t="n">
         <v>12</v>
       </c>
       <c r="D272" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E272" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F272" t="n">
         <v>18</v>
       </c>
       <c r="G272" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H272" t="n">
         <v>1</v>
@@ -15390,7 +15390,7 @@
         <v>2</v>
       </c>
       <c r="L272" t="n">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="M272" t="n">
         <v>155</v>
@@ -15415,7 +15415,7 @@
         </is>
       </c>
       <c r="B273" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C273" t="n">
         <v>3</v>
@@ -15430,7 +15430,7 @@
         <v>7</v>
       </c>
       <c r="G273" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H273" t="n">
         <v>5</v>
@@ -15445,7 +15445,7 @@
         <v>0</v>
       </c>
       <c r="L273" t="n">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="M273" t="n">
         <v>97</v>
@@ -15470,7 +15470,7 @@
         </is>
       </c>
       <c r="B274" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C274" t="n">
         <v>4</v>
@@ -15482,16 +15482,16 @@
         <v>8</v>
       </c>
       <c r="F274" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G274" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H274" t="n">
         <v>2</v>
       </c>
       <c r="I274" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J274" t="n">
         <v>0</v>
@@ -15500,7 +15500,7 @@
         <v>0</v>
       </c>
       <c r="L274" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="M274" t="n">
         <v>102</v>
@@ -15525,7 +15525,7 @@
         </is>
       </c>
       <c r="B275" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C275" t="n">
         <v>0</v>
@@ -15540,7 +15540,7 @@
         <v>11</v>
       </c>
       <c r="G275" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H275" t="n">
         <v>3</v>
@@ -15555,7 +15555,7 @@
         <v>2</v>
       </c>
       <c r="L275" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="M275" t="n">
         <v>94</v>
@@ -15580,7 +15580,7 @@
         </is>
       </c>
       <c r="B276" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C276" t="n">
         <v>3</v>
@@ -15595,7 +15595,7 @@
         <v>17</v>
       </c>
       <c r="G276" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H276" t="n">
         <v>1</v>
@@ -15610,7 +15610,7 @@
         <v>0</v>
       </c>
       <c r="L276" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="M276" t="n">
         <v>117</v>
@@ -15635,10 +15635,10 @@
         </is>
       </c>
       <c r="B277" t="n">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="C277" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D277" t="n">
         <v>29</v>
@@ -15647,7 +15647,7 @@
         <v>22</v>
       </c>
       <c r="F277" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G277" t="n">
         <v>13</v>
@@ -15665,7 +15665,7 @@
         <v>1</v>
       </c>
       <c r="L277" t="n">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="M277" t="n">
         <v>292</v>
@@ -15690,7 +15690,7 @@
         </is>
       </c>
       <c r="B278" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C278" t="n">
         <v>0</v>
@@ -15720,7 +15720,7 @@
         <v>1</v>
       </c>
       <c r="L278" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="M278" t="n">
         <v>25</v>
@@ -15745,7 +15745,7 @@
         </is>
       </c>
       <c r="B279" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C279" t="n">
         <v>0</v>
@@ -15775,7 +15775,7 @@
         <v>1</v>
       </c>
       <c r="L279" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="M279" t="n">
         <v>35</v>
@@ -15800,7 +15800,7 @@
         </is>
       </c>
       <c r="B280" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C280" t="n">
         <v>1</v>
@@ -15812,10 +15812,10 @@
         <v>11</v>
       </c>
       <c r="F280" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G280" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H280" t="n">
         <v>5</v>
@@ -15830,7 +15830,7 @@
         <v>1</v>
       </c>
       <c r="L280" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="M280" t="n">
         <v>100</v>
@@ -15855,13 +15855,13 @@
         </is>
       </c>
       <c r="B281" t="n">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="C281" t="n">
         <v>10</v>
       </c>
       <c r="D281" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E281" t="n">
         <v>21</v>
@@ -15873,7 +15873,7 @@
         <v>10</v>
       </c>
       <c r="H281" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I281" t="n">
         <v>1</v>
@@ -15885,7 +15885,7 @@
         <v>1</v>
       </c>
       <c r="L281" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="M281" t="n">
         <v>304</v>
@@ -15910,7 +15910,7 @@
         </is>
       </c>
       <c r="B282" t="n">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C282" t="n">
         <v>4</v>
@@ -15919,7 +15919,7 @@
         <v>9</v>
       </c>
       <c r="E282" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F282" t="n">
         <v>13</v>
@@ -15940,7 +15940,7 @@
         <v>1</v>
       </c>
       <c r="L282" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="M282" t="n">
         <v>122</v>
@@ -15965,7 +15965,7 @@
         </is>
       </c>
       <c r="B283" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C283" t="n">
         <v>0</v>
@@ -15995,7 +15995,7 @@
         <v>0</v>
       </c>
       <c r="L283" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="M283" t="n">
         <v>22</v>
@@ -16130,13 +16130,13 @@
         </is>
       </c>
       <c r="B286" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C286" t="n">
         <v>0</v>
       </c>
       <c r="D286" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E286" t="n">
         <v>36</v>
@@ -16145,10 +16145,10 @@
         <v>23</v>
       </c>
       <c r="G286" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H286" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I286" t="n">
         <v>2</v>
@@ -16160,7 +16160,7 @@
         <v>0</v>
       </c>
       <c r="L286" t="n">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="M286" t="n">
         <v>136</v>
@@ -16185,19 +16185,19 @@
         </is>
       </c>
       <c r="B287" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C287" t="n">
         <v>0</v>
       </c>
       <c r="D287" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E287" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F287" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="G287" t="n">
         <v>23</v>
@@ -16215,7 +16215,7 @@
         <v>0</v>
       </c>
       <c r="L287" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="M287" t="n">
         <v>122</v>
@@ -16240,7 +16240,7 @@
         </is>
       </c>
       <c r="B288" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C288" t="n">
         <v>1</v>
@@ -16255,7 +16255,7 @@
         <v>1</v>
       </c>
       <c r="G288" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H288" t="n">
         <v>4</v>
@@ -16270,7 +16270,7 @@
         <v>1</v>
       </c>
       <c r="L288" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="M288" t="n">
         <v>46</v>
@@ -16295,7 +16295,7 @@
         </is>
       </c>
       <c r="B289" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C289" t="n">
         <v>0</v>
@@ -16325,7 +16325,7 @@
         <v>0</v>
       </c>
       <c r="L289" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="M289" t="n">
         <v>20</v>
@@ -16405,7 +16405,7 @@
         </is>
       </c>
       <c r="B291" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C291" t="n">
         <v>0</v>
@@ -16435,7 +16435,7 @@
         <v>0</v>
       </c>
       <c r="L291" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="M291" t="n">
         <v>19</v>
@@ -16460,13 +16460,13 @@
         </is>
       </c>
       <c r="B292" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C292" t="n">
         <v>0</v>
       </c>
       <c r="D292" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E292" t="n">
         <v>0</v>
@@ -16490,7 +16490,7 @@
         <v>0</v>
       </c>
       <c r="L292" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="M292" t="n">
         <v>26</v>
@@ -16515,7 +16515,7 @@
         </is>
       </c>
       <c r="B293" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C293" t="n">
         <v>0</v>
@@ -16530,7 +16530,7 @@
         <v>0</v>
       </c>
       <c r="G293" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H293" t="n">
         <v>0</v>
@@ -16545,7 +16545,7 @@
         <v>0</v>
       </c>
       <c r="L293" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="M293" t="n">
         <v>25</v>
@@ -16579,13 +16579,13 @@
         <v>0</v>
       </c>
       <c r="E294" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F294" t="n">
         <v>13</v>
       </c>
       <c r="G294" t="n">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="H294" t="n">
         <v>14</v>
@@ -16600,7 +16600,7 @@
         <v>5</v>
       </c>
       <c r="L294" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="M294" t="n">
         <v>158</v>
@@ -16625,7 +16625,7 @@
         </is>
       </c>
       <c r="B295" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C295" t="n">
         <v>0</v>
@@ -16634,19 +16634,19 @@
         <v>0</v>
       </c>
       <c r="E295" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F295" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G295" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H295" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I295" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J295" t="n">
         <v>1</v>
@@ -16655,7 +16655,7 @@
         <v>0</v>
       </c>
       <c r="L295" t="n">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="M295" t="n">
         <v>46</v>
@@ -16692,16 +16692,16 @@
         <v>0</v>
       </c>
       <c r="F296" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G296" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="H296" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I296" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J296" t="n">
         <v>3</v>
@@ -16710,7 +16710,7 @@
         <v>0</v>
       </c>
       <c r="L296" t="n">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="M296" t="n">
         <v>72</v>
@@ -16735,28 +16735,28 @@
         </is>
       </c>
       <c r="B297" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C297" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D297" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E297" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F297" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="G297" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="H297" t="n">
         <v>5</v>
       </c>
       <c r="I297" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J297" t="n">
         <v>0</v>
@@ -16765,7 +16765,7 @@
         <v>2</v>
       </c>
       <c r="L297" t="n">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="M297" t="n">
         <v>78</v>
@@ -16790,7 +16790,7 @@
         </is>
       </c>
       <c r="B298" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C298" t="n">
         <v>0</v>
@@ -16802,10 +16802,10 @@
         <v>2</v>
       </c>
       <c r="F298" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G298" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H298" t="n">
         <v>0</v>
@@ -16820,7 +16820,7 @@
         <v>0</v>
       </c>
       <c r="L298" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="M298" t="n">
         <v>13</v>
@@ -16845,16 +16845,16 @@
         </is>
       </c>
       <c r="B299" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C299" t="n">
         <v>0</v>
       </c>
       <c r="D299" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E299" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F299" t="n">
         <v>0</v>
@@ -16875,7 +16875,7 @@
         <v>1</v>
       </c>
       <c r="L299" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="M299" t="n">
         <v>15</v>
@@ -16900,7 +16900,7 @@
         </is>
       </c>
       <c r="B300" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C300" t="n">
         <v>0</v>
@@ -16915,7 +16915,7 @@
         <v>11</v>
       </c>
       <c r="G300" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H300" t="n">
         <v>12</v>
@@ -16930,7 +16930,7 @@
         <v>2</v>
       </c>
       <c r="L300" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="M300" t="n">
         <v>78</v>
@@ -16964,13 +16964,13 @@
         <v>1</v>
       </c>
       <c r="E301" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F301" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G301" t="n">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="H301" t="n">
         <v>4</v>
@@ -16985,7 +16985,7 @@
         <v>0</v>
       </c>
       <c r="L301" t="n">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="M301" t="n">
         <v>109</v>
@@ -17019,16 +17019,16 @@
         <v>0</v>
       </c>
       <c r="E302" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F302" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G302" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H302" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I302" t="n">
         <v>1</v>
@@ -17040,7 +17040,7 @@
         <v>1</v>
       </c>
       <c r="L302" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="M302" t="n">
         <v>36</v>
@@ -17074,10 +17074,10 @@
         <v>12</v>
       </c>
       <c r="E303" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F303" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G303" t="n">
         <v>56</v>
@@ -17086,7 +17086,7 @@
         <v>11</v>
       </c>
       <c r="I303" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J303" t="n">
         <v>1</v>
@@ -17095,7 +17095,7 @@
         <v>1</v>
       </c>
       <c r="L303" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="M303" t="n">
         <v>149</v>
@@ -17120,25 +17120,25 @@
         </is>
       </c>
       <c r="B304" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C304" t="n">
         <v>3</v>
       </c>
       <c r="D304" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E304" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F304" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G304" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="H304" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="I304" t="n">
         <v>12</v>
@@ -17150,7 +17150,7 @@
         <v>1</v>
       </c>
       <c r="L304" t="n">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="M304" t="n">
         <v>232</v>
@@ -17184,7 +17184,7 @@
         <v>15</v>
       </c>
       <c r="E305" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F305" t="n">
         <v>44</v>
@@ -17193,10 +17193,10 @@
         <v>77</v>
       </c>
       <c r="H305" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I305" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J305" t="n">
         <v>2</v>
@@ -17205,7 +17205,7 @@
         <v>0</v>
       </c>
       <c r="L305" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="M305" t="n">
         <v>210</v>
@@ -17245,7 +17245,7 @@
         <v>19</v>
       </c>
       <c r="G306" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H306" t="n">
         <v>3</v>
@@ -17260,7 +17260,7 @@
         <v>0</v>
       </c>
       <c r="L306" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M306" t="n">
         <v>127</v>
@@ -17285,22 +17285,22 @@
         </is>
       </c>
       <c r="B307" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C307" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D307" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E307" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F307" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G307" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H307" t="n">
         <v>5</v>
@@ -17315,7 +17315,7 @@
         <v>0</v>
       </c>
       <c r="L307" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="M307" t="n">
         <v>59</v>
@@ -17340,7 +17340,7 @@
         </is>
       </c>
       <c r="B308" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C308" t="n">
         <v>2</v>
@@ -17352,13 +17352,13 @@
         <v>11</v>
       </c>
       <c r="F308" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G308" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="H308" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I308" t="n">
         <v>7</v>
@@ -17370,7 +17370,7 @@
         <v>0</v>
       </c>
       <c r="L308" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="M308" t="n">
         <v>82</v>
@@ -17395,13 +17395,13 @@
         </is>
       </c>
       <c r="B309" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C309" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D309" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E309" t="n">
         <v>6</v>
@@ -17410,7 +17410,7 @@
         <v>9</v>
       </c>
       <c r="G309" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="H309" t="n">
         <v>6</v>
@@ -17425,7 +17425,7 @@
         <v>0</v>
       </c>
       <c r="L309" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="M309" t="n">
         <v>91</v>
@@ -17670,7 +17670,7 @@
         </is>
       </c>
       <c r="B314" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C314" t="n">
         <v>0</v>
@@ -17679,7 +17679,7 @@
         <v>1</v>
       </c>
       <c r="E314" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F314" t="n">
         <v>2</v>
@@ -17700,7 +17700,7 @@
         <v>0</v>
       </c>
       <c r="L314" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M314" t="n">
         <v>13</v>

</xml_diff>

<commit_message>
daily auto-refresh 2026-08-31 09:33
</commit_message>
<xml_diff>
--- a/daily_slab_mix.xlsx
+++ b/daily_slab_mix.xlsx
@@ -11137,10 +11137,10 @@
         <v>17</v>
       </c>
       <c r="F195" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G195" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H195" t="n">
         <v>2</v>
@@ -14266,7 +14266,7 @@
         <v>88</v>
       </c>
       <c r="D252" t="n">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E252" t="n">
         <v>79</v>
@@ -14275,7 +14275,7 @@
         <v>58</v>
       </c>
       <c r="G252" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H252" t="n">
         <v>5</v>
@@ -17126,7 +17126,7 @@
         <v>3</v>
       </c>
       <c r="D304" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E304" t="n">
         <v>36</v>
@@ -17135,7 +17135,7 @@
         <v>30</v>
       </c>
       <c r="G304" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H304" t="n">
         <v>17</v>
@@ -17728,7 +17728,7 @@
         <v>0</v>
       </c>
       <c r="C315" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D315" t="n">
         <v>0</v>
@@ -17743,7 +17743,7 @@
         <v>4</v>
       </c>
       <c r="H315" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I315" t="n">
         <v>0</v>
@@ -17755,7 +17755,7 @@
         <v>0</v>
       </c>
       <c r="L315" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="M315" t="n">
         <v>22</v>
@@ -17780,22 +17780,22 @@
         </is>
       </c>
       <c r="B316" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C316" t="n">
         <v>0</v>
       </c>
       <c r="D316" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E316" t="n">
         <v>0</v>
       </c>
       <c r="F316" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G316" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H316" t="n">
         <v>1</v>
@@ -17810,7 +17810,7 @@
         <v>1</v>
       </c>
       <c r="L316" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="M316" t="n">
         <v>20</v>
@@ -17835,7 +17835,7 @@
         </is>
       </c>
       <c r="B317" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C317" t="n">
         <v>0</v>
@@ -17844,28 +17844,28 @@
         <v>0</v>
       </c>
       <c r="E317" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F317" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G317" t="n">
         <v>6</v>
       </c>
       <c r="H317" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I317" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J317" t="n">
         <v>0</v>
       </c>
       <c r="K317" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L317" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="M317" t="n">
         <v>31</v>
@@ -17890,7 +17890,7 @@
         </is>
       </c>
       <c r="B318" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C318" t="n">
         <v>0</v>
@@ -17899,7 +17899,7 @@
         <v>0</v>
       </c>
       <c r="E318" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F318" t="n">
         <v>1</v>
@@ -17920,7 +17920,7 @@
         <v>0</v>
       </c>
       <c r="L318" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="M318" t="n">
         <v>22</v>
@@ -17945,7 +17945,7 @@
         </is>
       </c>
       <c r="B319" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C319" t="n">
         <v>0</v>
@@ -17954,10 +17954,10 @@
         <v>1</v>
       </c>
       <c r="E319" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F319" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G319" t="n">
         <v>2</v>
@@ -17972,10 +17972,10 @@
         <v>0</v>
       </c>
       <c r="K319" t="n">
+        <v>5</v>
+      </c>
+      <c r="L319" t="n">
         <v>4</v>
-      </c>
-      <c r="L319" t="n">
-        <v>9</v>
       </c>
       <c r="M319" t="n">
         <v>18</v>
@@ -18000,19 +18000,19 @@
         </is>
       </c>
       <c r="B320" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C320" t="n">
         <v>0</v>
       </c>
       <c r="D320" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E320" t="n">
         <v>0</v>
       </c>
       <c r="F320" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G320" t="n">
         <v>3</v>
@@ -18030,7 +18030,7 @@
         <v>0</v>
       </c>
       <c r="L320" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="M320" t="n">
         <v>18</v>

</xml_diff>

<commit_message>
daily auto-refresh 2026-08-31 09:35
</commit_message>
<xml_diff>
--- a/daily_slab_mix.xlsx
+++ b/daily_slab_mix.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q320"/>
+  <dimension ref="A1:O320"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -492,16 +492,6 @@
           <t>Sample units</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>Gift units (Turmeric Ginger)</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>Units incl. gifts</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -551,12 +541,6 @@
       <c r="O2" t="n">
         <v>4</v>
       </c>
-      <c r="P2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>4</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -606,12 +590,6 @@
       <c r="O3" t="n">
         <v>3</v>
       </c>
-      <c r="P3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -661,12 +639,6 @@
       <c r="O4" t="n">
         <v>1</v>
       </c>
-      <c r="P4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -716,12 +688,6 @@
       <c r="O5" t="n">
         <v>2</v>
       </c>
-      <c r="P5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -771,12 +737,6 @@
       <c r="O6" t="n">
         <v>17</v>
       </c>
-      <c r="P6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>17</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -826,12 +786,6 @@
       <c r="O7" t="n">
         <v>3</v>
       </c>
-      <c r="P7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -881,12 +835,6 @@
       <c r="O8" t="n">
         <v>1</v>
       </c>
-      <c r="P8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -936,12 +884,6 @@
       <c r="O9" t="n">
         <v>6</v>
       </c>
-      <c r="P9" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>6</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -991,12 +933,6 @@
       <c r="O10" t="n">
         <v>4</v>
       </c>
-      <c r="P10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>4</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1046,12 +982,6 @@
       <c r="O11" t="n">
         <v>1</v>
       </c>
-      <c r="P11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1101,12 +1031,6 @@
       <c r="O12" t="n">
         <v>5</v>
       </c>
-      <c r="P12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>5</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1156,12 +1080,6 @@
       <c r="O13" t="n">
         <v>6</v>
       </c>
-      <c r="P13" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>6</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1211,12 +1129,6 @@
       <c r="O14" t="n">
         <v>9</v>
       </c>
-      <c r="P14" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>9</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1266,12 +1178,6 @@
       <c r="O15" t="n">
         <v>7</v>
       </c>
-      <c r="P15" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>7</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1321,12 +1227,6 @@
       <c r="O16" t="n">
         <v>21</v>
       </c>
-      <c r="P16" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>21</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1376,12 +1276,6 @@
       <c r="O17" t="n">
         <v>15</v>
       </c>
-      <c r="P17" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1431,12 +1325,6 @@
       <c r="O18" t="n">
         <v>34</v>
       </c>
-      <c r="P18" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>34</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1486,12 +1374,6 @@
       <c r="O19" t="n">
         <v>28</v>
       </c>
-      <c r="P19" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>28</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1541,12 +1423,6 @@
       <c r="O20" t="n">
         <v>26</v>
       </c>
-      <c r="P20" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>26</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1596,12 +1472,6 @@
       <c r="O21" t="n">
         <v>1</v>
       </c>
-      <c r="P21" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1651,12 +1521,6 @@
       <c r="O22" t="n">
         <v>29</v>
       </c>
-      <c r="P22" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q22" t="n">
-        <v>29</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1706,12 +1570,6 @@
       <c r="O23" t="n">
         <v>29</v>
       </c>
-      <c r="P23" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>29</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1761,12 +1619,6 @@
       <c r="O24" t="n">
         <v>22</v>
       </c>
-      <c r="P24" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>22</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1816,12 +1668,6 @@
       <c r="O25" t="n">
         <v>21</v>
       </c>
-      <c r="P25" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>21</v>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1871,12 +1717,6 @@
       <c r="O26" t="n">
         <v>14</v>
       </c>
-      <c r="P26" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>14</v>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1926,12 +1766,6 @@
       <c r="O27" t="n">
         <v>18</v>
       </c>
-      <c r="P27" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q27" t="n">
-        <v>18</v>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1981,12 +1815,6 @@
       <c r="O28" t="n">
         <v>10</v>
       </c>
-      <c r="P28" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q28" t="n">
-        <v>10</v>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2036,12 +1864,6 @@
       <c r="O29" t="n">
         <v>14</v>
       </c>
-      <c r="P29" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q29" t="n">
-        <v>14</v>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2091,12 +1913,6 @@
       <c r="O30" t="n">
         <v>27</v>
       </c>
-      <c r="P30" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q30" t="n">
-        <v>27</v>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2146,12 +1962,6 @@
       <c r="O31" t="n">
         <v>22</v>
       </c>
-      <c r="P31" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q31" t="n">
-        <v>22</v>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2201,12 +2011,6 @@
       <c r="O32" t="n">
         <v>15</v>
       </c>
-      <c r="P32" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q32" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2256,12 +2060,6 @@
       <c r="O33" t="n">
         <v>34</v>
       </c>
-      <c r="P33" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q33" t="n">
-        <v>34</v>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2311,12 +2109,6 @@
       <c r="O34" t="n">
         <v>9</v>
       </c>
-      <c r="P34" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q34" t="n">
-        <v>9</v>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2366,12 +2158,6 @@
       <c r="O35" t="n">
         <v>3</v>
       </c>
-      <c r="P35" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q35" t="n">
-        <v>4</v>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2421,12 +2207,6 @@
       <c r="O36" t="n">
         <v>23</v>
       </c>
-      <c r="P36" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q36" t="n">
-        <v>23</v>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2476,12 +2256,6 @@
       <c r="O37" t="n">
         <v>1</v>
       </c>
-      <c r="P37" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q37" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2531,12 +2305,6 @@
       <c r="O38" t="n">
         <v>5</v>
       </c>
-      <c r="P38" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q38" t="n">
-        <v>11</v>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2586,12 +2354,6 @@
       <c r="O39" t="n">
         <v>12</v>
       </c>
-      <c r="P39" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q39" t="n">
-        <v>16</v>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2641,12 +2403,6 @@
       <c r="O40" t="n">
         <v>19</v>
       </c>
-      <c r="P40" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q40" t="n">
-        <v>20</v>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2696,12 +2452,6 @@
       <c r="O41" t="n">
         <v>24</v>
       </c>
-      <c r="P41" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q41" t="n">
-        <v>24</v>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2751,12 +2501,6 @@
       <c r="O42" t="n">
         <v>24</v>
       </c>
-      <c r="P42" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q42" t="n">
-        <v>24</v>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2806,12 +2550,6 @@
       <c r="O43" t="n">
         <v>13</v>
       </c>
-      <c r="P43" t="n">
-        <v>9</v>
-      </c>
-      <c r="Q43" t="n">
-        <v>22</v>
-      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2861,12 +2599,6 @@
       <c r="O44" t="n">
         <v>1</v>
       </c>
-      <c r="P44" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q44" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2916,12 +2648,6 @@
       <c r="O45" t="n">
         <v>10</v>
       </c>
-      <c r="P45" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q45" t="n">
-        <v>16</v>
-      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2971,12 +2697,6 @@
       <c r="O46" t="n">
         <v>31</v>
       </c>
-      <c r="P46" t="n">
-        <v>21</v>
-      </c>
-      <c r="Q46" t="n">
-        <v>52</v>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3026,12 +2746,6 @@
       <c r="O47" t="n">
         <v>36</v>
       </c>
-      <c r="P47" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q47" t="n">
-        <v>44</v>
-      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3081,12 +2795,6 @@
       <c r="O48" t="n">
         <v>49</v>
       </c>
-      <c r="P48" t="n">
-        <v>9</v>
-      </c>
-      <c r="Q48" t="n">
-        <v>58</v>
-      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3136,12 +2844,6 @@
       <c r="O49" t="n">
         <v>24</v>
       </c>
-      <c r="P49" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q49" t="n">
-        <v>26</v>
-      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3191,12 +2893,6 @@
       <c r="O50" t="n">
         <v>38</v>
       </c>
-      <c r="P50" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q50" t="n">
-        <v>40</v>
-      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3246,12 +2942,6 @@
       <c r="O51" t="n">
         <v>3</v>
       </c>
-      <c r="P51" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q51" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3301,12 +2991,6 @@
       <c r="O52" t="n">
         <v>3</v>
       </c>
-      <c r="P52" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q52" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3356,12 +3040,6 @@
       <c r="O53" t="n">
         <v>31</v>
       </c>
-      <c r="P53" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q53" t="n">
-        <v>32</v>
-      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3411,12 +3089,6 @@
       <c r="O54" t="n">
         <v>1</v>
       </c>
-      <c r="P54" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q54" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3466,12 +3138,6 @@
       <c r="O55" t="n">
         <v>3</v>
       </c>
-      <c r="P55" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q55" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3521,12 +3187,6 @@
       <c r="O56" t="n">
         <v>70</v>
       </c>
-      <c r="P56" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q56" t="n">
-        <v>72</v>
-      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3576,12 +3236,6 @@
       <c r="O57" t="n">
         <v>26</v>
       </c>
-      <c r="P57" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q57" t="n">
-        <v>26</v>
-      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3631,12 +3285,6 @@
       <c r="O58" t="n">
         <v>44</v>
       </c>
-      <c r="P58" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q58" t="n">
-        <v>47</v>
-      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3686,12 +3334,6 @@
       <c r="O59" t="n">
         <v>29</v>
       </c>
-      <c r="P59" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q59" t="n">
-        <v>29</v>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3741,12 +3383,6 @@
       <c r="O60" t="n">
         <v>39</v>
       </c>
-      <c r="P60" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q60" t="n">
-        <v>40</v>
-      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3796,12 +3432,6 @@
       <c r="O61" t="n">
         <v>27</v>
       </c>
-      <c r="P61" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q61" t="n">
-        <v>27</v>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3851,12 +3481,6 @@
       <c r="O62" t="n">
         <v>18</v>
       </c>
-      <c r="P62" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q62" t="n">
-        <v>18</v>
-      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3906,12 +3530,6 @@
       <c r="O63" t="n">
         <v>1</v>
       </c>
-      <c r="P63" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q63" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3961,12 +3579,6 @@
       <c r="O64" t="n">
         <v>32</v>
       </c>
-      <c r="P64" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q64" t="n">
-        <v>32</v>
-      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4016,12 +3628,6 @@
       <c r="O65" t="n">
         <v>41</v>
       </c>
-      <c r="P65" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q65" t="n">
-        <v>41</v>
-      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -4071,12 +3677,6 @@
       <c r="O66" t="n">
         <v>3</v>
       </c>
-      <c r="P66" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q66" t="n">
-        <v>4</v>
-      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -4126,12 +3726,6 @@
       <c r="O67" t="n">
         <v>38</v>
       </c>
-      <c r="P67" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q67" t="n">
-        <v>39</v>
-      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -4181,12 +3775,6 @@
       <c r="O68" t="n">
         <v>29</v>
       </c>
-      <c r="P68" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q68" t="n">
-        <v>29</v>
-      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -4236,12 +3824,6 @@
       <c r="O69" t="n">
         <v>4</v>
       </c>
-      <c r="P69" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q69" t="n">
-        <v>4</v>
-      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4291,12 +3873,6 @@
       <c r="O70" t="n">
         <v>29</v>
       </c>
-      <c r="P70" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q70" t="n">
-        <v>29</v>
-      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4346,12 +3922,6 @@
       <c r="O71" t="n">
         <v>35</v>
       </c>
-      <c r="P71" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q71" t="n">
-        <v>35</v>
-      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -4401,12 +3971,6 @@
       <c r="O72" t="n">
         <v>35</v>
       </c>
-      <c r="P72" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q72" t="n">
-        <v>35</v>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4456,12 +4020,6 @@
       <c r="O73" t="n">
         <v>12</v>
       </c>
-      <c r="P73" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q73" t="n">
-        <v>13</v>
-      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -4511,12 +4069,6 @@
       <c r="O74" t="n">
         <v>46</v>
       </c>
-      <c r="P74" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q74" t="n">
-        <v>46</v>
-      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4566,12 +4118,6 @@
       <c r="O75" t="n">
         <v>25</v>
       </c>
-      <c r="P75" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q75" t="n">
-        <v>26</v>
-      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4621,12 +4167,6 @@
       <c r="O76" t="n">
         <v>2</v>
       </c>
-      <c r="P76" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q76" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4676,12 +4216,6 @@
       <c r="O77" t="n">
         <v>10</v>
       </c>
-      <c r="P77" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q77" t="n">
-        <v>11</v>
-      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4731,12 +4265,6 @@
       <c r="O78" t="n">
         <v>57</v>
       </c>
-      <c r="P78" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q78" t="n">
-        <v>63</v>
-      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4786,12 +4314,6 @@
       <c r="O79" t="n">
         <v>40</v>
       </c>
-      <c r="P79" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q79" t="n">
-        <v>44</v>
-      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4841,12 +4363,6 @@
       <c r="O80" t="n">
         <v>24</v>
       </c>
-      <c r="P80" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q80" t="n">
-        <v>32</v>
-      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4896,12 +4412,6 @@
       <c r="O81" t="n">
         <v>11</v>
       </c>
-      <c r="P81" t="n">
-        <v>9</v>
-      </c>
-      <c r="Q81" t="n">
-        <v>20</v>
-      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4951,12 +4461,6 @@
       <c r="O82" t="n">
         <v>22</v>
       </c>
-      <c r="P82" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q82" t="n">
-        <v>39</v>
-      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -5006,12 +4510,6 @@
       <c r="O83" t="n">
         <v>1</v>
       </c>
-      <c r="P83" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q83" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -5061,12 +4559,6 @@
       <c r="O84" t="n">
         <v>16</v>
       </c>
-      <c r="P84" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q84" t="n">
-        <v>21</v>
-      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -5116,12 +4608,6 @@
       <c r="O85" t="n">
         <v>20</v>
       </c>
-      <c r="P85" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q85" t="n">
-        <v>35</v>
-      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -5171,12 +4657,6 @@
       <c r="O86" t="n">
         <v>36</v>
       </c>
-      <c r="P86" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q86" t="n">
-        <v>51</v>
-      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -5226,12 +4706,6 @@
       <c r="O87" t="n">
         <v>21</v>
       </c>
-      <c r="P87" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q87" t="n">
-        <v>36</v>
-      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -5281,12 +4755,6 @@
       <c r="O88" t="n">
         <v>23</v>
       </c>
-      <c r="P88" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q88" t="n">
-        <v>38</v>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -5336,12 +4804,6 @@
       <c r="O89" t="n">
         <v>14</v>
       </c>
-      <c r="P89" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q89" t="n">
-        <v>20</v>
-      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -5391,12 +4853,6 @@
       <c r="O90" t="n">
         <v>13</v>
       </c>
-      <c r="P90" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q90" t="n">
-        <v>17</v>
-      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -5446,12 +4902,6 @@
       <c r="O91" t="n">
         <v>39</v>
       </c>
-      <c r="P91" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q91" t="n">
-        <v>39</v>
-      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -5501,12 +4951,6 @@
       <c r="O92" t="n">
         <v>28</v>
       </c>
-      <c r="P92" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q92" t="n">
-        <v>28</v>
-      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -5556,12 +5000,6 @@
       <c r="O93" t="n">
         <v>21</v>
       </c>
-      <c r="P93" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q93" t="n">
-        <v>21</v>
-      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -5611,12 +5049,6 @@
       <c r="O94" t="n">
         <v>46</v>
       </c>
-      <c r="P94" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q94" t="n">
-        <v>61</v>
-      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -5666,12 +5098,6 @@
       <c r="O95" t="n">
         <v>19</v>
       </c>
-      <c r="P95" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q95" t="n">
-        <v>24</v>
-      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -5721,12 +5147,6 @@
       <c r="O96" t="n">
         <v>8</v>
       </c>
-      <c r="P96" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q96" t="n">
-        <v>8</v>
-      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -5776,12 +5196,6 @@
       <c r="O97" t="n">
         <v>2</v>
       </c>
-      <c r="P97" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q97" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -5831,12 +5245,6 @@
       <c r="O98" t="n">
         <v>21</v>
       </c>
-      <c r="P98" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q98" t="n">
-        <v>27</v>
-      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -5886,12 +5294,6 @@
       <c r="O99" t="n">
         <v>23</v>
       </c>
-      <c r="P99" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q99" t="n">
-        <v>23</v>
-      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -5941,12 +5343,6 @@
       <c r="O100" t="n">
         <v>1</v>
       </c>
-      <c r="P100" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q100" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -5996,12 +5392,6 @@
       <c r="O101" t="n">
         <v>42</v>
       </c>
-      <c r="P101" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q101" t="n">
-        <v>49</v>
-      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -6051,12 +5441,6 @@
       <c r="O102" t="n">
         <v>27</v>
       </c>
-      <c r="P102" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q102" t="n">
-        <v>37</v>
-      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -6106,12 +5490,6 @@
       <c r="O103" t="n">
         <v>6</v>
       </c>
-      <c r="P103" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q103" t="n">
-        <v>6</v>
-      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -6161,12 +5539,6 @@
       <c r="O104" t="n">
         <v>53</v>
       </c>
-      <c r="P104" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q104" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -6216,12 +5588,6 @@
       <c r="O105" t="n">
         <v>29</v>
       </c>
-      <c r="P105" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q105" t="n">
-        <v>33</v>
-      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -6271,12 +5637,6 @@
       <c r="O106" t="n">
         <v>19</v>
       </c>
-      <c r="P106" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q106" t="n">
-        <v>26</v>
-      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -6326,12 +5686,6 @@
       <c r="O107" t="n">
         <v>1</v>
       </c>
-      <c r="P107" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q107" t="n">
-        <v>12</v>
-      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -6381,12 +5735,6 @@
       <c r="O108" t="n">
         <v>2</v>
       </c>
-      <c r="P108" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q108" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -6436,12 +5784,6 @@
       <c r="O109" t="n">
         <v>3</v>
       </c>
-      <c r="P109" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q109" t="n">
-        <v>14</v>
-      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -6491,12 +5833,6 @@
       <c r="O110" t="n">
         <v>27</v>
       </c>
-      <c r="P110" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q110" t="n">
-        <v>38</v>
-      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -6546,12 +5882,6 @@
       <c r="O111" t="n">
         <v>19</v>
       </c>
-      <c r="P111" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q111" t="n">
-        <v>21</v>
-      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -6601,12 +5931,6 @@
       <c r="O112" t="n">
         <v>34</v>
       </c>
-      <c r="P112" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q112" t="n">
-        <v>36</v>
-      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -6656,12 +5980,6 @@
       <c r="O113" t="n">
         <v>5</v>
       </c>
-      <c r="P113" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q113" t="n">
-        <v>5</v>
-      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -6711,12 +6029,6 @@
       <c r="O114" t="n">
         <v>40</v>
       </c>
-      <c r="P114" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q114" t="n">
-        <v>56</v>
-      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -6766,12 +6078,6 @@
       <c r="O115" t="n">
         <v>46</v>
       </c>
-      <c r="P115" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q115" t="n">
-        <v>56</v>
-      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -6821,12 +6127,6 @@
       <c r="O116" t="n">
         <v>33</v>
       </c>
-      <c r="P116" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q116" t="n">
-        <v>36</v>
-      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -6876,12 +6176,6 @@
       <c r="O117" t="n">
         <v>26</v>
       </c>
-      <c r="P117" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q117" t="n">
-        <v>32</v>
-      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -6931,12 +6225,6 @@
       <c r="O118" t="n">
         <v>31</v>
       </c>
-      <c r="P118" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q118" t="n">
-        <v>37</v>
-      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -6986,12 +6274,6 @@
       <c r="O119" t="n">
         <v>142</v>
       </c>
-      <c r="P119" t="n">
-        <v>14</v>
-      </c>
-      <c r="Q119" t="n">
-        <v>156</v>
-      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -7041,12 +6323,6 @@
       <c r="O120" t="n">
         <v>41</v>
       </c>
-      <c r="P120" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q120" t="n">
-        <v>41</v>
-      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -7096,12 +6372,6 @@
       <c r="O121" t="n">
         <v>34</v>
       </c>
-      <c r="P121" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q121" t="n">
-        <v>34</v>
-      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -7151,12 +6421,6 @@
       <c r="O122" t="n">
         <v>24</v>
       </c>
-      <c r="P122" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q122" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -7206,12 +6470,6 @@
       <c r="O123" t="n">
         <v>13</v>
       </c>
-      <c r="P123" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q123" t="n">
-        <v>14</v>
-      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -7261,12 +6519,6 @@
       <c r="O124" t="n">
         <v>98</v>
       </c>
-      <c r="P124" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q124" t="n">
-        <v>103</v>
-      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -7316,12 +6568,6 @@
       <c r="O125" t="n">
         <v>12</v>
       </c>
-      <c r="P125" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q125" t="n">
-        <v>12</v>
-      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -7371,12 +6617,6 @@
       <c r="O126" t="n">
         <v>29</v>
       </c>
-      <c r="P126" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q126" t="n">
-        <v>35</v>
-      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -7426,12 +6666,6 @@
       <c r="O127" t="n">
         <v>24</v>
       </c>
-      <c r="P127" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q127" t="n">
-        <v>27</v>
-      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -7481,12 +6715,6 @@
       <c r="O128" t="n">
         <v>21</v>
       </c>
-      <c r="P128" t="n">
-        <v>9</v>
-      </c>
-      <c r="Q128" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -7536,12 +6764,6 @@
       <c r="O129" t="n">
         <v>33</v>
       </c>
-      <c r="P129" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q129" t="n">
-        <v>46</v>
-      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -7591,12 +6813,6 @@
       <c r="O130" t="n">
         <v>5</v>
       </c>
-      <c r="P130" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q130" t="n">
-        <v>6</v>
-      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -7646,12 +6862,6 @@
       <c r="O131" t="n">
         <v>2</v>
       </c>
-      <c r="P131" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q131" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -7701,12 +6911,6 @@
       <c r="O132" t="n">
         <v>81</v>
       </c>
-      <c r="P132" t="n">
-        <v>25</v>
-      </c>
-      <c r="Q132" t="n">
-        <v>106</v>
-      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -7756,12 +6960,6 @@
       <c r="O133" t="n">
         <v>25</v>
       </c>
-      <c r="P133" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q133" t="n">
-        <v>42</v>
-      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -7811,12 +7009,6 @@
       <c r="O134" t="n">
         <v>32</v>
       </c>
-      <c r="P134" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q134" t="n">
-        <v>40</v>
-      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -7866,12 +7058,6 @@
       <c r="O135" t="n">
         <v>60</v>
       </c>
-      <c r="P135" t="n">
-        <v>28</v>
-      </c>
-      <c r="Q135" t="n">
-        <v>88</v>
-      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -7921,12 +7107,6 @@
       <c r="O136" t="n">
         <v>28</v>
       </c>
-      <c r="P136" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q136" t="n">
-        <v>43</v>
-      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -7976,12 +7156,6 @@
       <c r="O137" t="n">
         <v>2</v>
       </c>
-      <c r="P137" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q137" t="n">
-        <v>4</v>
-      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -8031,12 +7205,6 @@
       <c r="O138" t="n">
         <v>34</v>
       </c>
-      <c r="P138" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q138" t="n">
-        <v>49</v>
-      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -8086,12 +7254,6 @@
       <c r="O139" t="n">
         <v>45</v>
       </c>
-      <c r="P139" t="n">
-        <v>31</v>
-      </c>
-      <c r="Q139" t="n">
-        <v>76</v>
-      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -8141,12 +7303,6 @@
       <c r="O140" t="n">
         <v>45</v>
       </c>
-      <c r="P140" t="n">
-        <v>30</v>
-      </c>
-      <c r="Q140" t="n">
-        <v>75</v>
-      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -8196,12 +7352,6 @@
       <c r="O141" t="n">
         <v>35</v>
       </c>
-      <c r="P141" t="n">
-        <v>28</v>
-      </c>
-      <c r="Q141" t="n">
-        <v>63</v>
-      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -8251,12 +7401,6 @@
       <c r="O142" t="n">
         <v>29</v>
       </c>
-      <c r="P142" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q142" t="n">
-        <v>45</v>
-      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -8306,12 +7450,6 @@
       <c r="O143" t="n">
         <v>50</v>
       </c>
-      <c r="P143" t="n">
-        <v>28</v>
-      </c>
-      <c r="Q143" t="n">
-        <v>78</v>
-      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -8361,12 +7499,6 @@
       <c r="O144" t="n">
         <v>47</v>
       </c>
-      <c r="P144" t="n">
-        <v>23</v>
-      </c>
-      <c r="Q144" t="n">
-        <v>70</v>
-      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -8416,12 +7548,6 @@
       <c r="O145" t="n">
         <v>77</v>
       </c>
-      <c r="P145" t="n">
-        <v>36</v>
-      </c>
-      <c r="Q145" t="n">
-        <v>113</v>
-      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -8471,12 +7597,6 @@
       <c r="O146" t="n">
         <v>34</v>
       </c>
-      <c r="P146" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q146" t="n">
-        <v>44</v>
-      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -8526,12 +7646,6 @@
       <c r="O147" t="n">
         <v>81</v>
       </c>
-      <c r="P147" t="n">
-        <v>41</v>
-      </c>
-      <c r="Q147" t="n">
-        <v>122</v>
-      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -8581,12 +7695,6 @@
       <c r="O148" t="n">
         <v>1</v>
       </c>
-      <c r="P148" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q148" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -8636,12 +7744,6 @@
       <c r="O149" t="n">
         <v>47</v>
       </c>
-      <c r="P149" t="n">
-        <v>14</v>
-      </c>
-      <c r="Q149" t="n">
-        <v>61</v>
-      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -8691,12 +7793,6 @@
       <c r="O150" t="n">
         <v>42</v>
       </c>
-      <c r="P150" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q150" t="n">
-        <v>54</v>
-      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -8746,12 +7842,6 @@
       <c r="O151" t="n">
         <v>30</v>
       </c>
-      <c r="P151" t="n">
-        <v>19</v>
-      </c>
-      <c r="Q151" t="n">
-        <v>49</v>
-      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -8801,12 +7891,6 @@
       <c r="O152" t="n">
         <v>59</v>
       </c>
-      <c r="P152" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q152" t="n">
-        <v>70</v>
-      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -8856,12 +7940,6 @@
       <c r="O153" t="n">
         <v>113</v>
       </c>
-      <c r="P153" t="n">
-        <v>54</v>
-      </c>
-      <c r="Q153" t="n">
-        <v>167</v>
-      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -8911,12 +7989,6 @@
       <c r="O154" t="n">
         <v>44</v>
       </c>
-      <c r="P154" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q154" t="n">
-        <v>52</v>
-      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -8966,12 +8038,6 @@
       <c r="O155" t="n">
         <v>52</v>
       </c>
-      <c r="P155" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q155" t="n">
-        <v>70</v>
-      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -9021,12 +8087,6 @@
       <c r="O156" t="n">
         <v>55</v>
       </c>
-      <c r="P156" t="n">
-        <v>17</v>
-      </c>
-      <c r="Q156" t="n">
-        <v>72</v>
-      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -9076,12 +8136,6 @@
       <c r="O157" t="n">
         <v>42</v>
       </c>
-      <c r="P157" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q157" t="n">
-        <v>58</v>
-      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -9131,12 +8185,6 @@
       <c r="O158" t="n">
         <v>37</v>
       </c>
-      <c r="P158" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q158" t="n">
-        <v>55</v>
-      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -9186,12 +8234,6 @@
       <c r="O159" t="n">
         <v>27</v>
       </c>
-      <c r="P159" t="n">
-        <v>16</v>
-      </c>
-      <c r="Q159" t="n">
-        <v>43</v>
-      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -9241,12 +8283,6 @@
       <c r="O160" t="n">
         <v>39</v>
       </c>
-      <c r="P160" t="n">
-        <v>23</v>
-      </c>
-      <c r="Q160" t="n">
-        <v>62</v>
-      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -9296,12 +8332,6 @@
       <c r="O161" t="n">
         <v>34</v>
       </c>
-      <c r="P161" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q161" t="n">
-        <v>46</v>
-      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -9351,12 +8381,6 @@
       <c r="O162" t="n">
         <v>32</v>
       </c>
-      <c r="P162" t="n">
-        <v>12</v>
-      </c>
-      <c r="Q162" t="n">
-        <v>44</v>
-      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -9406,12 +8430,6 @@
       <c r="O163" t="n">
         <v>137</v>
       </c>
-      <c r="P163" t="n">
-        <v>60</v>
-      </c>
-      <c r="Q163" t="n">
-        <v>197</v>
-      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -9461,12 +8479,6 @@
       <c r="O164" t="n">
         <v>40</v>
       </c>
-      <c r="P164" t="n">
-        <v>21</v>
-      </c>
-      <c r="Q164" t="n">
-        <v>61</v>
-      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -9516,12 +8528,6 @@
       <c r="O165" t="n">
         <v>119</v>
       </c>
-      <c r="P165" t="n">
-        <v>52</v>
-      </c>
-      <c r="Q165" t="n">
-        <v>171</v>
-      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -9571,12 +8577,6 @@
       <c r="O166" t="n">
         <v>40</v>
       </c>
-      <c r="P166" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q166" t="n">
-        <v>41</v>
-      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -9626,12 +8626,6 @@
       <c r="O167" t="n">
         <v>70</v>
       </c>
-      <c r="P167" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q167" t="n">
-        <v>70</v>
-      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -9681,12 +8675,6 @@
       <c r="O168" t="n">
         <v>73</v>
       </c>
-      <c r="P168" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q168" t="n">
-        <v>73</v>
-      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -9736,12 +8724,6 @@
       <c r="O169" t="n">
         <v>50</v>
       </c>
-      <c r="P169" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q169" t="n">
-        <v>50</v>
-      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -9791,12 +8773,6 @@
       <c r="O170" t="n">
         <v>71</v>
       </c>
-      <c r="P170" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q170" t="n">
-        <v>75</v>
-      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -9846,12 +8822,6 @@
       <c r="O171" t="n">
         <v>126</v>
       </c>
-      <c r="P171" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q171" t="n">
-        <v>126</v>
-      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -9901,12 +8871,6 @@
       <c r="O172" t="n">
         <v>115</v>
       </c>
-      <c r="P172" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q172" t="n">
-        <v>115</v>
-      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -9956,12 +8920,6 @@
       <c r="O173" t="n">
         <v>38</v>
       </c>
-      <c r="P173" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q173" t="n">
-        <v>38</v>
-      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -10011,12 +8969,6 @@
       <c r="O174" t="n">
         <v>1</v>
       </c>
-      <c r="P174" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q174" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -10066,12 +9018,6 @@
       <c r="O175" t="n">
         <v>138</v>
       </c>
-      <c r="P175" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q175" t="n">
-        <v>138</v>
-      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -10121,12 +9067,6 @@
       <c r="O176" t="n">
         <v>129</v>
       </c>
-      <c r="P176" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q176" t="n">
-        <v>129</v>
-      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -10176,12 +9116,6 @@
       <c r="O177" t="n">
         <v>50</v>
       </c>
-      <c r="P177" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q177" t="n">
-        <v>53</v>
-      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -10231,12 +9165,6 @@
       <c r="O178" t="n">
         <v>68</v>
       </c>
-      <c r="P178" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q178" t="n">
-        <v>68</v>
-      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -10286,12 +9214,6 @@
       <c r="O179" t="n">
         <v>33</v>
       </c>
-      <c r="P179" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q179" t="n">
-        <v>33</v>
-      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -10341,12 +9263,6 @@
       <c r="O180" t="n">
         <v>2</v>
       </c>
-      <c r="P180" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q180" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -10396,12 +9312,6 @@
       <c r="O181" t="n">
         <v>133</v>
       </c>
-      <c r="P181" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q181" t="n">
-        <v>133</v>
-      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -10451,12 +9361,6 @@
       <c r="O182" t="n">
         <v>125</v>
       </c>
-      <c r="P182" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q182" t="n">
-        <v>128</v>
-      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -10506,12 +9410,6 @@
       <c r="O183" t="n">
         <v>2</v>
       </c>
-      <c r="P183" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q183" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -10561,12 +9459,6 @@
       <c r="O184" t="n">
         <v>84</v>
       </c>
-      <c r="P184" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q184" t="n">
-        <v>85</v>
-      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -10616,12 +9508,6 @@
       <c r="O185" t="n">
         <v>58</v>
       </c>
-      <c r="P185" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q185" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -10671,12 +9557,6 @@
       <c r="O186" t="n">
         <v>1</v>
       </c>
-      <c r="P186" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q186" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -10726,12 +9606,6 @@
       <c r="O187" t="n">
         <v>104</v>
       </c>
-      <c r="P187" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q187" t="n">
-        <v>104</v>
-      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -10781,12 +9655,6 @@
       <c r="O188" t="n">
         <v>63</v>
       </c>
-      <c r="P188" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q188" t="n">
-        <v>63</v>
-      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -10836,12 +9704,6 @@
       <c r="O189" t="n">
         <v>62</v>
       </c>
-      <c r="P189" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q189" t="n">
-        <v>62</v>
-      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -10891,12 +9753,6 @@
       <c r="O190" t="n">
         <v>58</v>
       </c>
-      <c r="P190" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q190" t="n">
-        <v>58</v>
-      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -10946,12 +9802,6 @@
       <c r="O191" t="n">
         <v>45</v>
       </c>
-      <c r="P191" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q191" t="n">
-        <v>45</v>
-      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -11001,12 +9851,6 @@
       <c r="O192" t="n">
         <v>1</v>
       </c>
-      <c r="P192" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q192" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -11056,12 +9900,6 @@
       <c r="O193" t="n">
         <v>182</v>
       </c>
-      <c r="P193" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q193" t="n">
-        <v>182</v>
-      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -11111,12 +9949,6 @@
       <c r="O194" t="n">
         <v>4</v>
       </c>
-      <c r="P194" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q194" t="n">
-        <v>5</v>
-      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -11166,12 +9998,6 @@
       <c r="O195" t="n">
         <v>105</v>
       </c>
-      <c r="P195" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q195" t="n">
-        <v>105</v>
-      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -11221,12 +10047,6 @@
       <c r="O196" t="n">
         <v>102</v>
       </c>
-      <c r="P196" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q196" t="n">
-        <v>103</v>
-      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -11276,12 +10096,6 @@
       <c r="O197" t="n">
         <v>28</v>
       </c>
-      <c r="P197" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q197" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -11331,12 +10145,6 @@
       <c r="O198" t="n">
         <v>9</v>
       </c>
-      <c r="P198" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q198" t="n">
-        <v>9</v>
-      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -11386,12 +10194,6 @@
       <c r="O199" t="n">
         <v>10</v>
       </c>
-      <c r="P199" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q199" t="n">
-        <v>10</v>
-      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -11441,12 +10243,6 @@
       <c r="O200" t="n">
         <v>15</v>
       </c>
-      <c r="P200" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q200" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -11496,12 +10292,6 @@
       <c r="O201" t="n">
         <v>10</v>
       </c>
-      <c r="P201" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q201" t="n">
-        <v>10</v>
-      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -11551,12 +10341,6 @@
       <c r="O202" t="n">
         <v>24</v>
       </c>
-      <c r="P202" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q202" t="n">
-        <v>24</v>
-      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -11606,12 +10390,6 @@
       <c r="O203" t="n">
         <v>21</v>
       </c>
-      <c r="P203" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q203" t="n">
-        <v>25</v>
-      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -11661,12 +10439,6 @@
       <c r="O204" t="n">
         <v>17</v>
       </c>
-      <c r="P204" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q204" t="n">
-        <v>18</v>
-      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -11716,12 +10488,6 @@
       <c r="O205" t="n">
         <v>1</v>
       </c>
-      <c r="P205" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q205" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -11771,12 +10537,6 @@
       <c r="O206" t="n">
         <v>22</v>
       </c>
-      <c r="P206" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q206" t="n">
-        <v>23</v>
-      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -11826,12 +10586,6 @@
       <c r="O207" t="n">
         <v>27</v>
       </c>
-      <c r="P207" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q207" t="n">
-        <v>27</v>
-      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -11881,12 +10635,6 @@
       <c r="O208" t="n">
         <v>2</v>
       </c>
-      <c r="P208" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q208" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -11936,12 +10684,6 @@
       <c r="O209" t="n">
         <v>53</v>
       </c>
-      <c r="P209" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q209" t="n">
-        <v>53</v>
-      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -11991,12 +10733,6 @@
       <c r="O210" t="n">
         <v>33</v>
       </c>
-      <c r="P210" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q210" t="n">
-        <v>33</v>
-      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -12046,12 +10782,6 @@
       <c r="O211" t="n">
         <v>1</v>
       </c>
-      <c r="P211" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q211" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -12101,12 +10831,6 @@
       <c r="O212" t="n">
         <v>1</v>
       </c>
-      <c r="P212" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q212" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -12156,12 +10880,6 @@
       <c r="O213" t="n">
         <v>59</v>
       </c>
-      <c r="P213" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q213" t="n">
-        <v>59</v>
-      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -12211,12 +10929,6 @@
       <c r="O214" t="n">
         <v>29</v>
       </c>
-      <c r="P214" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q214" t="n">
-        <v>29</v>
-      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -12266,12 +10978,6 @@
       <c r="O215" t="n">
         <v>25</v>
       </c>
-      <c r="P215" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q215" t="n">
-        <v>25</v>
-      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -12321,12 +11027,6 @@
       <c r="O216" t="n">
         <v>26</v>
       </c>
-      <c r="P216" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q216" t="n">
-        <v>26</v>
-      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -12376,12 +11076,6 @@
       <c r="O217" t="n">
         <v>23</v>
       </c>
-      <c r="P217" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q217" t="n">
-        <v>24</v>
-      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -12431,12 +11125,6 @@
       <c r="O218" t="n">
         <v>2</v>
       </c>
-      <c r="P218" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q218" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -12486,12 +11174,6 @@
       <c r="O219" t="n">
         <v>48</v>
       </c>
-      <c r="P219" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q219" t="n">
-        <v>50</v>
-      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -12541,12 +11223,6 @@
       <c r="O220" t="n">
         <v>39</v>
       </c>
-      <c r="P220" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q220" t="n">
-        <v>41</v>
-      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -12596,12 +11272,6 @@
       <c r="O221" t="n">
         <v>41</v>
       </c>
-      <c r="P221" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q221" t="n">
-        <v>46</v>
-      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -12651,12 +11321,6 @@
       <c r="O222" t="n">
         <v>65</v>
       </c>
-      <c r="P222" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q222" t="n">
-        <v>80</v>
-      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -12706,12 +11370,6 @@
       <c r="O223" t="n">
         <v>2</v>
       </c>
-      <c r="P223" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q223" t="n">
-        <v>3</v>
-      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -12761,12 +11419,6 @@
       <c r="O224" t="n">
         <v>89</v>
       </c>
-      <c r="P224" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q224" t="n">
-        <v>89</v>
-      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -12816,12 +11468,6 @@
       <c r="O225" t="n">
         <v>58</v>
       </c>
-      <c r="P225" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q225" t="n">
-        <v>61</v>
-      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -12871,12 +11517,6 @@
       <c r="O226" t="n">
         <v>73</v>
       </c>
-      <c r="P226" t="n">
-        <v>23</v>
-      </c>
-      <c r="Q226" t="n">
-        <v>96</v>
-      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -12926,12 +11566,6 @@
       <c r="O227" t="n">
         <v>199</v>
       </c>
-      <c r="P227" t="n">
-        <v>44</v>
-      </c>
-      <c r="Q227" t="n">
-        <v>243</v>
-      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -12981,12 +11615,6 @@
       <c r="O228" t="n">
         <v>94</v>
       </c>
-      <c r="P228" t="n">
-        <v>41</v>
-      </c>
-      <c r="Q228" t="n">
-        <v>135</v>
-      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -13036,12 +11664,6 @@
       <c r="O229" t="n">
         <v>139</v>
       </c>
-      <c r="P229" t="n">
-        <v>46</v>
-      </c>
-      <c r="Q229" t="n">
-        <v>185</v>
-      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -13091,12 +11713,6 @@
       <c r="O230" t="n">
         <v>2</v>
       </c>
-      <c r="P230" t="n">
-        <v>48</v>
-      </c>
-      <c r="Q230" t="n">
-        <v>50</v>
-      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -13146,12 +11762,6 @@
       <c r="O231" t="n">
         <v>168</v>
       </c>
-      <c r="P231" t="n">
-        <v>47</v>
-      </c>
-      <c r="Q231" t="n">
-        <v>215</v>
-      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -13201,12 +11811,6 @@
       <c r="O232" t="n">
         <v>71</v>
       </c>
-      <c r="P232" t="n">
-        <v>38</v>
-      </c>
-      <c r="Q232" t="n">
-        <v>109</v>
-      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -13256,12 +11860,6 @@
       <c r="O233" t="n">
         <v>77</v>
       </c>
-      <c r="P233" t="n">
-        <v>21</v>
-      </c>
-      <c r="Q233" t="n">
-        <v>98</v>
-      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -13311,12 +11909,6 @@
       <c r="O234" t="n">
         <v>46</v>
       </c>
-      <c r="P234" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q234" t="n">
-        <v>46</v>
-      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -13366,12 +11958,6 @@
       <c r="O235" t="n">
         <v>42</v>
       </c>
-      <c r="P235" t="n">
-        <v>19</v>
-      </c>
-      <c r="Q235" t="n">
-        <v>61</v>
-      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -13421,12 +12007,6 @@
       <c r="O236" t="n">
         <v>5</v>
       </c>
-      <c r="P236" t="n">
-        <v>42</v>
-      </c>
-      <c r="Q236" t="n">
-        <v>47</v>
-      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -13476,12 +12056,6 @@
       <c r="O237" t="n">
         <v>204</v>
       </c>
-      <c r="P237" t="n">
-        <v>30</v>
-      </c>
-      <c r="Q237" t="n">
-        <v>234</v>
-      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -13531,12 +12105,6 @@
       <c r="O238" t="n">
         <v>50</v>
       </c>
-      <c r="P238" t="n">
-        <v>40</v>
-      </c>
-      <c r="Q238" t="n">
-        <v>90</v>
-      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -13586,12 +12154,6 @@
       <c r="O239" t="n">
         <v>32</v>
       </c>
-      <c r="P239" t="n">
-        <v>29</v>
-      </c>
-      <c r="Q239" t="n">
-        <v>61</v>
-      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -13641,12 +12203,6 @@
       <c r="O240" t="n">
         <v>61</v>
       </c>
-      <c r="P240" t="n">
-        <v>29</v>
-      </c>
-      <c r="Q240" t="n">
-        <v>90</v>
-      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -13696,12 +12252,6 @@
       <c r="O241" t="n">
         <v>43</v>
       </c>
-      <c r="P241" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q241" t="n">
-        <v>43</v>
-      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -13751,12 +12301,6 @@
       <c r="O242" t="n">
         <v>2</v>
       </c>
-      <c r="P242" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q242" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -13806,12 +12350,6 @@
       <c r="O243" t="n">
         <v>1</v>
       </c>
-      <c r="P243" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q243" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -13861,12 +12399,6 @@
       <c r="O244" t="n">
         <v>2</v>
       </c>
-      <c r="P244" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q244" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -13916,12 +12448,6 @@
       <c r="O245" t="n">
         <v>60</v>
       </c>
-      <c r="P245" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q245" t="n">
-        <v>60</v>
-      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -13971,12 +12497,6 @@
       <c r="O246" t="n">
         <v>152</v>
       </c>
-      <c r="P246" t="n">
-        <v>19</v>
-      </c>
-      <c r="Q246" t="n">
-        <v>171</v>
-      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -14026,12 +12546,6 @@
       <c r="O247" t="n">
         <v>236</v>
       </c>
-      <c r="P247" t="n">
-        <v>32</v>
-      </c>
-      <c r="Q247" t="n">
-        <v>268</v>
-      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -14081,12 +12595,6 @@
       <c r="O248" t="n">
         <v>72</v>
       </c>
-      <c r="P248" t="n">
-        <v>36</v>
-      </c>
-      <c r="Q248" t="n">
-        <v>108</v>
-      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -14136,12 +12644,6 @@
       <c r="O249" t="n">
         <v>6</v>
       </c>
-      <c r="P249" t="n">
-        <v>30</v>
-      </c>
-      <c r="Q249" t="n">
-        <v>36</v>
-      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -14191,12 +12693,6 @@
       <c r="O250" t="n">
         <v>6</v>
       </c>
-      <c r="P250" t="n">
-        <v>18</v>
-      </c>
-      <c r="Q250" t="n">
-        <v>24</v>
-      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -14246,12 +12742,6 @@
       <c r="O251" t="n">
         <v>296</v>
       </c>
-      <c r="P251" t="n">
-        <v>23</v>
-      </c>
-      <c r="Q251" t="n">
-        <v>319</v>
-      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -14301,12 +12791,6 @@
       <c r="O252" t="n">
         <v>1172</v>
       </c>
-      <c r="P252" t="n">
-        <v>25</v>
-      </c>
-      <c r="Q252" t="n">
-        <v>1197</v>
-      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -14356,12 +12840,6 @@
       <c r="O253" t="n">
         <v>161</v>
       </c>
-      <c r="P253" t="n">
-        <v>38</v>
-      </c>
-      <c r="Q253" t="n">
-        <v>199</v>
-      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -14411,12 +12889,6 @@
       <c r="O254" t="n">
         <v>173</v>
       </c>
-      <c r="P254" t="n">
-        <v>33</v>
-      </c>
-      <c r="Q254" t="n">
-        <v>206</v>
-      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -14466,12 +12938,6 @@
       <c r="O255" t="n">
         <v>192</v>
       </c>
-      <c r="P255" t="n">
-        <v>49</v>
-      </c>
-      <c r="Q255" t="n">
-        <v>241</v>
-      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -14521,12 +12987,6 @@
       <c r="O256" t="n">
         <v>269</v>
       </c>
-      <c r="P256" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q256" t="n">
-        <v>269</v>
-      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -14576,12 +13036,6 @@
       <c r="O257" t="n">
         <v>61</v>
       </c>
-      <c r="P257" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q257" t="n">
-        <v>61</v>
-      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -14631,12 +13085,6 @@
       <c r="O258" t="n">
         <v>135</v>
       </c>
-      <c r="P258" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q258" t="n">
-        <v>145</v>
-      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -14686,12 +13134,6 @@
       <c r="O259" t="n">
         <v>67</v>
       </c>
-      <c r="P259" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q259" t="n">
-        <v>67</v>
-      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -14741,12 +13183,6 @@
       <c r="O260" t="n">
         <v>12</v>
       </c>
-      <c r="P260" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q260" t="n">
-        <v>12</v>
-      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -14796,12 +13232,6 @@
       <c r="O261" t="n">
         <v>64</v>
       </c>
-      <c r="P261" t="n">
-        <v>37</v>
-      </c>
-      <c r="Q261" t="n">
-        <v>101</v>
-      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -14851,12 +13281,6 @@
       <c r="O262" t="n">
         <v>49</v>
       </c>
-      <c r="P262" t="n">
-        <v>43</v>
-      </c>
-      <c r="Q262" t="n">
-        <v>92</v>
-      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -14906,12 +13330,6 @@
       <c r="O263" t="n">
         <v>26</v>
       </c>
-      <c r="P263" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q263" t="n">
-        <v>26</v>
-      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -14961,12 +13379,6 @@
       <c r="O264" t="n">
         <v>30</v>
       </c>
-      <c r="P264" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q264" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -15016,12 +13428,6 @@
       <c r="O265" t="n">
         <v>233</v>
       </c>
-      <c r="P265" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q265" t="n">
-        <v>233</v>
-      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -15071,12 +13477,6 @@
       <c r="O266" t="n">
         <v>274</v>
       </c>
-      <c r="P266" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q266" t="n">
-        <v>274</v>
-      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -15126,12 +13526,6 @@
       <c r="O267" t="n">
         <v>85</v>
       </c>
-      <c r="P267" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q267" t="n">
-        <v>85</v>
-      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -15181,12 +13575,6 @@
       <c r="O268" t="n">
         <v>103</v>
       </c>
-      <c r="P268" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q268" t="n">
-        <v>103</v>
-      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -15236,12 +13624,6 @@
       <c r="O269" t="n">
         <v>93</v>
       </c>
-      <c r="P269" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q269" t="n">
-        <v>93</v>
-      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -15291,12 +13673,6 @@
       <c r="O270" t="n">
         <v>5</v>
       </c>
-      <c r="P270" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q270" t="n">
-        <v>5</v>
-      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -15346,12 +13722,6 @@
       <c r="O271" t="n">
         <v>146</v>
       </c>
-      <c r="P271" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q271" t="n">
-        <v>146</v>
-      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -15401,12 +13771,6 @@
       <c r="O272" t="n">
         <v>155</v>
       </c>
-      <c r="P272" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q272" t="n">
-        <v>155</v>
-      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -15456,12 +13820,6 @@
       <c r="O273" t="n">
         <v>104</v>
       </c>
-      <c r="P273" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q273" t="n">
-        <v>104</v>
-      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -15511,12 +13869,6 @@
       <c r="O274" t="n">
         <v>104</v>
       </c>
-      <c r="P274" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q274" t="n">
-        <v>104</v>
-      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -15566,12 +13918,6 @@
       <c r="O275" t="n">
         <v>101</v>
       </c>
-      <c r="P275" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q275" t="n">
-        <v>101</v>
-      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -15621,12 +13967,6 @@
       <c r="O276" t="n">
         <v>122</v>
       </c>
-      <c r="P276" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q276" t="n">
-        <v>122</v>
-      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -15676,12 +14016,6 @@
       <c r="O277" t="n">
         <v>298</v>
       </c>
-      <c r="P277" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q277" t="n">
-        <v>298</v>
-      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -15731,12 +14065,6 @@
       <c r="O278" t="n">
         <v>30</v>
       </c>
-      <c r="P278" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q278" t="n">
-        <v>30</v>
-      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -15786,12 +14114,6 @@
       <c r="O279" t="n">
         <v>38</v>
       </c>
-      <c r="P279" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q279" t="n">
-        <v>38</v>
-      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -15841,12 +14163,6 @@
       <c r="O280" t="n">
         <v>110</v>
       </c>
-      <c r="P280" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q280" t="n">
-        <v>110</v>
-      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -15896,12 +14212,6 @@
       <c r="O281" t="n">
         <v>313</v>
       </c>
-      <c r="P281" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q281" t="n">
-        <v>313</v>
-      </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -15951,12 +14261,6 @@
       <c r="O282" t="n">
         <v>129</v>
       </c>
-      <c r="P282" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q282" t="n">
-        <v>129</v>
-      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -16006,12 +14310,6 @@
       <c r="O283" t="n">
         <v>26</v>
       </c>
-      <c r="P283" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q283" t="n">
-        <v>26</v>
-      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -16061,12 +14359,6 @@
       <c r="O284" t="n">
         <v>25</v>
       </c>
-      <c r="P284" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q284" t="n">
-        <v>25</v>
-      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -16116,12 +14408,6 @@
       <c r="O285" t="n">
         <v>14</v>
       </c>
-      <c r="P285" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q285" t="n">
-        <v>14</v>
-      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -16171,12 +14457,6 @@
       <c r="O286" t="n">
         <v>147</v>
       </c>
-      <c r="P286" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q286" t="n">
-        <v>147</v>
-      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -16226,12 +14506,6 @@
       <c r="O287" t="n">
         <v>130</v>
       </c>
-      <c r="P287" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q287" t="n">
-        <v>130</v>
-      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -16281,12 +14555,6 @@
       <c r="O288" t="n">
         <v>52</v>
       </c>
-      <c r="P288" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q288" t="n">
-        <v>52</v>
-      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -16336,12 +14604,6 @@
       <c r="O289" t="n">
         <v>21</v>
       </c>
-      <c r="P289" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q289" t="n">
-        <v>21</v>
-      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -16391,12 +14653,6 @@
       <c r="O290" t="n">
         <v>46</v>
       </c>
-      <c r="P290" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q290" t="n">
-        <v>46</v>
-      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -16446,12 +14702,6 @@
       <c r="O291" t="n">
         <v>19</v>
       </c>
-      <c r="P291" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q291" t="n">
-        <v>19</v>
-      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -16501,12 +14751,6 @@
       <c r="O292" t="n">
         <v>26</v>
       </c>
-      <c r="P292" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q292" t="n">
-        <v>26</v>
-      </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -16556,12 +14800,6 @@
       <c r="O293" t="n">
         <v>28</v>
       </c>
-      <c r="P293" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q293" t="n">
-        <v>28</v>
-      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -16611,12 +14849,6 @@
       <c r="O294" t="n">
         <v>227</v>
       </c>
-      <c r="P294" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q294" t="n">
-        <v>227</v>
-      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -16666,12 +14898,6 @@
       <c r="O295" t="n">
         <v>49</v>
       </c>
-      <c r="P295" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q295" t="n">
-        <v>49</v>
-      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -16721,12 +14947,6 @@
       <c r="O296" t="n">
         <v>74</v>
       </c>
-      <c r="P296" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q296" t="n">
-        <v>74</v>
-      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -16776,12 +14996,6 @@
       <c r="O297" t="n">
         <v>104</v>
       </c>
-      <c r="P297" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q297" t="n">
-        <v>107</v>
-      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -16831,12 +15045,6 @@
       <c r="O298" t="n">
         <v>14</v>
       </c>
-      <c r="P298" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q298" t="n">
-        <v>21</v>
-      </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -16886,12 +15094,6 @@
       <c r="O299" t="n">
         <v>15</v>
       </c>
-      <c r="P299" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q299" t="n">
-        <v>28</v>
-      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -16941,12 +15143,6 @@
       <c r="O300" t="n">
         <v>100</v>
       </c>
-      <c r="P300" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q300" t="n">
-        <v>105</v>
-      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -16996,12 +15192,6 @@
       <c r="O301" t="n">
         <v>126</v>
       </c>
-      <c r="P301" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q301" t="n">
-        <v>136</v>
-      </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -17051,12 +15241,6 @@
       <c r="O302" t="n">
         <v>37</v>
       </c>
-      <c r="P302" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q302" t="n">
-        <v>45</v>
-      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -17106,12 +15290,6 @@
       <c r="O303" t="n">
         <v>283</v>
       </c>
-      <c r="P303" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q303" t="n">
-        <v>290</v>
-      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -17161,12 +15339,6 @@
       <c r="O304" t="n">
         <v>393</v>
       </c>
-      <c r="P304" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q304" t="n">
-        <v>398</v>
-      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -17216,12 +15388,6 @@
       <c r="O305" t="n">
         <v>373</v>
       </c>
-      <c r="P305" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q305" t="n">
-        <v>384</v>
-      </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -17271,12 +15437,6 @@
       <c r="O306" t="n">
         <v>204</v>
       </c>
-      <c r="P306" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q306" t="n">
-        <v>217</v>
-      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -17326,12 +15486,6 @@
       <c r="O307" t="n">
         <v>95</v>
       </c>
-      <c r="P307" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q307" t="n">
-        <v>100</v>
-      </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -17381,12 +15535,6 @@
       <c r="O308" t="n">
         <v>110</v>
       </c>
-      <c r="P308" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q308" t="n">
-        <v>120</v>
-      </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
@@ -17436,12 +15584,6 @@
       <c r="O309" t="n">
         <v>109</v>
       </c>
-      <c r="P309" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q309" t="n">
-        <v>116</v>
-      </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -17491,12 +15633,6 @@
       <c r="O310" t="n">
         <v>31</v>
       </c>
-      <c r="P310" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q310" t="n">
-        <v>35</v>
-      </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -17546,12 +15682,6 @@
       <c r="O311" t="n">
         <v>34</v>
       </c>
-      <c r="P311" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q311" t="n">
-        <v>42</v>
-      </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -17601,12 +15731,6 @@
       <c r="O312" t="n">
         <v>46</v>
       </c>
-      <c r="P312" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q312" t="n">
-        <v>57</v>
-      </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -17656,12 +15780,6 @@
       <c r="O313" t="n">
         <v>23</v>
       </c>
-      <c r="P313" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q313" t="n">
-        <v>27</v>
-      </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -17711,12 +15829,6 @@
       <c r="O314" t="n">
         <v>15</v>
       </c>
-      <c r="P314" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q314" t="n">
-        <v>22</v>
-      </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -17766,12 +15878,6 @@
       <c r="O315" t="n">
         <v>32</v>
       </c>
-      <c r="P315" t="n">
-        <v>7</v>
-      </c>
-      <c r="Q315" t="n">
-        <v>39</v>
-      </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -17821,12 +15927,6 @@
       <c r="O316" t="n">
         <v>31</v>
       </c>
-      <c r="P316" t="n">
-        <v>11</v>
-      </c>
-      <c r="Q316" t="n">
-        <v>42</v>
-      </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -17876,12 +15976,6 @@
       <c r="O317" t="n">
         <v>46</v>
       </c>
-      <c r="P317" t="n">
-        <v>9</v>
-      </c>
-      <c r="Q317" t="n">
-        <v>55</v>
-      </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -17931,12 +16025,6 @@
       <c r="O318" t="n">
         <v>22</v>
       </c>
-      <c r="P318" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q318" t="n">
-        <v>35</v>
-      </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -17986,12 +16074,6 @@
       <c r="O319" t="n">
         <v>23</v>
       </c>
-      <c r="P319" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q319" t="n">
-        <v>31</v>
-      </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -18040,12 +16122,6 @@
       </c>
       <c r="O320" t="n">
         <v>19</v>
-      </c>
-      <c r="P320" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q320" t="n">
-        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily auto-refresh 2026-09-10 15:00
</commit_message>
<xml_diff>
--- a/daily_slab_mix.xlsx
+++ b/daily_slab_mix.xlsx
@@ -15053,7 +15053,7 @@
         </is>
       </c>
       <c r="B299" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C299" t="n">
         <v>0</v>
@@ -15083,7 +15083,7 @@
         <v>0</v>
       </c>
       <c r="L299" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="M299" t="n">
         <v>42</v>
@@ -16915,7 +16915,7 @@
         </is>
       </c>
       <c r="B337" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C337" t="n">
         <v>0</v>
@@ -16945,7 +16945,7 @@
         <v>0</v>
       </c>
       <c r="L337" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M337" t="n">
         <v>5</v>
@@ -16964,7 +16964,7 @@
         </is>
       </c>
       <c r="B338" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C338" t="n">
         <v>0</v>
@@ -16994,7 +16994,7 @@
         <v>1</v>
       </c>
       <c r="L338" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="M338" t="n">
         <v>50</v>
@@ -17013,7 +17013,7 @@
         </is>
       </c>
       <c r="B339" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C339" t="n">
         <v>1</v>
@@ -17043,7 +17043,7 @@
         <v>2</v>
       </c>
       <c r="L339" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="M339" t="n">
         <v>22</v>

</xml_diff>